<commit_message>
Update Privacy News Dashboard snapshot (2026-07-15 14:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -4975,7 +4975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5038,7 +5038,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5048,22 +5048,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -5079,19 +5079,19 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5101,12 +5101,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -5116,7 +5116,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -5127,96 +5127,92 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -5226,35 +5222,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -5264,22 +5264,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -5290,24 +5290,24 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -5317,12 +5317,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -5343,24 +5343,24 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -5370,22 +5370,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -5401,44 +5401,44 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -5454,44 +5454,44 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -5499,31 +5499,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -5533,12 +5529,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -5548,7 +5544,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -5580,22 +5576,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -5605,7 +5601,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -5613,27 +5609,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -5643,12 +5643,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -5658,113 +5658,113 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -5772,31 +5772,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -5806,12 +5802,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -5821,7 +5817,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -5853,32 +5849,32 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -5886,7 +5882,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -5906,22 +5906,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -5931,7 +5931,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -5959,22 +5959,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -5984,19 +5984,15 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6016,7 +6012,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -6026,12 +6022,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -6041,7 +6037,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -6073,40 +6069,44 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6126,22 +6126,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -6151,7 +6151,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -6159,11 +6159,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6183,32 +6179,32 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -6216,7 +6212,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6224,34 +6224,34 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -6261,7 +6261,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -6272,49 +6272,49 @@
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -6342,22 +6342,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -6367,7 +6367,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -6395,32 +6395,32 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -6448,22 +6448,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -6473,39 +6473,35 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -6515,27 +6511,27 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -6562,32 +6558,32 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -6595,52 +6591,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -6668,32 +6668,32 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -6721,32 +6721,32 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -6774,32 +6774,32 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -6827,32 +6827,32 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -6872,6 +6872,59 @@
         </is>
       </c>
       <c r="K35" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-15 18:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -4975,7 +4975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5038,22 +5038,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -5063,15 +5063,19 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -5079,19 +5083,19 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5101,27 +5105,27 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -5132,19 +5136,19 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -5154,22 +5158,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -5180,61 +5184,57 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -5242,19 +5242,19 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -5264,22 +5264,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -5295,52 +5295,56 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -5348,19 +5352,19 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -5370,22 +5374,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -5401,19 +5405,19 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -5423,22 +5427,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -5449,49 +5453,49 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -5507,44 +5511,44 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -5552,56 +5556,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -5609,46 +5609,42 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -5658,7 +5654,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -5666,42 +5662,46 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -5711,15 +5711,19 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -5727,44 +5731,44 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -5780,56 +5784,52 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -5837,44 +5837,44 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -5882,56 +5882,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -5939,7 +5935,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -5959,32 +5959,32 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -5992,7 +5992,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6012,22 +6016,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -6037,19 +6041,15 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6069,22 +6069,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -6094,19 +6094,15 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6126,40 +6122,44 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6179,7 +6179,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -6189,27 +6189,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -6236,7 +6236,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -6246,22 +6246,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -6277,44 +6277,44 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -6322,52 +6322,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -6378,49 +6382,49 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -6448,32 +6452,32 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -6501,89 +6505,85 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -6591,109 +6591,109 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -6701,52 +6701,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -6774,32 +6778,32 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -6827,32 +6831,32 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -6880,32 +6884,32 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -6925,6 +6929,112 @@
         </is>
       </c>
       <c r="K36" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>950</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>51749</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-16 11:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -1605,7 +1605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1668,32 +1668,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>10301</t>
+          <t>11221</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1280</t>
+          <t>1281</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.15.자)</t>
+          <t>AI 혁신을 뒷받침하고 국민 권익을 증진하는 예방중심 개인정보 보호 실현</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12276</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12281</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1713,44 +1713,44 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-15 09:45:30.272302+09:00</t>
+          <t>2026-07-16 11:00:27.819143+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-15 09:45:30.272302+09:00</t>
+          <t>2026-07-16 11:00:27.819143+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>9501</t>
+          <t>10301</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1279</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>개인정보 전송요구권 전송체계 기술적 기틀, 고용⋅교육 부문까지 확대 마련</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.15.자)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12266</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12276</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>인프라표준화팀</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1770,44 +1770,44 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-14 10:00:29.933870+09:00</t>
+          <t>2026-07-15 09:45:30.272302+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-14 10:00:29.933870+09:00</t>
+          <t>2026-07-15 09:45:30.272302+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>9381</t>
+          <t>9501</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1280</t>
+          <t>1279</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>정보주체의 본인전송요구권, 더 안전하게 이용할 수 있습니다</t>
+          <t>개인정보 전송요구권 전송체계 기술적 기틀, 고용⋅교육 부문까지 확대 마련</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12273</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12266</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>범정부마이데이터추진단 전략기획팀</t>
+          <t>인프라표준화팀</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1827,39 +1827,39 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-14 08:30:26.475160+09:00</t>
+          <t>2026-07-14 10:00:29.933870+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-14 08:30:26.475160+09:00</t>
+          <t>2026-07-14 10:00:29.933870+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>9271</t>
+          <t>9381</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>365</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>공공기관 종합청렴도 평가 관련 개인정보 제3자 제공사항 알림</t>
+          <t>정보주체의 본인전송요구권, 더 안전하게 이용할 수 있습니다</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12267</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12273</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>법무감사담당관</t>
+          <t>범정부마이데이터추진단 전략기획팀</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1869,116 +1869,116 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>303</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-13 17:16:17.898453+09:00</t>
+          <t>2026-07-14 08:30:26.475160+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-13 17:16:17.898453+09:00</t>
+          <t>2026-07-14 08:30:26.475160+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>6541</t>
+          <t>9271</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1278</t>
+          <t>365</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>개인정보 온라인 불법유통 청년들이 직접 차단한다.</t>
+          <t>공공기관 종합청렴도 평가 관련 개인정보 제3자 제공사항 알림</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12262</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12267</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>조사2과</t>
+          <t>법무감사담당관</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-10 14:00:31.832545+09:00</t>
+          <t>2026-07-13 17:16:17.898453+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-10 14:00:31.832545+09:00</t>
+          <t>2026-07-13 17:16:17.898453+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>5491</t>
+          <t>6541</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>364</t>
+          <t>1278</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>제4회 개인정보보호 모의재판 경연대회 참가자 모집</t>
+          <t>개인정보 온라인 불법유통 청년들이 직접 차단한다.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12245</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12262</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>침해평가과</t>
+          <t>조사2과</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1988,49 +1988,49 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-09 11:01:05.002078+09:00</t>
+          <t>2026-07-10 14:00:31.832545+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-09 11:01:05.002078+09:00</t>
+          <t>2026-07-10 14:00:31.832545+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>5402</t>
+          <t>5491</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1276</t>
+          <t>364</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>개인정보위, 안전조치 의무 위반 3개 사업자 제재</t>
+          <t>제4회 개인정보보호 모의재판 경연대회 참가자 모집</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12242</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12245</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>장석인</t>
+          <t>침해평가과</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2045,49 +2045,49 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-09 11:01:05.002078+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-09 11:01:05.002078+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>5401</t>
+          <t>5402</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1277</t>
+          <t>1276</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>미래의 개인정보 법률 전문가 모여 인공지능 시대 법적 쟁점 논의한다</t>
+          <t>개인정보위, 안전조치 의무 위반 3개 사업자 제재</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12243</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12242</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>침해평가과</t>
+          <t>장석인</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -2124,27 +2124,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>5391</t>
+          <t>5401</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>363</t>
+          <t>1277</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>「개인정보 보호책임자 경력 인정에 관한 고시」 일부개정고시안 행정예고</t>
+          <t>미래의 개인정보 법률 전문가 모여 인공지능 시대 법적 쟁점 논의한다</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12244</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12243</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>침해평가과</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -2159,54 +2159,54 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-09 09:46:03.809898+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-09 09:46:03.809898+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>4581</t>
+          <t>5391</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1275</t>
+          <t>363</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>개인정보위, 응용프로그램 인터페이스(API) 활용 확대에 따른 개인정보 유출 예방 당부</t>
+          <t>「개인정보 보호책임자 경력 인정에 관한 고시」 일부개정고시안 행정예고</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12241</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12244</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>사전실태점검과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2216,54 +2216,54 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-08 10:00:27.128578+09:00</t>
+          <t>2026-07-09 09:46:03.809898+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-08 10:00:27.128578+09:00</t>
+          <t>2026-07-09 09:46:03.809898+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>3251</t>
+          <t>4581</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>1275</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026년 가명정보 활용 지원체계 설명회 개최 안내</t>
+          <t>개인정보위, 응용프로그램 인터페이스(API) 활용 확대에 따른 개인정보 유출 예방 당부</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12238</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12241</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>사전실태점검과</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2273,49 +2273,49 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-06 13:46:04.662402+09:00</t>
+          <t>2026-07-08 10:00:27.128578+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-06 13:46:04.662402+09:00</t>
+          <t>2026-07-08 10:00:27.128578+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3182</t>
+          <t>3251</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1273</t>
+          <t>362</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>개인정보 처리방침 평가, 국민 눈높이에서 더 꼼꼼히 본다</t>
+          <t>2026년 가명정보 활용 지원체계 설명회 개최 안내</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12236</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12238</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -2330,49 +2330,49 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-06 13:46:04.662402+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-06 13:46:04.662402+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>3181</t>
+          <t>3182</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1274</t>
+          <t>1273</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>개인정보위, 교육‧고용 분야까지 개인정보 제3자 전송요구권 확대 추진</t>
+          <t>개인정보 처리방침 평가, 국민 눈높이에서 더 꼼꼼히 본다</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12237</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12236</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>60</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -2409,32 +2409,32 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1043</t>
+          <t>3181</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>1274</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>개인정보위, 대전에서 ‘찾아가는 개인정보 현장 컨설팅 및 교육’ 개최</t>
+          <t>개인정보위, 교육‧고용 분야까지 개인정보 제3자 전송요구권 확대 추진</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12227</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12237</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>58</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2454,39 +2454,39 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-03 16:00:28.543767+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-03 16:00:28.543767+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>1043</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1272</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.3.자)</t>
+          <t>개인정보위, 대전에서 ‘찾아가는 개인정보 현장 컨설팅 및 교육’ 개최</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12229</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12227</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2511,39 +2511,39 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-03 15:30:33.546332+09:00</t>
+          <t>2026-07-03 16:00:28.543767+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-03 15:30:33.546332+09:00</t>
+          <t>2026-07-03 16:00:28.543767+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>561</t>
+          <t>1001</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1271</t>
+          <t>1272</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>신뢰로 여는 인공지능(AI) 혁신, 달라지는 개인정보 체계로 이끈다</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.3.자)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12228</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12229</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>개인정보보호정책과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2568,44 +2568,44 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-03 10:00:33.422568+09:00</t>
+          <t>2026-07-03 15:30:33.546332+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-03 10:00:33.422568+09:00</t>
+          <t>2026-07-03 15:30:33.546332+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>561</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1269</t>
+          <t>1271</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>개인정보위, 인공지능(AI) 시대 데이터 혁신적 활용을 지역 주도로 확산한다.</t>
+          <t>신뢰로 여는 인공지능(AI) 혁신, 달라지는 개인정보 체계로 이끈다</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12225</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12228</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>개인정보보호정책과</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2625,19 +2625,19 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-02 16:45:30.717611+09:00</t>
+          <t>2026-07-03 10:00:33.422568+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-02 16:45:30.717611+09:00</t>
+          <t>2026-07-03 10:00:33.422568+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>281</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2647,17 +2647,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>개인정보위, 개인정보보호 현장 간담회 개최</t>
+          <t>개인정보위, 인공지능(AI) 시대 데이터 혁신적 활용을 지역 주도로 확산한다.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12224</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12225</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>조사1과</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2682,44 +2682,44 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 16:45:30.717611+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 16:45:30.717611+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1266</t>
+          <t>1269</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>글로벌 개인정보 감독기구에 인공지능(AI) 대응 ‘실전해법’ 제시</t>
+          <t>개인정보위, 개인정보보호 현장 간담회 개최</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12218</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12224</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>국제협력담당관</t>
+          <t>조사1과</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2729,7 +2729,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>924</t>
+          <t>98</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2751,27 +2751,27 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1267</t>
+          <t>1266</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>투숙객 개인정보보호에 앞장선 호텔, 호텔업 등급평가시 우대</t>
+          <t>글로벌 개인정보 감독기구에 인공지능(AI) 대응 ‘실전해법’ 제시</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12219</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12218</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>국제협력담당관</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1074</t>
+          <t>924</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2808,27 +2808,27 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1268</t>
+          <t>1267</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.1.자)</t>
+          <t>투숙객 개인정보보호에 앞장선 호텔, 호텔업 등급평가시 우대</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12220</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12219</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>743</t>
+          <t>1074</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2865,32 +2865,32 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>361</t>
+          <t>1268</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령(안) 입법예고</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.1.자)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12216</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12220</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>범정부 마이데이터추진단</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2900,49 +2900,49 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>743</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>1265</t>
+          <t>361</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.6.30.자)</t>
+          <t>「개인정보 보호법 시행령」 일부개정령(안) 입법예고</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12217</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12216</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>범정부 마이데이터추진단</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2957,54 +2957,54 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1029</t>
+          <t>1842</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>1265</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.6.30.자)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12202</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12217</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -3014,49 +3014,49 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2800</t>
+          <t>1029</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>1262</t>
+          <t>360</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>개인정보위원장, G7 개인정보 감독기구 라운드테이블 참석</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12201</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12202</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>국제협력담당관</t>
+          <t>신기술개인정보과</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3071,49 +3071,49 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2144</t>
+          <t>2800</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1263</t>
+          <t>1262</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>「2026 개인정보 보호·활용 기술 대상」 참여기업 모집</t>
+          <t>개인정보위원장, G7 개인정보 감독기구 라운드테이블 참석</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12203</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12201</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>국제협력담당관</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2092</t>
+          <t>2144</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -3150,27 +3150,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>1264</t>
+          <t>1263</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AI 범죄 대응 범부처 협의체 출범</t>
+          <t>「2026 개인정보 보호·활용 기술 대상」 참여기업 모집</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12204</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12203</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>인공지능프라이버시팀</t>
+          <t>신기술개인정보과</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3185,7 +3185,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2638</t>
+          <t>2092</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -3207,32 +3207,32 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>359</t>
+          <t>1264</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>본인전송요구 대리인의 사전협의 요청 시범기간(6.25.~7.10.) 운영 안내</t>
+          <t>AI 범죄 대응 범부처 협의체 출범</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12200</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12204</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>인공지능프라이버시팀</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3242,49 +3242,49 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>3745</t>
+          <t>2638</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>1260</t>
+          <t>359</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>개인정보위, 상조서비스 개인정보 보호 취약요인 선제 점검</t>
+          <t>본인전송요구 대리인의 사전협의 요청 시범기간(6.25.~7.10.) 운영 안내</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12197</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12200</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>사전실태점검과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3299,49 +3299,49 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2754</t>
+          <t>3745</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>1261</t>
+          <t>1260</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>개인정보위, 국민이 필요로 하는 정보 중심 ‘본인전송요구권’ 안착 지원한다</t>
+          <t>개인정보위, 상조서비스 개인정보 보호 취약요인 선제 점검</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12198</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12197</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>사전실태점검과</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3356,7 +3356,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>3085</t>
+          <t>2754</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3378,32 +3378,32 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>358</t>
+          <t>1261</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>정보보호 및 개인정보보호 관리체계 심사기관 지정 공고(제2026-73호)</t>
+          <t>개인정보위, 국민이 필요로 하는 정보 중심 ‘본인전송요구권’ 안착 지원한다</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12185</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12198</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3413,54 +3413,54 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>7681</t>
+          <t>3085</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>357</t>
+          <t>358</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>「자율기구 공공실태점검단 설치 및 운영에 관한 규정」 발령(2026-70)</t>
+          <t>정보보호 및 개인정보보호 관리체계 심사기관 지정 공고(제2026-73호)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12174</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12185</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>혁신기획담당관</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>6533</t>
+          <t>7681</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3492,32 +3492,32 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>357</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>공공기관 개인정보 보호수준 평가단원 지원 공고</t>
+          <t>「자율기구 공공실태점검단 설치 및 운영에 관한 규정」 발령(2026-70)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12160</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12174</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3527,7 +3527,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>9023</t>
+          <t>6533</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3549,32 +3549,32 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>352</t>
+          <t>356</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
+          <t>공공기관 개인정보 보호수준 평가단원 지원 공고</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12126</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12160</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>개인정보보호정책과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3584,7 +3584,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>11169</t>
+          <t>9023</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3606,12 +3606,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>354</t>
+          <t>352</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3621,17 +3621,17 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12131</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12126</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>개인정보보호정책과</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3641,7 +3641,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>13472</t>
+          <t>11169</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3663,27 +3663,27 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>355</t>
+          <t>354</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12136</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12131</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -3698,7 +3698,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>9724</t>
+          <t>13472</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3720,55 +3720,112 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>355</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12136</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>신기술개인정보과</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>9724</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>19</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>353</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>「개인정보 처리 방법에 관한 고시」 일부개정고시안 행정예고</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12127</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>전략기획팀</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
         <is>
           <t>11519</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>공지사항</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-16 12:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -5032,7 +5032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5095,79 +5095,75 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -5177,7 +5173,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -5185,7 +5181,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -5193,19 +5193,19 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -5215,12 +5215,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -5230,12 +5230,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -5246,19 +5246,19 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -5268,22 +5268,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -5299,19 +5299,19 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -5321,12 +5321,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -5336,7 +5336,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -5347,96 +5347,92 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -5446,35 +5442,39 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -5484,22 +5484,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -5510,24 +5510,24 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -5537,12 +5537,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -5552,7 +5552,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -5563,24 +5563,24 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -5590,22 +5590,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -5621,44 +5621,44 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -5674,44 +5674,44 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -5719,31 +5719,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -5753,12 +5749,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -5768,7 +5764,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -5800,22 +5796,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -5825,7 +5821,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -5833,27 +5829,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -5863,12 +5863,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -5878,113 +5878,113 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -5992,31 +5992,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -6026,12 +6022,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -6041,7 +6037,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -6073,32 +6069,32 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -6106,7 +6102,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6126,22 +6126,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -6151,7 +6151,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -6179,22 +6179,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -6204,19 +6204,15 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6236,7 +6232,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -6246,12 +6242,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -6261,7 +6257,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -6293,40 +6289,44 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6346,22 +6346,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -6371,7 +6371,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -6379,11 +6379,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6403,32 +6399,32 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -6436,7 +6432,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6444,34 +6444,34 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -6481,7 +6481,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -6492,49 +6492,49 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -6562,22 +6562,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -6587,7 +6587,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -6615,32 +6615,32 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -6668,22 +6668,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -6693,39 +6693,35 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -6735,27 +6731,27 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -6782,32 +6778,32 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -6815,52 +6811,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -6888,32 +6888,32 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -6941,32 +6941,32 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -6994,32 +6994,32 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -7047,32 +7047,32 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -7092,6 +7092,59 @@
         </is>
       </c>
       <c r="K38" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-16 13:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -1605,7 +1605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1668,27 +1668,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>11221</t>
+          <t>11392</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1281</t>
+          <t>367</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AI 혁신을 뒷받침하고 국민 권익을 증진하는 예방중심 개인정보 보호 실현</t>
+          <t>「개인정보 보호법 위반에 대한 과징금 부과기준」 일부개정안 행정예고</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12281</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12282</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>혁신기획담당관</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1703,54 +1703,54 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-16 11:00:27.819143+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-16 11:00:27.819143+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>10301</t>
+          <t>11391</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1280</t>
+          <t>368</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.15.자)</t>
+          <t>「개인정보 보호법 위반에 대한 과태료 부과기준」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12276</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12284</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1760,54 +1760,54 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-15 09:45:30.272302+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-15 09:45:30.272302+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>9501</t>
+          <t>11221</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1279</t>
+          <t>1281</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>개인정보 전송요구권 전송체계 기술적 기틀, 고용⋅교육 부문까지 확대 마련</t>
+          <t>AI 혁신을 뒷받침하고 국민 권익을 증진하는 예방중심 개인정보 보호 실현</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12266</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12281</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>인프라표준화팀</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1827,19 +1827,19 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-14 10:00:29.933870+09:00</t>
+          <t>2026-07-16 11:00:27.819143+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-14 10:00:29.933870+09:00</t>
+          <t>2026-07-16 11:00:27.819143+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>9381</t>
+          <t>10301</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1849,22 +1849,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>정보주체의 본인전송요구권, 더 안전하게 이용할 수 있습니다</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.15.자)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12273</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12276</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>범정부마이데이터추진단 전략기획팀</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1884,101 +1884,101 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-14 08:30:26.475160+09:00</t>
+          <t>2026-07-15 09:45:30.272302+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-14 08:30:26.475160+09:00</t>
+          <t>2026-07-15 09:45:30.272302+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>9271</t>
+          <t>9501</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>365</t>
+          <t>1279</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>공공기관 종합청렴도 평가 관련 개인정보 제3자 제공사항 알림</t>
+          <t>개인정보 전송요구권 전송체계 기술적 기틀, 고용⋅교육 부문까지 확대 마련</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12267</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12266</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>법무감사담당관</t>
+          <t>인프라표준화팀</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-13 17:16:17.898453+09:00</t>
+          <t>2026-07-14 10:00:29.933870+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-13 17:16:17.898453+09:00</t>
+          <t>2026-07-14 10:00:29.933870+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>6541</t>
+          <t>9381</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1278</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>개인정보 온라인 불법유통 청년들이 직접 차단한다.</t>
+          <t>정보주체의 본인전송요구권, 더 안전하게 이용할 수 있습니다</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12262</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12273</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>조사2과</t>
+          <t>범정부마이데이터추진단 전략기획팀</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1988,7 +1988,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>303</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1998,54 +1998,54 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-10 14:00:31.832545+09:00</t>
+          <t>2026-07-14 08:30:26.475160+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-10 14:00:31.832545+09:00</t>
+          <t>2026-07-14 08:30:26.475160+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>5491</t>
+          <t>9271</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>364</t>
+          <t>365</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>제4회 개인정보보호 모의재판 경연대회 참가자 모집</t>
+          <t>공공기관 종합청렴도 평가 관련 개인정보 제3자 제공사항 알림</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12245</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12267</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>침해평가과</t>
+          <t>법무감사담당관</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -2055,44 +2055,44 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-09 11:01:05.002078+09:00</t>
+          <t>2026-07-13 17:16:17.898453+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-09 11:01:05.002078+09:00</t>
+          <t>2026-07-13 17:16:17.898453+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>5402</t>
+          <t>6541</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1276</t>
+          <t>1278</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>개인정보위, 안전조치 의무 위반 3개 사업자 제재</t>
+          <t>개인정보 온라인 불법유통 청년들이 직접 차단한다.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12242</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12262</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>장석인</t>
+          <t>조사2과</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -2112,34 +2112,34 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-10 14:00:31.832545+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-10 14:00:31.832545+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>5401</t>
+          <t>5491</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1277</t>
+          <t>364</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>미래의 개인정보 법률 전문가 모여 인공지능 시대 법적 쟁점 논의한다</t>
+          <t>제4회 개인정보보호 모의재판 경연대회 참가자 모집</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12243</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12245</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -2159,49 +2159,49 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-09 11:01:05.002078+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-09 11:01:05.002078+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>5391</t>
+          <t>5402</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>363</t>
+          <t>1276</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>「개인정보 보호책임자 경력 인정에 관한 고시」 일부개정고시안 행정예고</t>
+          <t>개인정보위, 안전조치 의무 위반 3개 사업자 제재</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12244</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12242</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>장석인</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -2216,54 +2216,54 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-09 09:46:03.809898+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-09 09:46:03.809898+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>4581</t>
+          <t>5401</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1275</t>
+          <t>1277</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>개인정보위, 응용프로그램 인터페이스(API) 활용 확대에 따른 개인정보 유출 예방 당부</t>
+          <t>미래의 개인정보 법률 전문가 모여 인공지능 시대 법적 쟁점 논의한다</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12241</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12243</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>사전실태점검과</t>
+          <t>침해평가과</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -2283,44 +2283,44 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-08 10:00:27.128578+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-08 10:00:27.128578+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3251</t>
+          <t>5391</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>363</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026년 가명정보 활용 지원체계 설명회 개최 안내</t>
+          <t>「개인정보 보호책임자 경력 인정에 관한 고시」 일부개정고시안 행정예고</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12238</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12244</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2340,44 +2340,44 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-06 13:46:04.662402+09:00</t>
+          <t>2026-07-09 09:46:03.809898+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-06 13:46:04.662402+09:00</t>
+          <t>2026-07-09 09:46:03.809898+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>3182</t>
+          <t>4581</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1273</t>
+          <t>1275</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>개인정보 처리방침 평가, 국민 눈높이에서 더 꼼꼼히 본다</t>
+          <t>개인정보위, 응용프로그램 인터페이스(API) 활용 확대에 따른 개인정보 유출 예방 당부</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12236</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12241</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>사전실태점검과</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -2397,39 +2397,39 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-08 10:00:27.128578+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-08 10:00:27.128578+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>3181</t>
+          <t>3251</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1274</t>
+          <t>362</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>개인정보위, 교육‧고용 분야까지 개인정보 제3자 전송요구권 확대 추진</t>
+          <t>2026년 가명정보 활용 지원체계 설명회 개최 안내</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12237</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12238</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2444,54 +2444,54 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-06 13:46:04.662402+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-06 13:46:04.662402+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1043</t>
+          <t>3182</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>1273</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>개인정보위, 대전에서 ‘찾아가는 개인정보 현장 컨설팅 및 교육’ 개최</t>
+          <t>개인정보 처리방침 평가, 국민 눈높이에서 더 꼼꼼히 본다</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12227</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12236</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>60</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2511,44 +2511,44 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-03 16:00:28.543767+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-03 16:00:28.543767+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>3181</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1272</t>
+          <t>1274</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.3.자)</t>
+          <t>개인정보위, 교육‧고용 분야까지 개인정보 제3자 전송요구권 확대 추진</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12229</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12237</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>58</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2568,39 +2568,39 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-03 15:30:33.546332+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-03 15:30:33.546332+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>561</t>
+          <t>1043</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1271</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>신뢰로 여는 인공지능(AI) 혁신, 달라지는 개인정보 체계로 이끈다</t>
+          <t>개인정보위, 대전에서 ‘찾아가는 개인정보 현장 컨설팅 및 교육’ 개최</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12228</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12227</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>개인정보보호정책과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2625,44 +2625,44 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-03 10:00:33.422568+09:00</t>
+          <t>2026-07-03 16:00:28.543767+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-03 10:00:33.422568+09:00</t>
+          <t>2026-07-03 16:00:28.543767+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>1001</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1269</t>
+          <t>1272</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>개인정보위, 인공지능(AI) 시대 데이터 혁신적 활용을 지역 주도로 확산한다.</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.3.자)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12225</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12229</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2682,44 +2682,44 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-02 16:45:30.717611+09:00</t>
+          <t>2026-07-03 15:30:33.546332+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-02 16:45:30.717611+09:00</t>
+          <t>2026-07-03 15:30:33.546332+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>561</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1269</t>
+          <t>1271</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>개인정보위, 개인정보보호 현장 간담회 개최</t>
+          <t>신뢰로 여는 인공지능(AI) 혁신, 달라지는 개인정보 체계로 이끈다</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12224</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12228</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>조사1과</t>
+          <t>개인정보보호정책과</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2729,7 +2729,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2739,44 +2739,44 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-03 10:00:33.422568+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-03 10:00:33.422568+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>281</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1266</t>
+          <t>1269</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>글로벌 개인정보 감독기구에 인공지능(AI) 대응 ‘실전해법’ 제시</t>
+          <t>개인정보위, 인공지능(AI) 시대 데이터 혁신적 활용을 지역 주도로 확산한다.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12218</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12225</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>국제협력담당관</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>924</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2796,44 +2796,44 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 16:45:30.717611+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 16:45:30.717611+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1267</t>
+          <t>1269</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>투숙객 개인정보보호에 앞장선 호텔, 호텔업 등급평가시 우대</t>
+          <t>개인정보위, 개인정보보호 현장 간담회 개최</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12219</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12224</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>조사1과</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1074</t>
+          <t>98</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2865,27 +2865,27 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1268</t>
+          <t>1266</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.1.자)</t>
+          <t>글로벌 개인정보 감독기구에 인공지능(AI) 대응 ‘실전해법’ 제시</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12220</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12218</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>국제협력담당관</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>743</t>
+          <t>924</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2922,32 +2922,32 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>361</t>
+          <t>1267</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령(안) 입법예고</t>
+          <t>투숙객 개인정보보호에 앞장선 호텔, 호텔업 등급평가시 우대</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12216</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12219</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>범정부 마이데이터추진단</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2957,44 +2957,44 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1074</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>1265</t>
+          <t>1268</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.6.30.자)</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.1.자)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12217</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12220</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1029</t>
+          <t>743</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -3036,32 +3036,32 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>361</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고</t>
+          <t>「개인정보 보호법 시행령」 일부개정령(안) 입법예고</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12202</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12216</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>범정부 마이데이터추진단</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3071,7 +3071,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2800</t>
+          <t>1842</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -3093,32 +3093,32 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1262</t>
+          <t>1265</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>개인정보위원장, G7 개인정보 감독기구 라운드테이블 참석</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.6.30.자)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12201</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12217</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>국제협력담당관</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2144</t>
+          <t>1029</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -3150,22 +3150,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>1263</t>
+          <t>360</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>「2026 개인정보 보호·활용 기술 대상」 참여기업 모집</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12203</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12202</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -3185,49 +3185,49 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2092</t>
+          <t>2800</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>1264</t>
+          <t>1262</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AI 범죄 대응 범부처 협의체 출범</t>
+          <t>개인정보위원장, G7 개인정보 감독기구 라운드테이블 참석</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12204</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12201</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>인공지능프라이버시팀</t>
+          <t>국제협력담당관</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3242,7 +3242,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2638</t>
+          <t>2144</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -3264,32 +3264,32 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>359</t>
+          <t>1263</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>본인전송요구 대리인의 사전협의 요청 시범기간(6.25.~7.10.) 운영 안내</t>
+          <t>「2026 개인정보 보호·활용 기술 대상」 참여기업 모집</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12200</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12203</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>신기술개인정보과</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3299,54 +3299,54 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>3745</t>
+          <t>2092</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>1260</t>
+          <t>1264</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>개인정보위, 상조서비스 개인정보 보호 취약요인 선제 점검</t>
+          <t>AI 범죄 대응 범부처 협의체 출범</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12197</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12204</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>사전실태점검과</t>
+          <t>인공지능프라이버시팀</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3356,7 +3356,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2754</t>
+          <t>2638</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3378,22 +3378,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>1261</t>
+          <t>359</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>개인정보위, 국민이 필요로 하는 정보 중심 ‘본인전송요구권’ 안착 지원한다</t>
+          <t>본인전송요구 대리인의 사전협의 요청 시범기간(6.25.~7.10.) 운영 안내</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12198</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12200</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3413,54 +3413,54 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>3085</t>
+          <t>3745</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>358</t>
+          <t>1260</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>정보보호 및 개인정보보호 관리체계 심사기관 지정 공고(제2026-73호)</t>
+          <t>개인정보위, 상조서비스 개인정보 보호 취약요인 선제 점검</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12185</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12197</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>사전실태점검과</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3470,54 +3470,54 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>7681</t>
+          <t>2754</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>357</t>
+          <t>1261</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>「자율기구 공공실태점검단 설치 및 운영에 관한 규정」 발령(2026-70)</t>
+          <t>개인정보위, 국민이 필요로 하는 정보 중심 ‘본인전송요구권’ 안착 지원한다</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12174</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12198</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>혁신기획담당관</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3527,44 +3527,44 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>6533</t>
+          <t>3085</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>358</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>공공기관 개인정보 보호수준 평가단원 지원 공고</t>
+          <t>정보보호 및 개인정보보호 관리체계 심사기관 지정 공고(제2026-73호)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12160</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12185</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3574,7 +3574,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3584,7 +3584,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>9023</t>
+          <t>7681</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3606,32 +3606,32 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>352</t>
+          <t>357</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
+          <t>「자율기구 공공실태점검단 설치 및 운영에 관한 규정」 발령(2026-70)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12126</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12174</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>개인정보보호정책과</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3641,7 +3641,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>11169</t>
+          <t>6533</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3663,32 +3663,32 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>354</t>
+          <t>356</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
+          <t>공공기관 개인정보 보호수준 평가단원 지원 공고</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12131</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12160</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3698,7 +3698,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>13472</t>
+          <t>9023</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3720,32 +3720,32 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>355</t>
+          <t>352</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12136</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12126</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>개인정보보호정책과</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3755,7 +3755,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>9724</t>
+          <t>11169</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3777,55 +3777,169 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>354</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12131</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>조사총괄과</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>13472</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>355</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12136</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>신기술개인정보과</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>9724</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>19</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>353</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>「개인정보 처리 방법에 관한 고시」 일부개정고시안 행정예고</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12127</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>전략기획팀</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
         <is>
           <t>11519</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>공지사항</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="J41" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-20 12:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -5374,7 +5374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5437,7 +5437,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5447,12 +5447,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -5462,7 +5462,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -5478,34 +5478,34 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -5515,7 +5515,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -5523,56 +5523,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -5580,7 +5576,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -5588,34 +5588,34 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -5625,7 +5625,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -5636,96 +5636,92 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -5735,7 +5731,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -5743,7 +5739,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -5751,19 +5751,19 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -5773,12 +5773,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -5788,12 +5788,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -5804,19 +5804,19 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -5826,22 +5826,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -5857,19 +5857,19 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -5879,12 +5879,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -5905,96 +5905,92 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -6004,35 +6000,39 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -6042,22 +6042,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -6068,24 +6068,24 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -6095,12 +6095,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -6110,7 +6110,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -6121,24 +6121,24 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -6148,22 +6148,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -6179,44 +6179,44 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -6232,44 +6232,44 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -6277,31 +6277,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -6311,12 +6307,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -6326,7 +6322,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -6358,22 +6354,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -6383,7 +6379,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -6391,27 +6387,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -6421,12 +6421,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -6436,113 +6436,113 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -6550,31 +6550,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -6584,12 +6580,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -6599,7 +6595,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -6631,32 +6627,32 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -6664,7 +6660,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6684,22 +6684,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -6709,7 +6709,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -6737,22 +6737,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -6762,19 +6762,15 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6794,7 +6790,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -6804,12 +6800,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -6819,7 +6815,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -6851,40 +6847,44 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6904,22 +6904,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -6929,7 +6929,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -6937,11 +6937,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6961,32 +6957,32 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -6994,7 +6990,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7002,34 +7002,34 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -7039,7 +7039,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -7050,49 +7050,49 @@
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -7120,22 +7120,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -7173,32 +7173,32 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -7226,22 +7226,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -7251,39 +7251,35 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7293,27 +7289,27 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -7340,32 +7336,32 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -7373,52 +7369,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -7446,32 +7446,32 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -7499,32 +7499,32 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -7552,32 +7552,32 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -7585,46 +7585,42 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14403</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -7634,7 +7630,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>6587</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -7642,52 +7638,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -7707,6 +7707,59 @@
         </is>
       </c>
       <c r="K43" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-22 10:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -5374,7 +5374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5437,7 +5437,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5447,22 +5447,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -5478,19 +5478,19 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5500,12 +5500,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -5515,7 +5515,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -5531,34 +5531,34 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -5568,7 +5568,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -5576,56 +5576,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -5633,7 +5629,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -5641,34 +5641,34 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -5678,7 +5678,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -5689,96 +5689,92 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -5788,7 +5784,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -5796,7 +5792,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -5804,19 +5804,19 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -5826,12 +5826,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -5841,12 +5841,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -5857,19 +5857,19 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -5879,22 +5879,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -5910,19 +5910,19 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -5932,12 +5932,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -5947,7 +5947,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -5958,96 +5958,92 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -6057,35 +6053,39 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -6095,22 +6095,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -6121,24 +6121,24 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -6148,12 +6148,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -6163,7 +6163,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -6174,24 +6174,24 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -6201,22 +6201,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -6232,44 +6232,44 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -6285,44 +6285,44 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -6330,31 +6330,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -6364,12 +6360,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -6379,7 +6375,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -6411,22 +6407,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -6436,7 +6432,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -6444,27 +6440,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -6474,12 +6474,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -6489,113 +6489,113 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -6603,31 +6603,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -6637,12 +6633,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -6652,7 +6648,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -6684,32 +6680,32 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -6717,7 +6713,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6737,22 +6737,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -6762,7 +6762,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -6790,22 +6790,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -6815,19 +6815,15 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6847,7 +6843,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -6857,12 +6853,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -6872,7 +6868,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -6904,40 +6900,44 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6957,22 +6957,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -6990,11 +6990,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7014,32 +7010,32 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -7047,7 +7043,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7055,34 +7055,34 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -7092,7 +7092,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -7103,49 +7103,49 @@
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -7173,22 +7173,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -7198,7 +7198,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -7226,32 +7226,32 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -7279,22 +7279,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -7304,39 +7304,35 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7346,27 +7342,27 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -7393,32 +7389,32 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -7426,52 +7422,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -7499,32 +7499,32 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -7552,32 +7552,32 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -7605,32 +7605,32 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -7638,46 +7638,42 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14403</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -7687,7 +7683,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>6587</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -7695,52 +7691,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -7760,6 +7760,59 @@
         </is>
       </c>
       <c r="K44" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-22 13:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -1605,7 +1605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1668,32 +1668,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14451</t>
+          <t>16314</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>369</t>
+          <t>370</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>본인전송요구 대리인의 사전협의 요청 시범기간 추가운영(7.20.~31.) 안내</t>
+          <t>「개인정보 보호위원회의 조사 및 처분에 관한 규정」 일부개정안 행정예고</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12289</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12309</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1713,44 +1713,44 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-20 10:16:06.541093+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-20 10:16:06.541093+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>14433</t>
+          <t>16313</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>366</t>
+          <t>371</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>「개인정보 보호 법규 위반에 대한 고발 기준」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12278</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12310</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1770,44 +1770,44 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:08.116520+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:08.116520+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14422</t>
+          <t>16312</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1282</t>
+          <t>372</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>「개인정보 이노베이션 존」 신규 운영기관 공모</t>
+          <t>「개인정보 보호 법규 위반에 대한 징계권고 기준」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12287</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12311</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1817,54 +1817,54 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-20 10:00:27.102836+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-20 10:00:27.102836+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>16311</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1283</t>
+          <t>373</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>개인정보위, ‘본인전송요구권’ 사전협의 지원 시범운영 7월 31일까지 추가신청 받는다</t>
+          <t>「개인정보 보호법 위반에 대한 공표 및 공표명령 지침」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12288</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12312</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1874,54 +1874,54 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-20 10:00:27.102836+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-20 10:00:27.102836+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>11392</t>
+          <t>14451</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>367</t>
+          <t>369</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 위반에 대한 과징금 부과기준」 일부개정안 행정예고</t>
+          <t>본인전송요구 대리인의 사전협의 요청 시범기간 추가운영(7.20.~31.) 안내</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12282</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12289</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1931,7 +1931,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1941,44 +1941,44 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-16 13:01:06.075969+09:00</t>
+          <t>2026-07-20 10:16:06.541093+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-16 13:01:06.075969+09:00</t>
+          <t>2026-07-20 10:16:06.541093+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>11391</t>
+          <t>14433</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>368</t>
+          <t>366</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 위반에 대한 과태료 부과기준」 제정안 행정예고</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12284</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12278</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1988,7 +1988,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1998,44 +1998,44 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-16 13:01:06.075969+09:00</t>
+          <t>2026-07-20 10:01:08.116520+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-16 13:01:06.075969+09:00</t>
+          <t>2026-07-20 10:01:08.116520+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>11221</t>
+          <t>14422</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1281</t>
+          <t>1282</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AI 혁신을 뒷받침하고 국민 권익을 증진하는 예방중심 개인정보 보호 실현</t>
+          <t>「개인정보 이노베이션 존」 신규 운영기관 공모</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12281</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12287</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>혁신기획담당관</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -2055,44 +2055,44 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-16 11:00:27.819143+09:00</t>
+          <t>2026-07-20 10:00:27.102836+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-16 11:00:27.819143+09:00</t>
+          <t>2026-07-20 10:00:27.102836+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>10301</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1280</t>
+          <t>1283</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.15.자)</t>
+          <t>개인정보위, ‘본인전송요구권’ 사전협의 지원 시범운영 7월 31일까지 추가신청 받는다</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12276</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12288</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -2112,44 +2112,44 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-15 09:45:30.272302+09:00</t>
+          <t>2026-07-20 10:00:27.102836+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-15 09:45:30.272302+09:00</t>
+          <t>2026-07-20 10:00:27.102836+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>9501</t>
+          <t>11392</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1279</t>
+          <t>367</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>개인정보 전송요구권 전송체계 기술적 기틀, 고용⋅교육 부문까지 확대 마련</t>
+          <t>「개인정보 보호법 위반에 대한 과징금 부과기준」 일부개정안 행정예고</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12266</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12282</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>인프라표준화팀</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -2159,54 +2159,54 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-14 10:00:29.933870+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-14 10:00:29.933870+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>9381</t>
+          <t>11391</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1280</t>
+          <t>368</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>정보주체의 본인전송요구권, 더 안전하게 이용할 수 있습니다</t>
+          <t>「개인정보 보호법 위반에 대한 과태료 부과기준」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12273</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12284</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>범정부마이데이터추진단 전략기획팀</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2216,111 +2216,111 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-14 08:30:26.475160+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-14 08:30:26.475160+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>9271</t>
+          <t>11221</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>365</t>
+          <t>1281</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>공공기관 종합청렴도 평가 관련 개인정보 제3자 제공사항 알림</t>
+          <t>AI 혁신을 뒷받침하고 국민 권익을 증진하는 예방중심 개인정보 보호 실현</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12267</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12281</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>법무감사담당관</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-13 17:16:17.898453+09:00</t>
+          <t>2026-07-16 11:00:27.819143+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-13 17:16:17.898453+09:00</t>
+          <t>2026-07-16 11:00:27.819143+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>6541</t>
+          <t>10301</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1278</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>개인정보 온라인 불법유통 청년들이 직접 차단한다.</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.15.자)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12262</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12276</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>조사2과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2330,7 +2330,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -2340,44 +2340,44 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-10 14:00:31.832545+09:00</t>
+          <t>2026-07-15 09:45:30.272302+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-10 14:00:31.832545+09:00</t>
+          <t>2026-07-15 09:45:30.272302+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>5491</t>
+          <t>9501</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>364</t>
+          <t>1279</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>제4회 개인정보보호 모의재판 경연대회 참가자 모집</t>
+          <t>개인정보 전송요구권 전송체계 기술적 기틀, 고용⋅교육 부문까지 확대 마련</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12245</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12266</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>침해평가과</t>
+          <t>인프라표준화팀</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2387,54 +2387,54 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-09 11:01:05.002078+09:00</t>
+          <t>2026-07-14 10:00:29.933870+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-09 11:01:05.002078+09:00</t>
+          <t>2026-07-14 10:00:29.933870+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>5402</t>
+          <t>9381</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1276</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>개인정보위, 안전조치 의무 위반 3개 사업자 제재</t>
+          <t>정보주체의 본인전송요구권, 더 안전하게 이용할 수 있습니다</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12242</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12273</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>장석인</t>
+          <t>범정부마이데이터추진단 전략기획팀</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>303</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2454,101 +2454,101 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-14 08:30:26.475160+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-14 08:30:26.475160+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>5401</t>
+          <t>9271</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1277</t>
+          <t>365</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>미래의 개인정보 법률 전문가 모여 인공지능 시대 법적 쟁점 논의한다</t>
+          <t>공공기관 종합청렴도 평가 관련 개인정보 제3자 제공사항 알림</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12243</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12267</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>침해평가과</t>
+          <t>법무감사담당관</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-13 17:16:17.898453+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-13 17:16:17.898453+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>5391</t>
+          <t>6541</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>363</t>
+          <t>1278</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>「개인정보 보호책임자 경력 인정에 관한 고시」 일부개정고시안 행정예고</t>
+          <t>개인정보 온라인 불법유통 청년들이 직접 차단한다.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12244</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12262</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>조사2과</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2558,54 +2558,54 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-09 09:46:03.809898+09:00</t>
+          <t>2026-07-10 14:00:31.832545+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-09 09:46:03.809898+09:00</t>
+          <t>2026-07-10 14:00:31.832545+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>4581</t>
+          <t>5491</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1275</t>
+          <t>364</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>개인정보위, 응용프로그램 인터페이스(API) 활용 확대에 따른 개인정보 유출 예방 당부</t>
+          <t>제4회 개인정보보호 모의재판 경연대회 참가자 모집</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12241</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12245</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>사전실태점검과</t>
+          <t>침해평가과</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2615,54 +2615,54 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-08 10:00:27.128578+09:00</t>
+          <t>2026-07-09 11:01:05.002078+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-08 10:00:27.128578+09:00</t>
+          <t>2026-07-09 11:01:05.002078+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3251</t>
+          <t>5402</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>1276</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026년 가명정보 활용 지원체계 설명회 개최 안내</t>
+          <t>개인정보위, 안전조치 의무 위반 3개 사업자 제재</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12238</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12242</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>장석인</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2672,54 +2672,54 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-06 13:46:04.662402+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-06 13:46:04.662402+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>3182</t>
+          <t>5401</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1273</t>
+          <t>1277</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>개인정보 처리방침 평가, 국민 눈높이에서 더 꼼꼼히 본다</t>
+          <t>미래의 개인정보 법률 전문가 모여 인공지능 시대 법적 쟁점 논의한다</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12236</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12243</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>침해평가과</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2729,7 +2729,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2739,44 +2739,44 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>3181</t>
+          <t>5391</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1274</t>
+          <t>363</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>개인정보위, 교육‧고용 분야까지 개인정보 제3자 전송요구권 확대 추진</t>
+          <t>「개인정보 보호책임자 경력 인정에 관한 고시」 일부개정고시안 행정예고</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12237</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12244</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2786,54 +2786,54 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-09 09:46:03.809898+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-09 09:46:03.809898+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1043</t>
+          <t>4581</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>1275</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>개인정보위, 대전에서 ‘찾아가는 개인정보 현장 컨설팅 및 교육’ 개최</t>
+          <t>개인정보위, 응용프로그램 인터페이스(API) 활용 확대에 따른 개인정보 유출 예방 당부</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12227</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12241</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>사전실태점검과</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2853,44 +2853,44 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-03 16:00:28.543767+09:00</t>
+          <t>2026-07-08 10:00:27.128578+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-03 16:00:28.543767+09:00</t>
+          <t>2026-07-08 10:00:27.128578+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>3251</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1272</t>
+          <t>362</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.3.자)</t>
+          <t>2026년 가명정보 활용 지원체계 설명회 개최 안내</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12229</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12238</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2900,54 +2900,54 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-03 15:30:33.546332+09:00</t>
+          <t>2026-07-06 13:46:04.662402+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-03 15:30:33.546332+09:00</t>
+          <t>2026-07-06 13:46:04.662402+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>561</t>
+          <t>3182</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>1271</t>
+          <t>1273</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>신뢰로 여는 인공지능(AI) 혁신, 달라지는 개인정보 체계로 이끈다</t>
+          <t>개인정보 처리방침 평가, 국민 눈높이에서 더 꼼꼼히 본다</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12228</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12236</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>개인정보보호정책과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2957,7 +2957,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>60</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2967,44 +2967,44 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-03 10:00:33.422568+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-03 10:00:33.422568+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>3181</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>1269</t>
+          <t>1274</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>개인정보위, 인공지능(AI) 시대 데이터 혁신적 활용을 지역 주도로 확산한다.</t>
+          <t>개인정보위, 교육‧고용 분야까지 개인정보 제3자 전송요구권 확대 추진</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12225</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12237</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>58</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -3024,44 +3024,44 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-02 16:45:30.717611+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-02 16:45:30.717611+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1043</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>1269</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>개인정보위, 개인정보보호 현장 간담회 개최</t>
+          <t>개인정보위, 대전에서 ‘찾아가는 개인정보 현장 컨설팅 및 교육’ 개최</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12224</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12227</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>조사1과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3071,7 +3071,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -3081,44 +3081,44 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-03 16:00:28.543767+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-03 16:00:28.543767+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1001</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1266</t>
+          <t>1272</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>글로벌 개인정보 감독기구에 인공지능(AI) 대응 ‘실전해법’ 제시</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.3.자)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12218</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12229</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>국제협력담당관</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>924</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -3138,44 +3138,44 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-03 15:30:33.546332+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-03 15:30:33.546332+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>561</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>1267</t>
+          <t>1271</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>투숙객 개인정보보호에 앞장선 호텔, 호텔업 등급평가시 우대</t>
+          <t>신뢰로 여는 인공지능(AI) 혁신, 달라지는 개인정보 체계로 이끈다</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12219</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12228</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>개인정보보호정책과</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -3185,7 +3185,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1074</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -3195,44 +3195,44 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-03 10:00:33.422568+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-03 10:00:33.422568+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>281</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>1268</t>
+          <t>1269</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.1.자)</t>
+          <t>개인정보위, 인공지능(AI) 시대 데이터 혁신적 활용을 지역 주도로 확산한다.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12220</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12225</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3242,7 +3242,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>743</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -3252,44 +3252,44 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 16:45:30.717611+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 16:45:30.717611+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>361</t>
+          <t>1269</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령(안) 입법예고</t>
+          <t>개인정보위, 개인정보보호 현장 간담회 개최</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12216</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12224</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>범정부 마이데이터추진단</t>
+          <t>조사1과</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3299,54 +3299,54 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>98</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>1265</t>
+          <t>1266</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.6.30.자)</t>
+          <t>글로벌 개인정보 감독기구에 인공지능(AI) 대응 ‘실전해법’ 제시</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12217</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12218</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>국제협력담당관</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3356,7 +3356,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1029</t>
+          <t>924</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3378,32 +3378,32 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>1267</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고</t>
+          <t>투숙객 개인정보보호에 앞장선 호텔, 호텔업 등급평가시 우대</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12202</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12219</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3413,54 +3413,54 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>2800</t>
+          <t>1074</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>1262</t>
+          <t>1268</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>개인정보위원장, G7 개인정보 감독기구 라운드테이블 참석</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.1.자)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12201</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12220</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>국제협력담당관</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>2144</t>
+          <t>743</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3492,32 +3492,32 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>1263</t>
+          <t>361</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>「2026 개인정보 보호·활용 기술 대상」 참여기업 모집</t>
+          <t>「개인정보 보호법 시행령」 일부개정령(안) 입법예고</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12203</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12216</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>범정부 마이데이터추진단</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3527,54 +3527,54 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>2092</t>
+          <t>1842</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>1264</t>
+          <t>1265</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>AI 범죄 대응 범부처 협의체 출범</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.6.30.자)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12204</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12217</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>인공지능프라이버시팀</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3584,7 +3584,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>2638</t>
+          <t>1029</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3606,32 +3606,32 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>359</t>
+          <t>360</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>본인전송요구 대리인의 사전협의 요청 시범기간(6.25.~7.10.) 운영 안내</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12200</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12202</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>신기술개인정보과</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3641,7 +3641,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>3745</t>
+          <t>2800</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3663,32 +3663,32 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>1260</t>
+          <t>1262</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>개인정보위, 상조서비스 개인정보 보호 취약요인 선제 점검</t>
+          <t>개인정보위원장, G7 개인정보 감독기구 라운드테이블 참석</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12197</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12201</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>사전실태점검과</t>
+          <t>국제협력담당관</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3698,7 +3698,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>2754</t>
+          <t>2144</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3720,32 +3720,32 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>1261</t>
+          <t>1263</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>개인정보위, 국민이 필요로 하는 정보 중심 ‘본인전송요구권’ 안착 지원한다</t>
+          <t>「2026 개인정보 보호·활용 기술 대상」 참여기업 모집</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12198</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12203</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>신기술개인정보과</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3755,7 +3755,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>3085</t>
+          <t>2092</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3777,32 +3777,32 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>358</t>
+          <t>1264</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>정보보호 및 개인정보보호 관리체계 심사기관 지정 공고(제2026-73호)</t>
+          <t>AI 범죄 대응 범부처 협의체 출범</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12185</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12204</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>인공지능프라이버시팀</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3812,54 +3812,54 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>7681</t>
+          <t>2638</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>357</t>
+          <t>359</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>「자율기구 공공실태점검단 설치 및 운영에 관한 규정」 발령(2026-70)</t>
+          <t>본인전송요구 대리인의 사전협의 요청 시범기간(6.25.~7.10.) 운영 안내</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12174</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12200</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>혁신기획담당관</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>6533</t>
+          <t>3745</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3891,32 +3891,32 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>1260</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>공공기관 개인정보 보호수준 평가단원 지원 공고</t>
+          <t>개인정보위, 상조서비스 개인정보 보호 취약요인 선제 점검</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12160</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12197</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>사전실태점검과</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3926,54 +3926,54 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>9023</t>
+          <t>2754</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>352</t>
+          <t>1261</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
+          <t>개인정보위, 국민이 필요로 하는 정보 중심 ‘본인전송요구권’ 안착 지원한다</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12126</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12198</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>개인정보보호정책과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -3983,54 +3983,54 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>11169</t>
+          <t>3085</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>354</t>
+          <t>358</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
+          <t>정보보호 및 개인정보보호 관리체계 심사기관 지정 공고(제2026-73호)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12131</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12185</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4040,7 +4040,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>13472</t>
+          <t>7681</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4062,32 +4062,32 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>355</t>
+          <t>357</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+          <t>「자율기구 공공실태점검단 설치 및 운영에 관한 규정」 발령(2026-70)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12136</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12174</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -4097,7 +4097,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>9724</t>
+          <t>6533</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4119,55 +4119,283 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>356</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>공공기관 개인정보 보호수준 평가단원 지원 공고</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12160</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>자율보호정책과</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>9023</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>352</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12126</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>개인정보보호정책과</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>11169</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>354</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12131</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>조사총괄과</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>13472</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>355</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12136</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>신기술개인정보과</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>9724</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>19</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>353</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>「개인정보 처리 방법에 관한 고시」 일부개정고시안 행정예고</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12127</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>전략기획팀</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
         <is>
           <t>11519</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>공지사항</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="J49" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="K49" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-22 15:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -5602,7 +5602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5665,7 +5665,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>16051</t>
+          <t>16464</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5675,12 +5675,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
+          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -5690,35 +5690,35 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5728,22 +5728,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -5759,19 +5759,19 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -5781,12 +5781,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -5796,7 +5796,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -5812,34 +5812,34 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -5849,7 +5849,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -5857,56 +5857,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -5914,7 +5910,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -5922,34 +5922,34 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -5959,7 +5959,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -5970,96 +5970,92 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -6069,7 +6065,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -6077,7 +6073,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6085,19 +6085,19 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6107,12 +6107,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -6122,12 +6122,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -6138,19 +6138,19 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -6160,22 +6160,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -6191,19 +6191,19 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -6213,12 +6213,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -6228,7 +6228,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -6239,96 +6239,92 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -6338,35 +6334,39 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -6376,22 +6376,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -6402,24 +6402,24 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -6429,12 +6429,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -6444,7 +6444,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -6455,24 +6455,24 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -6482,22 +6482,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -6513,44 +6513,44 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -6566,44 +6566,44 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -6611,31 +6611,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -6645,12 +6641,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -6660,7 +6656,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -6692,22 +6688,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -6717,7 +6713,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -6725,27 +6721,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -6755,12 +6755,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -6770,113 +6770,113 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -6884,31 +6884,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -6918,12 +6914,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -6933,7 +6929,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -6965,32 +6961,32 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -6998,7 +6994,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7018,22 +7018,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -7043,7 +7043,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -7071,22 +7071,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -7096,19 +7096,15 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7128,7 +7124,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -7138,12 +7134,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -7153,7 +7149,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -7185,40 +7181,44 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7238,22 +7238,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -7271,11 +7271,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7295,32 +7291,32 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -7328,7 +7324,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7336,34 +7336,34 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -7373,7 +7373,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -7384,49 +7384,49 @@
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -7454,22 +7454,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -7479,7 +7479,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -7507,32 +7507,32 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -7560,22 +7560,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -7585,39 +7585,35 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -7627,27 +7623,27 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -7674,32 +7670,32 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -7707,52 +7703,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -7780,32 +7780,32 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -7833,32 +7833,32 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -7886,32 +7886,32 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -7919,46 +7919,42 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14403</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -7968,7 +7964,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>6587</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -7976,52 +7972,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -8041,6 +8041,59 @@
         </is>
       </c>
       <c r="K45" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-22 18:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -5602,7 +5602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:K47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5665,7 +5665,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>16464</t>
+          <t>16691</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5675,12 +5675,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
+          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -5690,35 +5690,35 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>278</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>16051</t>
+          <t>16464</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5728,12 +5728,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
+          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -5743,35 +5743,35 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -5781,22 +5781,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -5812,19 +5812,19 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -5834,12 +5834,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -5849,7 +5849,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -5865,34 +5865,34 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -5902,7 +5902,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -5910,56 +5910,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -5967,7 +5963,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -5975,34 +5975,34 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -6012,7 +6012,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -6023,96 +6023,92 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -6122,7 +6118,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -6130,7 +6126,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6138,19 +6138,19 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -6160,12 +6160,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -6175,12 +6175,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -6191,19 +6191,19 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -6213,22 +6213,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -6244,19 +6244,19 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -6266,12 +6266,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -6281,7 +6281,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -6292,96 +6292,92 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -6391,35 +6387,39 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -6429,22 +6429,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -6455,24 +6455,24 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -6482,12 +6482,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -6497,7 +6497,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -6508,24 +6508,24 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -6535,22 +6535,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -6566,44 +6566,44 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -6619,44 +6619,44 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -6664,31 +6664,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -6698,12 +6694,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -6713,7 +6709,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -6745,22 +6741,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -6770,7 +6766,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -6778,27 +6774,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -6808,12 +6808,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -6823,113 +6823,113 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -6937,31 +6937,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -6971,12 +6967,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -6986,7 +6982,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -7018,32 +7014,32 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -7051,7 +7047,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7071,22 +7071,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -7096,7 +7096,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -7124,22 +7124,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -7149,19 +7149,15 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7181,7 +7177,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7191,12 +7187,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -7206,7 +7202,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -7238,40 +7234,44 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7291,22 +7291,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -7316,7 +7316,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -7324,11 +7324,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7348,32 +7344,32 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -7381,7 +7377,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7389,34 +7389,34 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -7426,7 +7426,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -7437,49 +7437,49 @@
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -7507,22 +7507,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -7532,7 +7532,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -7560,32 +7560,32 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -7613,22 +7613,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -7638,39 +7638,35 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7680,27 +7676,27 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -7727,32 +7723,32 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -7760,52 +7756,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -7833,32 +7833,32 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -7886,32 +7886,32 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -7939,32 +7939,32 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -7972,46 +7972,42 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14403</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -8021,7 +8017,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>6587</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -8029,52 +8025,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -8094,6 +8094,59 @@
         </is>
       </c>
       <c r="K46" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-23 09:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -5602,7 +5602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K47"/>
+  <dimension ref="A1:K50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5665,22 +5665,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>16691</t>
+          <t>16785</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1496</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -5690,50 +5690,50 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>16464</t>
+          <t>16784</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1497</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -5743,7 +5743,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>260</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -5759,34 +5759,34 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>16051</t>
+          <t>16781</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -5796,35 +5796,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>242</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16691</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -5834,22 +5838,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>278</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -5865,19 +5869,19 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>16464</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -5887,75 +5891,75 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -5963,56 +5967,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -6023,24 +6023,24 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6050,22 +6050,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -6081,19 +6081,19 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6103,17 +6103,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -6123,7 +6123,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -6138,49 +6138,49 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -6191,19 +6191,19 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -6213,22 +6213,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -6239,57 +6239,61 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6297,19 +6301,19 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -6319,87 +6323,83 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6407,19 +6407,19 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -6429,22 +6429,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -6455,24 +6455,24 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -6482,22 +6482,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -6508,77 +6508,81 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -6588,22 +6592,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -6619,44 +6623,44 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -6667,49 +6671,49 @@
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -6717,56 +6721,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -6774,56 +6774,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -6839,34 +6835,34 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -6876,15 +6872,19 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6892,44 +6892,44 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -6937,52 +6937,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -6990,68 +6994,60 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7059,44 +7055,44 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -7107,49 +7103,49 @@
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -7157,7 +7153,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7177,7 +7177,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7187,27 +7187,27 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -7234,22 +7234,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -7259,19 +7259,15 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7291,32 +7287,32 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -7344,7 +7340,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -7354,27 +7350,27 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -7401,40 +7397,44 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7442,44 +7442,44 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -7490,49 +7490,49 @@
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -7540,52 +7540,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -7596,49 +7600,49 @@
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -7666,89 +7670,85 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -7756,56 +7756,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -7833,85 +7829,89 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -7919,52 +7919,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -7992,32 +7996,32 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -8025,56 +8029,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -8102,32 +8102,32 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -8147,6 +8147,169 @@
         </is>
       </c>
       <c r="K47" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>14403</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>공지</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>6587</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>950</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>51749</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-23 10:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -1605,7 +1605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1668,32 +1668,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>16314</t>
+          <t>16883</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>370</t>
+          <t>1285</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>「개인정보 보호위원회의 조사 및 처분에 관한 규정」 일부개정안 행정예고</t>
+          <t>국민이 신뢰할 수 있는 공공 인공지능 전환(AX),프라이버시 보호로 적극 뒷받침</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12309</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12307</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>인공지능프라이버시팀</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1703,54 +1703,54 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-22 13:01:11.478354+09:00</t>
+          <t>2026-07-23 10:00:38.625145+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-22 13:01:11.478354+09:00</t>
+          <t>2026-07-23 10:00:38.625145+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>16313</t>
+          <t>16882</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>371</t>
+          <t>1286</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>「개인정보 보호 법규 위반에 대한 고발 기준」 제정안 행정예고</t>
+          <t>대도약의 골든타임, 초격차 성장동력 확보와 AI 생태계 발전기반 강화</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12310</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12308</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>인공지능프라이버시팀</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1760,54 +1760,54 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-22 13:01:11.478354+09:00</t>
+          <t>2026-07-23 10:00:38.625145+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-22 13:01:11.478354+09:00</t>
+          <t>2026-07-23 10:00:38.625145+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>16312</t>
+          <t>16881</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>372</t>
+          <t>1287</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>「개인정보 보호 법규 위반에 대한 징계권고 기준」 제정안 행정예고</t>
+          <t>개인정보위, 적법 근거 없이 개인정보수집·이용한 틱톡·애플 제재</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12311</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12330</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>조사1과</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1817,44 +1817,44 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-22 13:01:11.478354+09:00</t>
+          <t>2026-07-23 10:00:38.625145+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-22 13:01:11.478354+09:00</t>
+          <t>2026-07-23 10:00:38.625145+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>16311</t>
+          <t>16314</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>373</t>
+          <t>370</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 위반에 대한 공표 및 공표명령 지침」 제정안 행정예고</t>
+          <t>「개인정보 보호위원회의 조사 및 처분에 관한 규정」 일부개정안 행정예고</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12312</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12309</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1896,32 +1896,32 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>14451</t>
+          <t>16313</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>369</t>
+          <t>371</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>본인전송요구 대리인의 사전협의 요청 시범기간 추가운영(7.20.~31.) 안내</t>
+          <t>「개인정보 보호 법규 위반에 대한 고발 기준」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12289</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12310</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1931,7 +1931,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1941,44 +1941,44 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-20 10:16:06.541093+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-20 10:16:06.541093+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>14433</t>
+          <t>16312</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>366</t>
+          <t>372</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>「개인정보 보호 법규 위반에 대한 징계권고 기준」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12278</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12311</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1988,7 +1988,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1998,44 +1998,44 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:08.116520+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:08.116520+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>14422</t>
+          <t>16311</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1282</t>
+          <t>373</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>「개인정보 이노베이션 존」 신규 운영기관 공모</t>
+          <t>「개인정보 보호법 위반에 대한 공표 및 공표명령 지침」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12287</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12312</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -2050,39 +2050,39 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-20 10:00:27.102836+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-20 10:00:27.102836+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14451</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1283</t>
+          <t>369</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>개인정보위, ‘본인전송요구권’ 사전협의 지원 시범운영 7월 31일까지 추가신청 받는다</t>
+          <t>본인전송요구 대리인의 사전협의 요청 시범기간 추가운영(7.20.~31.) 안내</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12288</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12289</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -2102,54 +2102,54 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-20 10:00:27.102836+09:00</t>
+          <t>2026-07-20 10:16:06.541093+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-20 10:00:27.102836+09:00</t>
+          <t>2026-07-20 10:16:06.541093+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>11392</t>
+          <t>14433</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>367</t>
+          <t>366</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 위반에 대한 과징금 부과기준」 일부개정안 행정예고</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12282</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12278</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -2169,44 +2169,44 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-16 13:01:06.075969+09:00</t>
+          <t>2026-07-20 10:01:08.116520+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-16 13:01:06.075969+09:00</t>
+          <t>2026-07-20 10:01:08.116520+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>11391</t>
+          <t>14422</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>368</t>
+          <t>1282</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 위반에 대한 과태료 부과기준」 제정안 행정예고</t>
+          <t>「개인정보 이노베이션 존」 신규 운영기관 공모</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12284</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12287</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2221,49 +2221,49 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-16 13:01:06.075969+09:00</t>
+          <t>2026-07-20 10:00:27.102836+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-16 13:01:06.075969+09:00</t>
+          <t>2026-07-20 10:00:27.102836+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>11221</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1281</t>
+          <t>1283</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AI 혁신을 뒷받침하고 국민 권익을 증진하는 예방중심 개인정보 보호 실현</t>
+          <t>개인정보위, ‘본인전송요구권’ 사전협의 지원 시범운영 7월 31일까지 추가신청 받는다</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12281</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12288</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>혁신기획담당관</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -2283,44 +2283,44 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-16 11:00:27.819143+09:00</t>
+          <t>2026-07-20 10:00:27.102836+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-16 11:00:27.819143+09:00</t>
+          <t>2026-07-20 10:00:27.102836+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>10301</t>
+          <t>11392</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1280</t>
+          <t>367</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.15.자)</t>
+          <t>「개인정보 보호법 위반에 대한 과징금 부과기준」 일부개정안 행정예고</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12276</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12282</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2330,54 +2330,54 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-15 09:45:30.272302+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-15 09:45:30.272302+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>9501</t>
+          <t>11391</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1279</t>
+          <t>368</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>개인정보 전송요구권 전송체계 기술적 기틀, 고용⋅교육 부문까지 확대 마련</t>
+          <t>「개인정보 보호법 위반에 대한 과태료 부과기준」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12266</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12284</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>인프라표준화팀</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2392,49 +2392,49 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-14 10:00:29.933870+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-14 10:00:29.933870+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>9381</t>
+          <t>11221</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1280</t>
+          <t>1281</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>정보주체의 본인전송요구권, 더 안전하게 이용할 수 있습니다</t>
+          <t>AI 혁신을 뒷받침하고 국민 권익을 증진하는 예방중심 개인정보 보호 실현</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12273</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12281</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>범정부마이데이터추진단 전략기획팀</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2454,101 +2454,101 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-14 08:30:26.475160+09:00</t>
+          <t>2026-07-16 11:00:27.819143+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-14 08:30:26.475160+09:00</t>
+          <t>2026-07-16 11:00:27.819143+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>9271</t>
+          <t>10301</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>365</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>공공기관 종합청렴도 평가 관련 개인정보 제3자 제공사항 알림</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.15.자)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12267</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12276</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>법무감사담당관</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-13 17:16:17.898453+09:00</t>
+          <t>2026-07-15 09:45:30.272302+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-13 17:16:17.898453+09:00</t>
+          <t>2026-07-15 09:45:30.272302+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>6541</t>
+          <t>9501</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1278</t>
+          <t>1279</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>개인정보 온라인 불법유통 청년들이 직접 차단한다.</t>
+          <t>개인정보 전송요구권 전송체계 기술적 기틀, 고용⋅교육 부문까지 확대 마련</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12262</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12266</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>조사2과</t>
+          <t>인프라표준화팀</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2568,44 +2568,44 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-10 14:00:31.832545+09:00</t>
+          <t>2026-07-14 10:00:29.933870+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-10 14:00:31.832545+09:00</t>
+          <t>2026-07-14 10:00:29.933870+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>5491</t>
+          <t>9381</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>364</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>제4회 개인정보보호 모의재판 경연대회 참가자 모집</t>
+          <t>정보주체의 본인전송요구권, 더 안전하게 이용할 수 있습니다</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12245</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12273</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>침해평가과</t>
+          <t>범정부마이데이터추진단 전략기획팀</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2615,111 +2615,111 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>303</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-09 11:01:05.002078+09:00</t>
+          <t>2026-07-14 08:30:26.475160+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-09 11:01:05.002078+09:00</t>
+          <t>2026-07-14 08:30:26.475160+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>5402</t>
+          <t>9271</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1276</t>
+          <t>365</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>개인정보위, 안전조치 의무 위반 3개 사업자 제재</t>
+          <t>공공기관 종합청렴도 평가 관련 개인정보 제3자 제공사항 알림</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12242</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12267</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>장석인</t>
+          <t>법무감사담당관</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-13 17:16:17.898453+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-13 17:16:17.898453+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>5401</t>
+          <t>6541</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1277</t>
+          <t>1278</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>미래의 개인정보 법률 전문가 모여 인공지능 시대 법적 쟁점 논의한다</t>
+          <t>개인정보 온라인 불법유통 청년들이 직접 차단한다.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12243</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12262</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>침해평가과</t>
+          <t>조사2과</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2729,7 +2729,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2739,39 +2739,39 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-10 14:00:31.832545+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-10 14:00:31.832545+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>5391</t>
+          <t>5491</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>363</t>
+          <t>364</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>「개인정보 보호책임자 경력 인정에 관한 고시」 일부개정고시안 행정예고</t>
+          <t>제4회 개인정보보호 모의재판 경연대회 참가자 모집</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12244</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12245</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>침해평가과</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2796,44 +2796,44 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-09 09:46:03.809898+09:00</t>
+          <t>2026-07-09 11:01:05.002078+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-09 09:46:03.809898+09:00</t>
+          <t>2026-07-09 11:01:05.002078+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>4581</t>
+          <t>5402</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1275</t>
+          <t>1276</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>개인정보위, 응용프로그램 인터페이스(API) 활용 확대에 따른 개인정보 유출 예방 당부</t>
+          <t>개인정보위, 안전조치 의무 위반 3개 사업자 제재</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12241</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12242</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>사전실태점검과</t>
+          <t>장석인</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2853,44 +2853,44 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-08 10:00:27.128578+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-08 10:00:27.128578+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>3251</t>
+          <t>5401</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>1277</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026년 가명정보 활용 지원체계 설명회 개최 안내</t>
+          <t>미래의 개인정보 법률 전문가 모여 인공지능 시대 법적 쟁점 논의한다</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12238</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12243</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>침해평가과</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2900,44 +2900,44 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-06 13:46:04.662402+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-06 13:46:04.662402+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>3182</t>
+          <t>5391</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>1273</t>
+          <t>363</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>개인정보 처리방침 평가, 국민 눈높이에서 더 꼼꼼히 본다</t>
+          <t>「개인정보 보호책임자 경력 인정에 관한 고시」 일부개정고시안 행정예고</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12236</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12244</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2957,54 +2957,54 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-09 09:46:03.809898+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-09 09:46:03.809898+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>3181</t>
+          <t>4581</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>1274</t>
+          <t>1275</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>개인정보위, 교육‧고용 분야까지 개인정보 제3자 전송요구권 확대 추진</t>
+          <t>개인정보위, 응용프로그램 인터페이스(API) 활용 확대에 따른 개인정보 유출 예방 당부</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12237</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12241</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>사전실태점검과</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -3024,44 +3024,44 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-08 10:00:27.128578+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-08 10:00:27.128578+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1043</t>
+          <t>3251</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>362</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>개인정보위, 대전에서 ‘찾아가는 개인정보 현장 컨설팅 및 교육’ 개최</t>
+          <t>2026년 가명정보 활용 지원체계 설명회 개최 안내</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12227</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12238</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3071,54 +3071,54 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-03 16:00:28.543767+09:00</t>
+          <t>2026-07-06 13:46:04.662402+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-03 16:00:28.543767+09:00</t>
+          <t>2026-07-06 13:46:04.662402+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>3182</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1272</t>
+          <t>1273</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.3.자)</t>
+          <t>개인정보 처리방침 평가, 국민 눈높이에서 더 꼼꼼히 본다</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12229</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12236</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>60</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -3138,44 +3138,44 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-03 15:30:33.546332+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-03 15:30:33.546332+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>561</t>
+          <t>3181</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>1271</t>
+          <t>1274</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>신뢰로 여는 인공지능(AI) 혁신, 달라지는 개인정보 체계로 이끈다</t>
+          <t>개인정보위, 교육‧고용 분야까지 개인정보 제3자 전송요구권 확대 추진</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12228</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12237</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>개인정보보호정책과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -3185,7 +3185,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>58</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -3195,44 +3195,44 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-03 10:00:33.422568+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-03 10:00:33.422568+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>1043</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>1269</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>개인정보위, 인공지능(AI) 시대 데이터 혁신적 활용을 지역 주도로 확산한다.</t>
+          <t>개인정보위, 대전에서 ‘찾아가는 개인정보 현장 컨설팅 및 교육’ 개최</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12225</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12227</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3242,7 +3242,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -3252,56 +3252,56 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-02 16:45:30.717611+09:00</t>
+          <t>2026-07-03 16:00:28.543767+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-02 16:45:30.717611+09:00</t>
+          <t>2026-07-03 16:00:28.543767+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>1001</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1272</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.3.자)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12229</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>운영지원과</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>1269</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>개인정보위, 개인정보보호 현장 간담회 개최</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12224</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>조사1과</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>98</t>
-        </is>
-      </c>
       <c r="I30" t="inlineStr">
         <is>
           <t>보도자료</t>
@@ -3309,44 +3309,44 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-03 15:30:33.546332+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-03 15:30:33.546332+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>561</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>1266</t>
+          <t>1271</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>글로벌 개인정보 감독기구에 인공지능(AI) 대응 ‘실전해법’ 제시</t>
+          <t>신뢰로 여는 인공지능(AI) 혁신, 달라지는 개인정보 체계로 이끈다</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12218</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12228</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>국제협력담당관</t>
+          <t>개인정보보호정책과</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3356,7 +3356,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>924</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3366,44 +3366,44 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-03 10:00:33.422568+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-03 10:00:33.422568+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>281</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>1267</t>
+          <t>1269</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>투숙객 개인정보보호에 앞장선 호텔, 호텔업 등급평가시 우대</t>
+          <t>개인정보위, 인공지능(AI) 시대 데이터 혁신적 활용을 지역 주도로 확산한다.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12219</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12225</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3413,7 +3413,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1074</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3423,44 +3423,44 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 16:45:30.717611+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 16:45:30.717611+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>1268</t>
+          <t>1269</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.1.자)</t>
+          <t>개인정보위, 개인정보보호 현장 간담회 개최</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12220</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12224</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>조사1과</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>743</t>
+          <t>98</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3492,32 +3492,32 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>361</t>
+          <t>1266</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령(안) 입법예고</t>
+          <t>글로벌 개인정보 감독기구에 인공지능(AI) 대응 ‘실전해법’ 제시</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12216</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12218</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>범정부 마이데이터추진단</t>
+          <t>국제협력담당관</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3527,54 +3527,54 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>924</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>1265</t>
+          <t>1267</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.6.30.자)</t>
+          <t>투숙객 개인정보보호에 앞장선 호텔, 호텔업 등급평가시 우대</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12217</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12219</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3584,7 +3584,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1029</t>
+          <t>1074</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3606,32 +3606,32 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>1268</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.1.자)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12202</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12220</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3641,54 +3641,54 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>2800</t>
+          <t>743</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>1262</t>
+          <t>361</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>개인정보위원장, G7 개인정보 감독기구 라운드테이블 참석</t>
+          <t>「개인정보 보호법 시행령」 일부개정령(안) 입법예고</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12201</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12216</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>국제협력담당관</t>
+          <t>범정부 마이데이터추진단</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3698,54 +3698,54 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>2144</t>
+          <t>1842</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>1263</t>
+          <t>1265</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>「2026 개인정보 보호·활용 기술 대상」 참여기업 모집</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.6.30.자)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12203</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12217</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3755,7 +3755,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>2092</t>
+          <t>1029</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3777,27 +3777,27 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>1264</t>
+          <t>360</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>AI 범죄 대응 범부처 협의체 출범</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12204</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12202</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>인공지능프라이버시팀</t>
+          <t>신기술개인정보과</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3812,54 +3812,54 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>2638</t>
+          <t>2800</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>359</t>
+          <t>1262</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>본인전송요구 대리인의 사전협의 요청 시범기간(6.25.~7.10.) 운영 안내</t>
+          <t>개인정보위원장, G7 개인정보 감독기구 라운드테이블 참석</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12200</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12201</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>국제협력담당관</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3869,54 +3869,54 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>3745</t>
+          <t>2144</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>1260</t>
+          <t>1263</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>개인정보위, 상조서비스 개인정보 보호 취약요인 선제 점검</t>
+          <t>「2026 개인정보 보호·활용 기술 대상」 참여기업 모집</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12197</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12203</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>사전실태점검과</t>
+          <t>신기술개인정보과</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3926,7 +3926,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>2754</t>
+          <t>2092</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3948,32 +3948,32 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>1261</t>
+          <t>1264</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>개인정보위, 국민이 필요로 하는 정보 중심 ‘본인전송요구권’ 안착 지원한다</t>
+          <t>AI 범죄 대응 범부처 협의체 출범</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12198</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12204</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>인공지능프라이버시팀</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>3085</t>
+          <t>2638</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4005,32 +4005,32 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>358</t>
+          <t>359</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>정보보호 및 개인정보보호 관리체계 심사기관 지정 공고(제2026-73호)</t>
+          <t>본인전송요구 대리인의 사전협의 요청 시범기간(6.25.~7.10.) 운영 안내</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12185</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12200</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4040,7 +4040,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>7681</t>
+          <t>3745</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4062,32 +4062,32 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>357</t>
+          <t>1260</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>「자율기구 공공실태점검단 설치 및 운영에 관한 규정」 발령(2026-70)</t>
+          <t>개인정보위, 상조서비스 개인정보 보호 취약요인 선제 점검</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12174</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12197</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>혁신기획담당관</t>
+          <t>사전실태점검과</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -4097,54 +4097,54 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>6533</t>
+          <t>2754</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>1261</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>공공기관 개인정보 보호수준 평가단원 지원 공고</t>
+          <t>개인정보위, 국민이 필요로 하는 정보 중심 ‘본인전송요구권’ 안착 지원한다</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12160</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12198</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4154,54 +4154,54 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>9023</t>
+          <t>3085</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>352</t>
+          <t>358</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
+          <t>정보보호 및 개인정보보호 관리체계 심사기관 지정 공고(제2026-73호)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12126</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12185</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>개인정보보호정책과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -4211,7 +4211,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>11169</t>
+          <t>7681</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4233,32 +4233,32 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>354</t>
+          <t>357</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
+          <t>「자율기구 공공실태점검단 설치 및 운영에 관한 규정」 발령(2026-70)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12131</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12174</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -4268,7 +4268,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>13472</t>
+          <t>6533</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -4290,32 +4290,32 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>355</t>
+          <t>356</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+          <t>공공기관 개인정보 보호수준 평가단원 지원 공고</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12136</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12160</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>9724</t>
+          <t>9023</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -4347,55 +4347,226 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>352</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12126</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>개인정보보호정책과</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>11169</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>354</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12131</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>조사총괄과</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>13472</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>355</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12136</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>신기술개인정보과</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>9724</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>19</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>353</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>「개인정보 처리 방법에 관한 고시」 일부개정고시안 행정예고</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12127</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>전략기획팀</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
         <is>
           <t>11519</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>공지사항</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="J52" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
+      <c r="K52" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-23 16:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -1605,7 +1605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K52"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1668,27 +1668,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>16883</t>
+          <t>17362</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1285</t>
+          <t>1286</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>국민이 신뢰할 수 있는 공공 인공지능 전환(AX),프라이버시 보호로 적극 뒷받침</t>
+          <t>「2026 개인정보 미래포럼」 제3차 전체회의 개최</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12307</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12329</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>인공지능프라이버시팀</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1713,34 +1713,34 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-23 10:00:38.625145+09:00</t>
+          <t>2026-07-23 16:00:30.422263+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-23 10:00:38.625145+09:00</t>
+          <t>2026-07-23 16:00:30.422263+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>16882</t>
+          <t>16883</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1286</t>
+          <t>1285</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>대도약의 골든타임, 초격차 성장동력 확보와 AI 생태계 발전기반 강화</t>
+          <t>국민이 신뢰할 수 있는 공공 인공지능 전환(AX),프라이버시 보호로 적극 뒷받침</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12308</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12307</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1782,27 +1782,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>16881</t>
+          <t>16882</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1287</t>
+          <t>1286</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>개인정보위, 적법 근거 없이 개인정보수집·이용한 틱톡·애플 제재</t>
+          <t>대도약의 골든타임, 초격차 성장동력 확보와 AI 생태계 발전기반 강화</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12330</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12308</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>조사1과</t>
+          <t>인공지능프라이버시팀</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1839,32 +1839,32 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>16314</t>
+          <t>16881</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>370</t>
+          <t>1287</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>「개인정보 보호위원회의 조사 및 처분에 관한 규정」 일부개정안 행정예고</t>
+          <t>개인정보위, 적법 근거 없이 개인정보수집·이용한 틱톡·애플 제재</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12309</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12330</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>조사1과</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1874,44 +1874,44 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-22 13:01:11.478354+09:00</t>
+          <t>2026-07-23 10:00:38.625145+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-22 13:01:11.478354+09:00</t>
+          <t>2026-07-23 10:00:38.625145+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>16313</t>
+          <t>16314</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>371</t>
+          <t>370</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>「개인정보 보호 법규 위반에 대한 고발 기준」 제정안 행정예고</t>
+          <t>「개인정보 보호위원회의 조사 및 처분에 관한 규정」 일부개정안 행정예고</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12310</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12309</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1931,7 +1931,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1953,22 +1953,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>16312</t>
+          <t>16313</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>372</t>
+          <t>371</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>「개인정보 보호 법규 위반에 대한 징계권고 기준」 제정안 행정예고</t>
+          <t>「개인정보 보호 법규 위반에 대한 고발 기준」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12311</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12310</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -2010,22 +2010,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>16311</t>
+          <t>16312</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>373</t>
+          <t>372</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 위반에 대한 공표 및 공표명령 지침」 제정안 행정예고</t>
+          <t>「개인정보 보호 법규 위반에 대한 징계권고 기준」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12312</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12311</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -2067,32 +2067,32 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>14451</t>
+          <t>16311</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>369</t>
+          <t>373</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>본인전송요구 대리인의 사전협의 요청 시범기간 추가운영(7.20.~31.) 안내</t>
+          <t>「개인정보 보호법 위반에 대한 공표 및 공표명령 지침」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12289</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12312</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -2112,39 +2112,39 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-20 10:16:06.541093+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-20 10:16:06.541093+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>14433</t>
+          <t>14451</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>366</t>
+          <t>369</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>본인전송요구 대리인의 사전협의 요청 시범기간 추가운영(7.20.~31.) 안내</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12278</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12289</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -2169,34 +2169,34 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:08.116520+09:00</t>
+          <t>2026-07-20 10:16:06.541093+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:08.116520+09:00</t>
+          <t>2026-07-20 10:16:06.541093+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>14422</t>
+          <t>14433</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1282</t>
+          <t>366</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>「개인정보 이노베이션 존」 신규 운영기관 공모</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12287</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12278</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -2216,49 +2216,49 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-20 10:00:27.102836+09:00</t>
+          <t>2026-07-20 10:01:08.116520+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-20 10:00:27.102836+09:00</t>
+          <t>2026-07-20 10:01:08.116520+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14422</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1283</t>
+          <t>1282</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>개인정보위, ‘본인전송요구권’ 사전협의 지원 시범운영 7월 31일까지 추가신청 받는다</t>
+          <t>「개인정보 이노베이션 존」 신규 운영기관 공모</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12288</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12287</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -2295,32 +2295,32 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>11392</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>367</t>
+          <t>1283</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 위반에 대한 과징금 부과기준」 일부개정안 행정예고</t>
+          <t>개인정보위, ‘본인전송요구권’ 사전협의 지원 시범운영 7월 31일까지 추가신청 받는다</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12282</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12288</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2330,44 +2330,44 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-16 13:01:06.075969+09:00</t>
+          <t>2026-07-20 10:00:27.102836+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-16 13:01:06.075969+09:00</t>
+          <t>2026-07-20 10:00:27.102836+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>11391</t>
+          <t>11392</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>368</t>
+          <t>367</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 위반에 대한 과태료 부과기준」 제정안 행정예고</t>
+          <t>「개인정보 보호법 위반에 대한 과징금 부과기준」 일부개정안 행정예고</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12284</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12282</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -2409,27 +2409,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>11221</t>
+          <t>11391</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1281</t>
+          <t>368</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AI 혁신을 뒷받침하고 국민 권익을 증진하는 예방중심 개인정보 보호 실현</t>
+          <t>「개인정보 보호법 위반에 대한 과태료 부과기준」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12281</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12284</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>혁신기획담당관</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2444,54 +2444,54 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-16 11:00:27.819143+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-16 11:00:27.819143+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>10301</t>
+          <t>11221</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1280</t>
+          <t>1281</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.15.자)</t>
+          <t>AI 혁신을 뒷받침하고 국민 권익을 증진하는 예방중심 개인정보 보호 실현</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12276</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12281</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2511,44 +2511,44 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-15 09:45:30.272302+09:00</t>
+          <t>2026-07-16 11:00:27.819143+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-15 09:45:30.272302+09:00</t>
+          <t>2026-07-16 11:00:27.819143+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>9501</t>
+          <t>10301</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1279</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>개인정보 전송요구권 전송체계 기술적 기틀, 고용⋅교육 부문까지 확대 마련</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.15.자)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12266</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12276</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>인프라표준화팀</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2568,44 +2568,44 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-14 10:00:29.933870+09:00</t>
+          <t>2026-07-15 09:45:30.272302+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-14 10:00:29.933870+09:00</t>
+          <t>2026-07-15 09:45:30.272302+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>9381</t>
+          <t>9501</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1280</t>
+          <t>1279</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>정보주체의 본인전송요구권, 더 안전하게 이용할 수 있습니다</t>
+          <t>개인정보 전송요구권 전송체계 기술적 기틀, 고용⋅교육 부문까지 확대 마련</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12273</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12266</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>범정부마이데이터추진단 전략기획팀</t>
+          <t>인프라표준화팀</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2625,39 +2625,39 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-14 08:30:26.475160+09:00</t>
+          <t>2026-07-14 10:00:29.933870+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-14 08:30:26.475160+09:00</t>
+          <t>2026-07-14 10:00:29.933870+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>9271</t>
+          <t>9381</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>365</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>공공기관 종합청렴도 평가 관련 개인정보 제3자 제공사항 알림</t>
+          <t>정보주체의 본인전송요구권, 더 안전하게 이용할 수 있습니다</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12267</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12273</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>법무감사담당관</t>
+          <t>범정부마이데이터추진단 전략기획팀</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2667,116 +2667,116 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>303</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-13 17:16:17.898453+09:00</t>
+          <t>2026-07-14 08:30:26.475160+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-13 17:16:17.898453+09:00</t>
+          <t>2026-07-14 08:30:26.475160+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>6541</t>
+          <t>9271</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1278</t>
+          <t>365</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>개인정보 온라인 불법유통 청년들이 직접 차단한다.</t>
+          <t>공공기관 종합청렴도 평가 관련 개인정보 제3자 제공사항 알림</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12262</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12267</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>조사2과</t>
+          <t>법무감사담당관</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-10 14:00:31.832545+09:00</t>
+          <t>2026-07-13 17:16:17.898453+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-10 14:00:31.832545+09:00</t>
+          <t>2026-07-13 17:16:17.898453+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>5491</t>
+          <t>6541</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>364</t>
+          <t>1278</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>제4회 개인정보보호 모의재판 경연대회 참가자 모집</t>
+          <t>개인정보 온라인 불법유통 청년들이 직접 차단한다.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12245</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12262</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>침해평가과</t>
+          <t>조사2과</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2786,49 +2786,49 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-09 11:01:05.002078+09:00</t>
+          <t>2026-07-10 14:00:31.832545+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-09 11:01:05.002078+09:00</t>
+          <t>2026-07-10 14:00:31.832545+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>5402</t>
+          <t>5491</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1276</t>
+          <t>364</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>개인정보위, 안전조치 의무 위반 3개 사업자 제재</t>
+          <t>제4회 개인정보보호 모의재판 경연대회 참가자 모집</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12242</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12245</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>장석인</t>
+          <t>침해평가과</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2843,49 +2843,49 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-09 11:01:05.002078+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-09 11:01:05.002078+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>5401</t>
+          <t>5402</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1277</t>
+          <t>1276</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>미래의 개인정보 법률 전문가 모여 인공지능 시대 법적 쟁점 논의한다</t>
+          <t>개인정보위, 안전조치 의무 위반 3개 사업자 제재</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12243</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12242</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>침해평가과</t>
+          <t>장석인</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2922,27 +2922,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>5391</t>
+          <t>5401</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>363</t>
+          <t>1277</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>「개인정보 보호책임자 경력 인정에 관한 고시」 일부개정고시안 행정예고</t>
+          <t>미래의 개인정보 법률 전문가 모여 인공지능 시대 법적 쟁점 논의한다</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12244</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12243</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>침해평가과</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2957,54 +2957,54 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-09 09:46:03.809898+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-09 09:46:03.809898+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>4581</t>
+          <t>5391</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>1275</t>
+          <t>363</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>개인정보위, 응용프로그램 인터페이스(API) 활용 확대에 따른 개인정보 유출 예방 당부</t>
+          <t>「개인정보 보호책임자 경력 인정에 관한 고시」 일부개정고시안 행정예고</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12241</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12244</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>사전실태점검과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -3014,54 +3014,54 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-08 10:00:27.128578+09:00</t>
+          <t>2026-07-09 09:46:03.809898+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-08 10:00:27.128578+09:00</t>
+          <t>2026-07-09 09:46:03.809898+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>3251</t>
+          <t>4581</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>1275</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026년 가명정보 활용 지원체계 설명회 개최 안내</t>
+          <t>개인정보위, 응용프로그램 인터페이스(API) 활용 확대에 따른 개인정보 유출 예방 당부</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12238</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12241</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>사전실태점검과</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3071,49 +3071,49 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-06 13:46:04.662402+09:00</t>
+          <t>2026-07-08 10:00:27.128578+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-06 13:46:04.662402+09:00</t>
+          <t>2026-07-08 10:00:27.128578+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>3182</t>
+          <t>3251</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1273</t>
+          <t>362</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>개인정보 처리방침 평가, 국민 눈높이에서 더 꼼꼼히 본다</t>
+          <t>2026년 가명정보 활용 지원체계 설명회 개최 안내</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12236</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12238</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3128,49 +3128,49 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-06 13:46:04.662402+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-06 13:46:04.662402+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>3181</t>
+          <t>3182</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>1274</t>
+          <t>1273</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>개인정보위, 교육‧고용 분야까지 개인정보 제3자 전송요구권 확대 추진</t>
+          <t>개인정보 처리방침 평가, 국민 눈높이에서 더 꼼꼼히 본다</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12237</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12236</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3185,7 +3185,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>60</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -3207,32 +3207,32 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1043</t>
+          <t>3181</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>1274</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>개인정보위, 대전에서 ‘찾아가는 개인정보 현장 컨설팅 및 교육’ 개최</t>
+          <t>개인정보위, 교육‧고용 분야까지 개인정보 제3자 전송요구권 확대 추진</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12227</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12237</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3242,7 +3242,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>58</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -3252,39 +3252,39 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-03 16:00:28.543767+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-03 16:00:28.543767+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>1043</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>1272</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.3.자)</t>
+          <t>개인정보위, 대전에서 ‘찾아가는 개인정보 현장 컨설팅 및 교육’ 개최</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12229</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12227</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3299,7 +3299,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -3309,39 +3309,39 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-03 15:30:33.546332+09:00</t>
+          <t>2026-07-03 16:00:28.543767+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-03 15:30:33.546332+09:00</t>
+          <t>2026-07-03 16:00:28.543767+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>561</t>
+          <t>1001</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>1271</t>
+          <t>1272</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>신뢰로 여는 인공지능(AI) 혁신, 달라지는 개인정보 체계로 이끈다</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.3.자)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12228</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12229</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>개인정보보호정책과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3356,7 +3356,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3366,44 +3366,44 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-03 10:00:33.422568+09:00</t>
+          <t>2026-07-03 15:30:33.546332+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-03 10:00:33.422568+09:00</t>
+          <t>2026-07-03 15:30:33.546332+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>561</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>1269</t>
+          <t>1271</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>개인정보위, 인공지능(AI) 시대 데이터 혁신적 활용을 지역 주도로 확산한다.</t>
+          <t>신뢰로 여는 인공지능(AI) 혁신, 달라지는 개인정보 체계로 이끈다</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12225</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12228</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>개인정보보호정책과</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3413,7 +3413,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3423,19 +3423,19 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-02 16:45:30.717611+09:00</t>
+          <t>2026-07-03 10:00:33.422568+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-02 16:45:30.717611+09:00</t>
+          <t>2026-07-03 10:00:33.422568+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>281</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3445,17 +3445,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>개인정보위, 개인정보보호 현장 간담회 개최</t>
+          <t>개인정보위, 인공지능(AI) 시대 데이터 혁신적 활용을 지역 주도로 확산한다.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12224</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12225</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>조사1과</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3480,44 +3480,44 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 16:45:30.717611+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 16:45:30.717611+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>1266</t>
+          <t>1269</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>글로벌 개인정보 감독기구에 인공지능(AI) 대응 ‘실전해법’ 제시</t>
+          <t>개인정보위, 개인정보보호 현장 간담회 개최</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12218</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12224</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>국제협력담당관</t>
+          <t>조사1과</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3527,7 +3527,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>924</t>
+          <t>98</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3549,27 +3549,27 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>1267</t>
+          <t>1266</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>투숙객 개인정보보호에 앞장선 호텔, 호텔업 등급평가시 우대</t>
+          <t>글로벌 개인정보 감독기구에 인공지능(AI) 대응 ‘실전해법’ 제시</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12219</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12218</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>국제협력담당관</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -3584,7 +3584,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1074</t>
+          <t>924</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3606,27 +3606,27 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>1268</t>
+          <t>1267</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.1.자)</t>
+          <t>투숙객 개인정보보호에 앞장선 호텔, 호텔업 등급평가시 우대</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12220</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12219</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -3641,7 +3641,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>743</t>
+          <t>1074</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3663,32 +3663,32 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>361</t>
+          <t>1268</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령(안) 입법예고</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.1.자)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12216</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12220</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>범정부 마이데이터추진단</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3698,49 +3698,49 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>743</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>1265</t>
+          <t>361</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.6.30.자)</t>
+          <t>「개인정보 보호법 시행령」 일부개정령(안) 입법예고</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12217</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12216</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>범정부 마이데이터추진단</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3755,54 +3755,54 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1029</t>
+          <t>1842</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>1265</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.6.30.자)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12202</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12217</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3812,49 +3812,49 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>2800</t>
+          <t>1029</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>1262</t>
+          <t>360</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>개인정보위원장, G7 개인정보 감독기구 라운드테이블 참석</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12201</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12202</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>국제협력담당관</t>
+          <t>신기술개인정보과</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3869,49 +3869,49 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>2144</t>
+          <t>2800</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>1263</t>
+          <t>1262</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>「2026 개인정보 보호·활용 기술 대상」 참여기업 모집</t>
+          <t>개인정보위원장, G7 개인정보 감독기구 라운드테이블 참석</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12203</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12201</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>국제협력담당관</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3926,7 +3926,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>2092</t>
+          <t>2144</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3948,27 +3948,27 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>1264</t>
+          <t>1263</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>AI 범죄 대응 범부처 협의체 출범</t>
+          <t>「2026 개인정보 보호·활용 기술 대상」 참여기업 모집</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12204</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12203</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>인공지능프라이버시팀</t>
+          <t>신기술개인정보과</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>2638</t>
+          <t>2092</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4005,32 +4005,32 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>359</t>
+          <t>1264</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>본인전송요구 대리인의 사전협의 요청 시범기간(6.25.~7.10.) 운영 안내</t>
+          <t>AI 범죄 대응 범부처 협의체 출범</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12200</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12204</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>인공지능프라이버시팀</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4040,49 +4040,49 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>3745</t>
+          <t>2638</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>1260</t>
+          <t>359</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>개인정보위, 상조서비스 개인정보 보호 취약요인 선제 점검</t>
+          <t>본인전송요구 대리인의 사전협의 요청 시범기간(6.25.~7.10.) 운영 안내</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12197</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12200</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>사전실태점검과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -4097,49 +4097,49 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>2754</t>
+          <t>3745</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>1261</t>
+          <t>1260</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>개인정보위, 국민이 필요로 하는 정보 중심 ‘본인전송요구권’ 안착 지원한다</t>
+          <t>개인정보위, 상조서비스 개인정보 보호 취약요인 선제 점검</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12198</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12197</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>사전실태점검과</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -4154,7 +4154,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>3085</t>
+          <t>2754</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4176,32 +4176,32 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>358</t>
+          <t>1261</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>정보보호 및 개인정보보호 관리체계 심사기관 지정 공고(제2026-73호)</t>
+          <t>개인정보위, 국민이 필요로 하는 정보 중심 ‘본인전송요구권’ 안착 지원한다</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12185</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12198</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -4211,54 +4211,54 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>7681</t>
+          <t>3085</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>357</t>
+          <t>358</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>「자율기구 공공실태점검단 설치 및 운영에 관한 규정」 발령(2026-70)</t>
+          <t>정보보호 및 개인정보보호 관리체계 심사기관 지정 공고(제2026-73호)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12174</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12185</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>혁신기획담당관</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -4268,7 +4268,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>6533</t>
+          <t>7681</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -4290,32 +4290,32 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>357</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>공공기관 개인정보 보호수준 평가단원 지원 공고</t>
+          <t>「자율기구 공공실태점검단 설치 및 운영에 관한 규정」 발령(2026-70)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12160</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12174</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>9023</t>
+          <t>6533</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -4347,32 +4347,32 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>352</t>
+          <t>356</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
+          <t>공공기관 개인정보 보호수준 평가단원 지원 공고</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12126</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12160</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>개인정보보호정책과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -4382,7 +4382,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>11169</t>
+          <t>9023</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -4404,12 +4404,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>354</t>
+          <t>352</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -4419,17 +4419,17 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12131</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12126</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>개인정보보호정책과</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -4439,7 +4439,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>13472</t>
+          <t>11169</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -4461,27 +4461,27 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>355</t>
+          <t>354</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12136</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12131</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>9724</t>
+          <t>13472</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -4518,55 +4518,112 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>355</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12136</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>신기술개인정보과</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>9724</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>19</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>353</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>「개인정보 처리 방법에 관한 고시」 일부개정고시안 행정예고</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12127</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>전략기획팀</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
         <is>
           <t>11519</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
+      <c r="I53" t="inlineStr">
         <is>
           <t>공지사항</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="J53" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
+      <c r="K53" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-24 10:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -1605,7 +1605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K53"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1668,32 +1668,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>17362</t>
+          <t>17701</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1286</t>
+          <t>1288</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>「2026 개인정보 미래포럼」 제3차 전체회의 개최</t>
+          <t>유럽연합, 한국 개인정보 보호 수준 재확인… 적정성 결정 유지</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12329</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12333</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>혁신기획담당관</t>
+          <t>국제협력담당관</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1713,39 +1713,39 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-23 16:00:30.422263+09:00</t>
+          <t>2026-07-24 10:00:27.219427+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-23 16:00:30.422263+09:00</t>
+          <t>2026-07-24 10:00:27.219427+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>16883</t>
+          <t>17362</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1285</t>
+          <t>1286</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>국민이 신뢰할 수 있는 공공 인공지능 전환(AX),프라이버시 보호로 적극 뒷받침</t>
+          <t>「2026 개인정보 미래포럼」 제3차 전체회의 개최</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12307</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12329</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>인공지능프라이버시팀</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1770,34 +1770,34 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-23 10:00:38.625145+09:00</t>
+          <t>2026-07-23 16:00:30.422263+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-23 10:00:38.625145+09:00</t>
+          <t>2026-07-23 16:00:30.422263+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>16882</t>
+          <t>16883</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1286</t>
+          <t>1285</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>대도약의 골든타임, 초격차 성장동력 확보와 AI 생태계 발전기반 강화</t>
+          <t>국민이 신뢰할 수 있는 공공 인공지능 전환(AX),프라이버시 보호로 적극 뒷받침</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12308</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12307</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1839,27 +1839,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>16881</t>
+          <t>16882</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1287</t>
+          <t>1286</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>개인정보위, 적법 근거 없이 개인정보수집·이용한 틱톡·애플 제재</t>
+          <t>대도약의 골든타임, 초격차 성장동력 확보와 AI 생태계 발전기반 강화</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12330</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12308</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>조사1과</t>
+          <t>인공지능프라이버시팀</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1896,32 +1896,32 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>16314</t>
+          <t>16881</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>370</t>
+          <t>1287</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>「개인정보 보호위원회의 조사 및 처분에 관한 규정」 일부개정안 행정예고</t>
+          <t>개인정보위, 적법 근거 없이 개인정보수집·이용한 틱톡·애플 제재</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12309</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12330</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>조사1과</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1931,44 +1931,44 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-22 13:01:11.478354+09:00</t>
+          <t>2026-07-23 10:00:38.625145+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-22 13:01:11.478354+09:00</t>
+          <t>2026-07-23 10:00:38.625145+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>16313</t>
+          <t>16314</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>371</t>
+          <t>370</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>「개인정보 보호 법규 위반에 대한 고발 기준」 제정안 행정예고</t>
+          <t>「개인정보 보호위원회의 조사 및 처분에 관한 규정」 일부개정안 행정예고</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12310</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12309</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1988,7 +1988,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -2010,22 +2010,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>16312</t>
+          <t>16313</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>372</t>
+          <t>371</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>「개인정보 보호 법규 위반에 대한 징계권고 기준」 제정안 행정예고</t>
+          <t>「개인정보 보호 법규 위반에 대한 고발 기준」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12311</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12310</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -2067,22 +2067,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>16311</t>
+          <t>16312</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>373</t>
+          <t>372</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 위반에 대한 공표 및 공표명령 지침」 제정안 행정예고</t>
+          <t>「개인정보 보호 법규 위반에 대한 징계권고 기준」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12312</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12311</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -2124,32 +2124,32 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>14451</t>
+          <t>16311</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>369</t>
+          <t>373</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>본인전송요구 대리인의 사전협의 요청 시범기간 추가운영(7.20.~31.) 안내</t>
+          <t>「개인정보 보호법 위반에 대한 공표 및 공표명령 지침」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12289</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12312</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -2169,39 +2169,39 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-20 10:16:06.541093+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-20 10:16:06.541093+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>14433</t>
+          <t>14451</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>366</t>
+          <t>369</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>본인전송요구 대리인의 사전협의 요청 시범기간 추가운영(7.20.~31.) 안내</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12278</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12289</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -2226,34 +2226,34 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:08.116520+09:00</t>
+          <t>2026-07-20 10:16:06.541093+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:08.116520+09:00</t>
+          <t>2026-07-20 10:16:06.541093+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>14422</t>
+          <t>14433</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1282</t>
+          <t>366</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>「개인정보 이노베이션 존」 신규 운영기관 공모</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12287</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12278</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -2273,49 +2273,49 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-20 10:00:27.102836+09:00</t>
+          <t>2026-07-20 10:01:08.116520+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-20 10:00:27.102836+09:00</t>
+          <t>2026-07-20 10:01:08.116520+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14422</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1283</t>
+          <t>1282</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>개인정보위, ‘본인전송요구권’ 사전협의 지원 시범운영 7월 31일까지 추가신청 받는다</t>
+          <t>「개인정보 이노베이션 존」 신규 운영기관 공모</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12288</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12287</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -2330,7 +2330,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -2352,32 +2352,32 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>11392</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>367</t>
+          <t>1283</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 위반에 대한 과징금 부과기준」 일부개정안 행정예고</t>
+          <t>개인정보위, ‘본인전송요구권’ 사전협의 지원 시범운영 7월 31일까지 추가신청 받는다</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12282</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12288</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2387,44 +2387,44 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-16 13:01:06.075969+09:00</t>
+          <t>2026-07-20 10:00:27.102836+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-16 13:01:06.075969+09:00</t>
+          <t>2026-07-20 10:00:27.102836+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>11391</t>
+          <t>11392</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>368</t>
+          <t>367</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 위반에 대한 과태료 부과기준」 제정안 행정예고</t>
+          <t>「개인정보 보호법 위반에 대한 과징금 부과기준」 일부개정안 행정예고</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12284</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12282</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2466,27 +2466,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>11221</t>
+          <t>11391</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1281</t>
+          <t>368</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AI 혁신을 뒷받침하고 국민 권익을 증진하는 예방중심 개인정보 보호 실현</t>
+          <t>「개인정보 보호법 위반에 대한 과태료 부과기준」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12281</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12284</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>혁신기획담당관</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2501,54 +2501,54 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-16 11:00:27.819143+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-16 11:00:27.819143+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>10301</t>
+          <t>11221</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1280</t>
+          <t>1281</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.15.자)</t>
+          <t>AI 혁신을 뒷받침하고 국민 권익을 증진하는 예방중심 개인정보 보호 실현</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12276</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12281</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2568,44 +2568,44 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-15 09:45:30.272302+09:00</t>
+          <t>2026-07-16 11:00:27.819143+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-15 09:45:30.272302+09:00</t>
+          <t>2026-07-16 11:00:27.819143+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>9501</t>
+          <t>10301</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1279</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>개인정보 전송요구권 전송체계 기술적 기틀, 고용⋅교육 부문까지 확대 마련</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.15.자)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12266</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12276</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>인프라표준화팀</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2625,44 +2625,44 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-14 10:00:29.933870+09:00</t>
+          <t>2026-07-15 09:45:30.272302+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-14 10:00:29.933870+09:00</t>
+          <t>2026-07-15 09:45:30.272302+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>9381</t>
+          <t>9501</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1280</t>
+          <t>1279</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>정보주체의 본인전송요구권, 더 안전하게 이용할 수 있습니다</t>
+          <t>개인정보 전송요구권 전송체계 기술적 기틀, 고용⋅교육 부문까지 확대 마련</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12273</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12266</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>범정부마이데이터추진단 전략기획팀</t>
+          <t>인프라표준화팀</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2682,39 +2682,39 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-14 08:30:26.475160+09:00</t>
+          <t>2026-07-14 10:00:29.933870+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-14 08:30:26.475160+09:00</t>
+          <t>2026-07-14 10:00:29.933870+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>9271</t>
+          <t>9381</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>365</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>공공기관 종합청렴도 평가 관련 개인정보 제3자 제공사항 알림</t>
+          <t>정보주체의 본인전송요구권, 더 안전하게 이용할 수 있습니다</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12267</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12273</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>법무감사담당관</t>
+          <t>범정부마이데이터추진단 전략기획팀</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2724,116 +2724,116 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>303</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-13 17:16:17.898453+09:00</t>
+          <t>2026-07-14 08:30:26.475160+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-13 17:16:17.898453+09:00</t>
+          <t>2026-07-14 08:30:26.475160+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>6541</t>
+          <t>9271</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1278</t>
+          <t>365</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>개인정보 온라인 불법유통 청년들이 직접 차단한다.</t>
+          <t>공공기관 종합청렴도 평가 관련 개인정보 제3자 제공사항 알림</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12262</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12267</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>조사2과</t>
+          <t>법무감사담당관</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-10 14:00:31.832545+09:00</t>
+          <t>2026-07-13 17:16:17.898453+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-10 14:00:31.832545+09:00</t>
+          <t>2026-07-13 17:16:17.898453+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>5491</t>
+          <t>6541</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>364</t>
+          <t>1278</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>제4회 개인정보보호 모의재판 경연대회 참가자 모집</t>
+          <t>개인정보 온라인 불법유통 청년들이 직접 차단한다.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12245</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12262</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>침해평가과</t>
+          <t>조사2과</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2843,49 +2843,49 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-09 11:01:05.002078+09:00</t>
+          <t>2026-07-10 14:00:31.832545+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-09 11:01:05.002078+09:00</t>
+          <t>2026-07-10 14:00:31.832545+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>5402</t>
+          <t>5491</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1276</t>
+          <t>364</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>개인정보위, 안전조치 의무 위반 3개 사업자 제재</t>
+          <t>제4회 개인정보보호 모의재판 경연대회 참가자 모집</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12242</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12245</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>장석인</t>
+          <t>침해평가과</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2900,49 +2900,49 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-09 11:01:05.002078+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-09 11:01:05.002078+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>5401</t>
+          <t>5402</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>1277</t>
+          <t>1276</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>미래의 개인정보 법률 전문가 모여 인공지능 시대 법적 쟁점 논의한다</t>
+          <t>개인정보위, 안전조치 의무 위반 3개 사업자 제재</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12243</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12242</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>침해평가과</t>
+          <t>장석인</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2957,7 +2957,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2979,27 +2979,27 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>5391</t>
+          <t>5401</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>363</t>
+          <t>1277</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>「개인정보 보호책임자 경력 인정에 관한 고시」 일부개정고시안 행정예고</t>
+          <t>미래의 개인정보 법률 전문가 모여 인공지능 시대 법적 쟁점 논의한다</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12244</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12243</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>침해평가과</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3014,54 +3014,54 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-09 09:46:03.809898+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-09 09:46:03.809898+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>4581</t>
+          <t>5391</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>1275</t>
+          <t>363</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>개인정보위, 응용프로그램 인터페이스(API) 활용 확대에 따른 개인정보 유출 예방 당부</t>
+          <t>「개인정보 보호책임자 경력 인정에 관한 고시」 일부개정고시안 행정예고</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12241</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12244</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>사전실태점검과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3071,54 +3071,54 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-08 10:00:27.128578+09:00</t>
+          <t>2026-07-09 09:46:03.809898+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-08 10:00:27.128578+09:00</t>
+          <t>2026-07-09 09:46:03.809898+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>3251</t>
+          <t>4581</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>1275</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026년 가명정보 활용 지원체계 설명회 개최 안내</t>
+          <t>개인정보위, 응용프로그램 인터페이스(API) 활용 확대에 따른 개인정보 유출 예방 당부</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12238</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12241</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>사전실태점검과</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3128,49 +3128,49 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-06 13:46:04.662402+09:00</t>
+          <t>2026-07-08 10:00:27.128578+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-06 13:46:04.662402+09:00</t>
+          <t>2026-07-08 10:00:27.128578+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>3182</t>
+          <t>3251</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>1273</t>
+          <t>362</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>개인정보 처리방침 평가, 국민 눈높이에서 더 꼼꼼히 본다</t>
+          <t>2026년 가명정보 활용 지원체계 설명회 개최 안내</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12236</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12238</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3185,49 +3185,49 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-06 13:46:04.662402+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-06 13:46:04.662402+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>3181</t>
+          <t>3182</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>1274</t>
+          <t>1273</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>개인정보위, 교육‧고용 분야까지 개인정보 제3자 전송요구권 확대 추진</t>
+          <t>개인정보 처리방침 평가, 국민 눈높이에서 더 꼼꼼히 본다</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12237</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12236</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3242,7 +3242,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>60</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -3264,32 +3264,32 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1043</t>
+          <t>3181</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>1274</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>개인정보위, 대전에서 ‘찾아가는 개인정보 현장 컨설팅 및 교육’ 개최</t>
+          <t>개인정보위, 교육‧고용 분야까지 개인정보 제3자 전송요구권 확대 추진</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12227</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12237</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3299,7 +3299,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>58</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -3309,39 +3309,39 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-03 16:00:28.543767+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-03 16:00:28.543767+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>1043</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>1272</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.3.자)</t>
+          <t>개인정보위, 대전에서 ‘찾아가는 개인정보 현장 컨설팅 및 교육’ 개최</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12229</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12227</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3356,7 +3356,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3366,39 +3366,39 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-03 15:30:33.546332+09:00</t>
+          <t>2026-07-03 16:00:28.543767+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-03 15:30:33.546332+09:00</t>
+          <t>2026-07-03 16:00:28.543767+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>561</t>
+          <t>1001</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>1271</t>
+          <t>1272</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>신뢰로 여는 인공지능(AI) 혁신, 달라지는 개인정보 체계로 이끈다</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.3.자)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12228</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12229</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>개인정보보호정책과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3413,7 +3413,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3423,44 +3423,44 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-03 10:00:33.422568+09:00</t>
+          <t>2026-07-03 15:30:33.546332+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-03 10:00:33.422568+09:00</t>
+          <t>2026-07-03 15:30:33.546332+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>561</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>1269</t>
+          <t>1271</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>개인정보위, 인공지능(AI) 시대 데이터 혁신적 활용을 지역 주도로 확산한다.</t>
+          <t>신뢰로 여는 인공지능(AI) 혁신, 달라지는 개인정보 체계로 이끈다</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12225</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12228</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>개인정보보호정책과</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3480,19 +3480,19 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-02 16:45:30.717611+09:00</t>
+          <t>2026-07-03 10:00:33.422568+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-02 16:45:30.717611+09:00</t>
+          <t>2026-07-03 10:00:33.422568+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>281</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3502,17 +3502,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>개인정보위, 개인정보보호 현장 간담회 개최</t>
+          <t>개인정보위, 인공지능(AI) 시대 데이터 혁신적 활용을 지역 주도로 확산한다.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12224</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12225</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>조사1과</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -3527,7 +3527,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3537,44 +3537,44 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 16:45:30.717611+09:00</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 16:45:30.717611+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>1266</t>
+          <t>1269</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>글로벌 개인정보 감독기구에 인공지능(AI) 대응 ‘실전해법’ 제시</t>
+          <t>개인정보위, 개인정보보호 현장 간담회 개최</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12218</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12224</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>국제협력담당관</t>
+          <t>조사1과</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3584,7 +3584,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>924</t>
+          <t>98</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3606,27 +3606,27 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>1267</t>
+          <t>1266</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>투숙객 개인정보보호에 앞장선 호텔, 호텔업 등급평가시 우대</t>
+          <t>글로벌 개인정보 감독기구에 인공지능(AI) 대응 ‘실전해법’ 제시</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12219</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12218</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>국제협력담당관</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -3641,7 +3641,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1074</t>
+          <t>924</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3663,27 +3663,27 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>1268</t>
+          <t>1267</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.1.자)</t>
+          <t>투숙객 개인정보보호에 앞장선 호텔, 호텔업 등급평가시 우대</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12220</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12219</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -3698,7 +3698,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>743</t>
+          <t>1074</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3720,32 +3720,32 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>361</t>
+          <t>1268</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령(안) 입법예고</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.1.자)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12216</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12220</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>범정부 마이데이터추진단</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3755,49 +3755,49 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>743</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>1265</t>
+          <t>361</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.6.30.자)</t>
+          <t>「개인정보 보호법 시행령」 일부개정령(안) 입법예고</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12217</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12216</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>범정부 마이데이터추진단</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3812,54 +3812,54 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1029</t>
+          <t>1842</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>1265</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.6.30.자)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12202</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12217</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3869,49 +3869,49 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>2800</t>
+          <t>1029</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>1262</t>
+          <t>360</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>개인정보위원장, G7 개인정보 감독기구 라운드테이블 참석</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12201</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12202</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>국제협력담당관</t>
+          <t>신기술개인정보과</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3926,49 +3926,49 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>2144</t>
+          <t>2800</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>1263</t>
+          <t>1262</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>「2026 개인정보 보호·활용 기술 대상」 참여기업 모집</t>
+          <t>개인정보위원장, G7 개인정보 감독기구 라운드테이블 참석</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12203</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12201</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>국제협력담당관</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>2092</t>
+          <t>2144</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4005,27 +4005,27 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>1264</t>
+          <t>1263</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>AI 범죄 대응 범부처 협의체 출범</t>
+          <t>「2026 개인정보 보호·활용 기술 대상」 참여기업 모집</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12204</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12203</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>인공지능프라이버시팀</t>
+          <t>신기술개인정보과</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -4040,7 +4040,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>2638</t>
+          <t>2092</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4062,32 +4062,32 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>359</t>
+          <t>1264</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>본인전송요구 대리인의 사전협의 요청 시범기간(6.25.~7.10.) 운영 안내</t>
+          <t>AI 범죄 대응 범부처 협의체 출범</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12200</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12204</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>인공지능프라이버시팀</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -4097,49 +4097,49 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>3745</t>
+          <t>2638</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>1260</t>
+          <t>359</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>개인정보위, 상조서비스 개인정보 보호 취약요인 선제 점검</t>
+          <t>본인전송요구 대리인의 사전협의 요청 시범기간(6.25.~7.10.) 운영 안내</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12197</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12200</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>사전실태점검과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -4154,49 +4154,49 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>2754</t>
+          <t>3745</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>1261</t>
+          <t>1260</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>개인정보위, 국민이 필요로 하는 정보 중심 ‘본인전송요구권’ 안착 지원한다</t>
+          <t>개인정보위, 상조서비스 개인정보 보호 취약요인 선제 점검</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12198</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12197</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>사전실태점검과</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -4211,7 +4211,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>3085</t>
+          <t>2754</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4233,32 +4233,32 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>358</t>
+          <t>1261</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>정보보호 및 개인정보보호 관리체계 심사기관 지정 공고(제2026-73호)</t>
+          <t>개인정보위, 국민이 필요로 하는 정보 중심 ‘본인전송요구권’ 안착 지원한다</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12185</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12198</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -4268,54 +4268,54 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>7681</t>
+          <t>3085</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>357</t>
+          <t>358</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>「자율기구 공공실태점검단 설치 및 운영에 관한 규정」 발령(2026-70)</t>
+          <t>정보보호 및 개인정보보호 관리체계 심사기관 지정 공고(제2026-73호)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12174</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12185</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>혁신기획담당관</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>6533</t>
+          <t>7681</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -4347,32 +4347,32 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>357</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>공공기관 개인정보 보호수준 평가단원 지원 공고</t>
+          <t>「자율기구 공공실태점검단 설치 및 운영에 관한 규정」 발령(2026-70)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12160</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12174</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -4382,7 +4382,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>9023</t>
+          <t>6533</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -4404,32 +4404,32 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>352</t>
+          <t>356</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
+          <t>공공기관 개인정보 보호수준 평가단원 지원 공고</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12126</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12160</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>개인정보보호정책과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -4439,7 +4439,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>11169</t>
+          <t>9023</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -4461,12 +4461,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>354</t>
+          <t>352</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -4476,17 +4476,17 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12131</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12126</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>개인정보보호정책과</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>13472</t>
+          <t>11169</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -4518,27 +4518,27 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>355</t>
+          <t>354</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12136</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12131</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -4553,7 +4553,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>9724</t>
+          <t>13472</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -4575,55 +4575,112 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>355</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12136</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>신기술개인정보과</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>9724</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>19</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>353</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>「개인정보 처리 방법에 관한 고시」 일부개정고시안 행정예고</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12127</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>전략기획팀</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
         <is>
           <t>11519</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
+      <c r="I54" t="inlineStr">
         <is>
           <t>공지사항</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="J54" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr">
+      <c r="K54" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-27 09:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -5887,7 +5887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K50"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5950,40 +5950,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>16785</t>
+          <t>20061</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1496</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
+          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>246</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -5991,34 +5995,34 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>16784</t>
+          <t>16785</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1497</t>
+          <t>1496</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -6028,7 +6032,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -6056,22 +6060,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>16781</t>
+          <t>16784</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1497</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -6081,7 +6085,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>260</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -6089,11 +6093,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6113,22 +6113,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>16691</t>
+          <t>16781</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -6138,35 +6138,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>242</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>16464</t>
+          <t>16691</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6176,12 +6180,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
+          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -6191,35 +6195,35 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>278</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>16051</t>
+          <t>16464</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6229,12 +6233,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
+          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -6244,35 +6248,35 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6282,22 +6286,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -6313,19 +6317,19 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6335,12 +6339,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -6350,7 +6354,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -6366,34 +6370,34 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -6403,7 +6407,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -6411,56 +6415,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -6468,7 +6468,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6476,34 +6480,34 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -6513,7 +6517,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -6524,96 +6528,92 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -6631,7 +6631,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6639,19 +6643,19 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -6661,12 +6665,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -6676,12 +6680,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -6692,19 +6696,19 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -6714,22 +6718,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -6745,19 +6749,19 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -6767,12 +6771,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -6782,7 +6786,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -6793,96 +6797,92 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -6892,35 +6892,39 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -6930,22 +6934,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -6956,24 +6960,24 @@
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -6983,12 +6987,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -6998,7 +7002,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -7009,24 +7013,24 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -7036,22 +7040,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -7067,44 +7071,44 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -7120,44 +7124,44 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -7165,31 +7169,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -7199,12 +7199,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -7246,22 +7246,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -7271,7 +7271,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -7279,27 +7279,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -7309,12 +7313,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -7324,113 +7328,113 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -7438,31 +7442,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7472,12 +7472,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -7487,7 +7487,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -7519,32 +7519,32 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -7552,7 +7552,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7572,22 +7576,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -7597,7 +7601,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -7625,22 +7629,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -7650,19 +7654,15 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7682,7 +7682,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -7692,12 +7692,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -7707,7 +7707,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -7739,40 +7739,44 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7792,22 +7796,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -7817,7 +7821,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -7825,11 +7829,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7849,32 +7849,32 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -7882,7 +7882,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7890,34 +7894,34 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -7927,7 +7931,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -7938,49 +7942,49 @@
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -8008,22 +8012,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -8033,7 +8037,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -8061,32 +8065,32 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -8114,22 +8118,22 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -8139,39 +8143,35 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -8181,27 +8181,27 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -8228,32 +8228,32 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -8261,52 +8261,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -8334,32 +8338,32 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -8387,32 +8391,32 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -8440,32 +8444,32 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -8473,46 +8477,42 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14403</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -8522,7 +8522,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>6587</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -8530,52 +8530,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -8595,6 +8599,59 @@
         </is>
       </c>
       <c r="K50" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-27 10:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -5887,7 +5887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K51"/>
+  <dimension ref="A1:K52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5950,22 +5950,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>20061</t>
+          <t>20191</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
+          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -5975,7 +5975,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>287</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -5983,64 +5983,64 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>16785</t>
+          <t>20061</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1496</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
+          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>246</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6048,34 +6048,34 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>16784</t>
+          <t>16785</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1497</t>
+          <t>1496</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -6085,7 +6085,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -6113,22 +6113,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>16781</t>
+          <t>16784</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1497</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -6138,7 +6138,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>260</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -6146,11 +6146,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6170,22 +6166,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>16691</t>
+          <t>16781</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -6195,35 +6191,39 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>242</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>16464</t>
+          <t>16691</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6233,12 +6233,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
+          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -6248,35 +6248,35 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>278</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>16051</t>
+          <t>16464</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6286,12 +6286,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
+          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -6301,35 +6301,35 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6339,22 +6339,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -6370,19 +6370,19 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6392,12 +6392,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -6407,7 +6407,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -6423,34 +6423,34 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -6460,7 +6460,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -6468,56 +6468,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -6525,7 +6521,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6533,34 +6533,34 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -6570,7 +6570,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -6581,96 +6581,92 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -6680,7 +6676,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -6688,7 +6684,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6696,19 +6696,19 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -6718,12 +6718,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -6733,12 +6733,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -6749,19 +6749,19 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -6771,22 +6771,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -6802,19 +6802,19 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -6824,12 +6824,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -6839,7 +6839,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -6850,96 +6850,92 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -6949,35 +6945,39 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -6987,22 +6987,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -7013,24 +7013,24 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -7040,12 +7040,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -7055,7 +7055,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -7066,24 +7066,24 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -7093,22 +7093,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -7124,44 +7124,44 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -7177,44 +7177,44 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -7222,31 +7222,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -7256,12 +7252,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -7271,7 +7267,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -7303,22 +7299,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -7328,7 +7324,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -7336,27 +7332,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -7366,12 +7366,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -7381,113 +7381,113 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -7495,31 +7495,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7529,12 +7525,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -7544,7 +7540,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -7576,32 +7572,32 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -7609,7 +7605,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7629,22 +7629,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -7654,7 +7654,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -7682,22 +7682,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -7707,19 +7707,15 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7739,7 +7735,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -7749,12 +7745,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -7764,7 +7760,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -7796,40 +7792,44 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7849,22 +7849,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -7874,7 +7874,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -7882,11 +7882,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7906,32 +7902,32 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -7939,7 +7935,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7947,34 +7947,34 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -7984,7 +7984,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -7995,49 +7995,49 @@
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -8065,22 +8065,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -8090,7 +8090,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -8118,32 +8118,32 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -8171,22 +8171,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -8196,39 +8196,35 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -8238,27 +8234,27 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -8285,32 +8281,32 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -8318,52 +8314,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -8391,32 +8391,32 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -8444,32 +8444,32 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -8497,32 +8497,32 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -8530,46 +8530,42 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14403</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -8579,7 +8575,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>6587</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -8587,52 +8583,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -8652,6 +8652,59 @@
         </is>
       </c>
       <c r="K51" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-27 17:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -5887,7 +5887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K52"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5950,7 +5950,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>20191</t>
+          <t>20771</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5960,12 +5960,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
+          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -5975,7 +5975,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -5991,34 +5991,34 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>20061</t>
+          <t>20191</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
+          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -6028,7 +6028,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>287</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -6036,64 +6036,64 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>16785</t>
+          <t>20061</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1496</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
+          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>246</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6101,34 +6101,34 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>16784</t>
+          <t>16785</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1497</t>
+          <t>1496</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -6138,7 +6138,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -6166,22 +6166,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>16781</t>
+          <t>16784</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1497</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -6191,7 +6191,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>260</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -6199,11 +6199,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6223,22 +6219,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>16691</t>
+          <t>16781</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -6248,35 +6244,39 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>242</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>16464</t>
+          <t>16691</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6286,12 +6286,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
+          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -6301,35 +6301,35 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>278</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>16051</t>
+          <t>16464</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6339,12 +6339,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
+          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -6354,35 +6354,35 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6392,22 +6392,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -6423,19 +6423,19 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -6445,12 +6445,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -6460,7 +6460,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -6476,34 +6476,34 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -6513,7 +6513,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -6521,56 +6521,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -6578,7 +6574,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6586,34 +6586,34 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -6634,96 +6634,92 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -6733,7 +6729,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -6741,7 +6737,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6749,19 +6749,19 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -6771,12 +6771,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -6786,12 +6786,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -6802,19 +6802,19 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -6824,22 +6824,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -6855,19 +6855,19 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -6877,12 +6877,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -6892,7 +6892,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -6903,96 +6903,92 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -7002,35 +6998,39 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -7040,22 +7040,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -7066,24 +7066,24 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -7093,12 +7093,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -7119,24 +7119,24 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -7146,22 +7146,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -7177,44 +7177,44 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -7230,44 +7230,44 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -7275,31 +7275,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -7309,12 +7305,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -7324,7 +7320,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -7356,22 +7352,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -7381,7 +7377,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -7389,27 +7385,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -7419,12 +7419,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -7434,113 +7434,113 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -7548,31 +7548,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -7582,12 +7578,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -7597,7 +7593,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -7629,32 +7625,32 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -7662,7 +7658,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7682,22 +7682,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -7707,7 +7707,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -7735,22 +7735,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -7760,19 +7760,15 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7792,7 +7788,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7802,12 +7798,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -7817,7 +7813,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -7849,40 +7845,44 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7902,22 +7902,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -7927,7 +7927,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -7935,11 +7935,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7959,32 +7955,32 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -7992,7 +7988,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8000,34 +8000,34 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -8037,7 +8037,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -8048,49 +8048,49 @@
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -8118,22 +8118,22 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -8143,7 +8143,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -8171,32 +8171,32 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -8224,22 +8224,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -8249,39 +8249,35 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -8291,27 +8287,27 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -8338,32 +8334,32 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -8371,52 +8367,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -8444,32 +8444,32 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -8497,32 +8497,32 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -8550,32 +8550,32 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -8583,46 +8583,42 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14403</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -8632,7 +8628,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>6587</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -8640,52 +8636,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -8705,6 +8705,59 @@
         </is>
       </c>
       <c r="K52" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-29 17:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -1605,7 +1605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K54"/>
+  <dimension ref="A1:K56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1668,32 +1668,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>17701</t>
+          <t>22391</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1288</t>
+          <t>374</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>유럽연합, 한국 개인정보 보호 수준 재확인… 적정성 결정 유지</t>
+          <t>개인정보 영향평가기관 지정갱신 공고</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12333</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12346</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>국제협력담당관</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1703,54 +1703,54 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-24 10:00:27.219427+09:00</t>
+          <t>2026-07-29 17:16:05.593491+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-24 10:00:27.219427+09:00</t>
+          <t>2026-07-29 17:16:05.593491+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>17362</t>
+          <t>22351</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1286</t>
+          <t>374</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>「2026 개인정보 미래포럼」 제3차 전체회의 개최</t>
+          <t>개인정보 영향평가기관 지정갱신 공고</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12329</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12345</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>혁신기획담당관</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1760,54 +1760,54 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-23 16:00:30.422263+09:00</t>
+          <t>2026-07-29 16:46:07.286593+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-23 16:00:30.422263+09:00</t>
+          <t>2026-07-29 16:46:07.286593+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>16883</t>
+          <t>17701</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1285</t>
+          <t>1288</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>국민이 신뢰할 수 있는 공공 인공지능 전환(AX),프라이버시 보호로 적극 뒷받침</t>
+          <t>유럽연합, 한국 개인정보 보호 수준 재확인… 적정성 결정 유지</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12307</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12333</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>인공지능프라이버시팀</t>
+          <t>국제협력담당관</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1827,19 +1827,19 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-23 10:00:38.625145+09:00</t>
+          <t>2026-07-24 10:00:27.219427+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-23 10:00:38.625145+09:00</t>
+          <t>2026-07-24 10:00:27.219427+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>16882</t>
+          <t>17362</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1849,17 +1849,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>대도약의 골든타임, 초격차 성장동력 확보와 AI 생태계 발전기반 강화</t>
+          <t>「2026 개인정보 미래포럼」 제3차 전체회의 개최</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12308</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12329</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>인공지능프라이버시팀</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1884,39 +1884,39 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-23 10:00:38.625145+09:00</t>
+          <t>2026-07-23 16:00:30.422263+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-23 10:00:38.625145+09:00</t>
+          <t>2026-07-23 16:00:30.422263+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>16881</t>
+          <t>16883</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1287</t>
+          <t>1285</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>개인정보위, 적법 근거 없이 개인정보수집·이용한 틱톡·애플 제재</t>
+          <t>국민이 신뢰할 수 있는 공공 인공지능 전환(AX),프라이버시 보호로 적극 뒷받침</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12330</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12307</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>조사1과</t>
+          <t>인공지능프라이버시팀</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1931,7 +1931,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1953,32 +1953,32 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>16314</t>
+          <t>16882</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>370</t>
+          <t>1286</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>「개인정보 보호위원회의 조사 및 처분에 관한 규정」 일부개정안 행정예고</t>
+          <t>대도약의 골든타임, 초격차 성장동력 확보와 AI 생태계 발전기반 강화</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12309</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12308</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>인공지능프라이버시팀</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1988,54 +1988,54 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-22 13:01:11.478354+09:00</t>
+          <t>2026-07-23 10:00:38.625145+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-22 13:01:11.478354+09:00</t>
+          <t>2026-07-23 10:00:38.625145+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>16313</t>
+          <t>16881</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>371</t>
+          <t>1287</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>「개인정보 보호 법규 위반에 대한 고발 기준」 제정안 행정예고</t>
+          <t>개인정보위, 적법 근거 없이 개인정보수집·이용한 틱톡·애플 제재</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12310</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12330</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>조사1과</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -2045,44 +2045,44 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-22 13:01:11.478354+09:00</t>
+          <t>2026-07-23 10:00:38.625145+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-22 13:01:11.478354+09:00</t>
+          <t>2026-07-23 10:00:38.625145+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>16312</t>
+          <t>16314</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>372</t>
+          <t>370</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>「개인정보 보호 법규 위반에 대한 징계권고 기준」 제정안 행정예고</t>
+          <t>「개인정보 보호위원회의 조사 및 처분에 관한 규정」 일부개정안 행정예고</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12311</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12309</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -2124,22 +2124,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>16311</t>
+          <t>16313</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>373</t>
+          <t>371</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 위반에 대한 공표 및 공표명령 지침」 제정안 행정예고</t>
+          <t>「개인정보 보호 법규 위반에 대한 고발 기준」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12312</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12310</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -2181,32 +2181,32 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>14451</t>
+          <t>16312</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>369</t>
+          <t>372</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>본인전송요구 대리인의 사전협의 요청 시범기간 추가운영(7.20.~31.) 안내</t>
+          <t>「개인정보 보호 법규 위반에 대한 징계권고 기준」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12289</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12311</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -2226,44 +2226,44 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-20 10:16:06.541093+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-20 10:16:06.541093+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>14433</t>
+          <t>16311</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>366</t>
+          <t>373</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>「개인정보 보호법 위반에 대한 공표 및 공표명령 지침」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12278</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12312</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -2283,39 +2283,39 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:08.116520+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:08.116520+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>14422</t>
+          <t>14451</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1282</t>
+          <t>369</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>「개인정보 이노베이션 존」 신규 운영기관 공모</t>
+          <t>본인전송요구 대리인의 사전협의 요청 시범기간 추가운영(7.20.~31.) 안내</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12287</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12289</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -2330,49 +2330,49 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-20 10:00:27.102836+09:00</t>
+          <t>2026-07-20 10:16:06.541093+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-20 10:00:27.102836+09:00</t>
+          <t>2026-07-20 10:16:06.541093+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14433</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1283</t>
+          <t>366</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>개인정보위, ‘본인전송요구권’ 사전협의 지원 시범운영 7월 31일까지 추가신청 받는다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12288</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12278</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -2387,54 +2387,54 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-20 10:00:27.102836+09:00</t>
+          <t>2026-07-20 10:01:08.116520+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-20 10:00:27.102836+09:00</t>
+          <t>2026-07-20 10:01:08.116520+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>11392</t>
+          <t>14422</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>367</t>
+          <t>1282</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 위반에 대한 과징금 부과기준」 일부개정안 행정예고</t>
+          <t>「개인정보 이노베이션 존」 신규 운영기관 공모</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12282</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12287</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2444,54 +2444,54 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-16 13:01:06.075969+09:00</t>
+          <t>2026-07-20 10:00:27.102836+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-16 13:01:06.075969+09:00</t>
+          <t>2026-07-20 10:00:27.102836+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>11391</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>368</t>
+          <t>1283</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 위반에 대한 과태료 부과기준」 제정안 행정예고</t>
+          <t>개인정보위, ‘본인전송요구권’ 사전협의 지원 시범운영 7월 31일까지 추가신청 받는다</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12284</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12288</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2501,49 +2501,49 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-16 13:01:06.075969+09:00</t>
+          <t>2026-07-20 10:00:27.102836+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-16 13:01:06.075969+09:00</t>
+          <t>2026-07-20 10:00:27.102836+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>11221</t>
+          <t>11392</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1281</t>
+          <t>367</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AI 혁신을 뒷받침하고 국민 권익을 증진하는 예방중심 개인정보 보호 실현</t>
+          <t>「개인정보 보호법 위반에 대한 과징금 부과기준」 일부개정안 행정예고</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12281</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12282</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>혁신기획담당관</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2558,54 +2558,54 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-16 11:00:27.819143+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-16 11:00:27.819143+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>10301</t>
+          <t>11391</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1280</t>
+          <t>368</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.15.자)</t>
+          <t>「개인정보 보호법 위반에 대한 과태료 부과기준」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12276</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12284</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2615,54 +2615,54 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-15 09:45:30.272302+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-15 09:45:30.272302+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>9501</t>
+          <t>11221</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1279</t>
+          <t>1281</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>개인정보 전송요구권 전송체계 기술적 기틀, 고용⋅교육 부문까지 확대 마련</t>
+          <t>AI 혁신을 뒷받침하고 국민 권익을 증진하는 예방중심 개인정보 보호 실현</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12266</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12281</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>인프라표준화팀</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2682,19 +2682,19 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-14 10:00:29.933870+09:00</t>
+          <t>2026-07-16 11:00:27.819143+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-14 10:00:29.933870+09:00</t>
+          <t>2026-07-16 11:00:27.819143+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>9381</t>
+          <t>10301</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2704,22 +2704,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>정보주체의 본인전송요구권, 더 안전하게 이용할 수 있습니다</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.15.자)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12273</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12276</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>범정부마이데이터추진단 전략기획팀</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2729,7 +2729,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2739,101 +2739,101 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-14 08:30:26.475160+09:00</t>
+          <t>2026-07-15 09:45:30.272302+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-14 08:30:26.475160+09:00</t>
+          <t>2026-07-15 09:45:30.272302+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>9271</t>
+          <t>9501</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>365</t>
+          <t>1279</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>공공기관 종합청렴도 평가 관련 개인정보 제3자 제공사항 알림</t>
+          <t>개인정보 전송요구권 전송체계 기술적 기틀, 고용⋅교육 부문까지 확대 마련</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12267</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12266</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>법무감사담당관</t>
+          <t>인프라표준화팀</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-13 17:16:17.898453+09:00</t>
+          <t>2026-07-14 10:00:29.933870+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-13 17:16:17.898453+09:00</t>
+          <t>2026-07-14 10:00:29.933870+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>6541</t>
+          <t>9381</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1278</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>개인정보 온라인 불법유통 청년들이 직접 차단한다.</t>
+          <t>정보주체의 본인전송요구권, 더 안전하게 이용할 수 있습니다</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12262</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12273</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>조사2과</t>
+          <t>범정부마이데이터추진단 전략기획팀</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>303</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2853,54 +2853,54 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-10 14:00:31.832545+09:00</t>
+          <t>2026-07-14 08:30:26.475160+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-10 14:00:31.832545+09:00</t>
+          <t>2026-07-14 08:30:26.475160+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>5491</t>
+          <t>9271</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>364</t>
+          <t>365</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>제4회 개인정보보호 모의재판 경연대회 참가자 모집</t>
+          <t>공공기관 종합청렴도 평가 관련 개인정보 제3자 제공사항 알림</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12245</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12267</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>침해평가과</t>
+          <t>법무감사담당관</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2910,44 +2910,44 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-09 11:01:05.002078+09:00</t>
+          <t>2026-07-13 17:16:17.898453+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-09 11:01:05.002078+09:00</t>
+          <t>2026-07-13 17:16:17.898453+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>5402</t>
+          <t>6541</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>1276</t>
+          <t>1278</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>개인정보위, 안전조치 의무 위반 3개 사업자 제재</t>
+          <t>개인정보 온라인 불법유통 청년들이 직접 차단한다.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12242</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12262</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>장석인</t>
+          <t>조사2과</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2957,7 +2957,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2967,34 +2967,34 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-10 14:00:31.832545+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-10 14:00:31.832545+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>5401</t>
+          <t>5491</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>1277</t>
+          <t>364</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>미래의 개인정보 법률 전문가 모여 인공지능 시대 법적 쟁점 논의한다</t>
+          <t>제4회 개인정보보호 모의재판 경연대회 참가자 모집</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12243</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12245</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -3014,49 +3014,49 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-09 11:01:05.002078+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-09 11:01:05.002078+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>5391</t>
+          <t>5402</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>363</t>
+          <t>1276</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>「개인정보 보호책임자 경력 인정에 관한 고시」 일부개정고시안 행정예고</t>
+          <t>개인정보위, 안전조치 의무 위반 3개 사업자 제재</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12244</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12242</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>장석인</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3071,54 +3071,54 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-09 09:46:03.809898+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-09 09:46:03.809898+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>4581</t>
+          <t>5401</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1275</t>
+          <t>1277</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>개인정보위, 응용프로그램 인터페이스(API) 활용 확대에 따른 개인정보 유출 예방 당부</t>
+          <t>미래의 개인정보 법률 전문가 모여 인공지능 시대 법적 쟁점 논의한다</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12241</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12243</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>사전실태점검과</t>
+          <t>침해평가과</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -3138,44 +3138,44 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-08 10:00:27.128578+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-08 10:00:27.128578+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>3251</t>
+          <t>5391</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>363</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026년 가명정보 활용 지원체계 설명회 개최 안내</t>
+          <t>「개인정보 보호책임자 경력 인정에 관한 고시」 일부개정고시안 행정예고</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12238</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12244</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -3195,44 +3195,44 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-06 13:46:04.662402+09:00</t>
+          <t>2026-07-09 09:46:03.809898+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-06 13:46:04.662402+09:00</t>
+          <t>2026-07-09 09:46:03.809898+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>3182</t>
+          <t>4581</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>1273</t>
+          <t>1275</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>개인정보 처리방침 평가, 국민 눈높이에서 더 꼼꼼히 본다</t>
+          <t>개인정보위, 응용프로그램 인터페이스(API) 활용 확대에 따른 개인정보 유출 예방 당부</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12236</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12241</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>사전실태점검과</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3242,7 +3242,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -3252,39 +3252,39 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-08 10:00:27.128578+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-08 10:00:27.128578+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>3181</t>
+          <t>3251</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>1274</t>
+          <t>362</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>개인정보위, 교육‧고용 분야까지 개인정보 제3자 전송요구권 확대 추진</t>
+          <t>2026년 가명정보 활용 지원체계 설명회 개최 안내</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12237</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12238</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3299,54 +3299,54 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-06 13:46:04.662402+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-06 13:46:04.662402+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1043</t>
+          <t>3182</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>1273</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>개인정보위, 대전에서 ‘찾아가는 개인정보 현장 컨설팅 및 교육’ 개최</t>
+          <t>개인정보 처리방침 평가, 국민 눈높이에서 더 꼼꼼히 본다</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12227</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12236</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3356,7 +3356,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>60</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3366,44 +3366,44 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-03 16:00:28.543767+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-03 16:00:28.543767+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>3181</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>1272</t>
+          <t>1274</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.3.자)</t>
+          <t>개인정보위, 교육‧고용 분야까지 개인정보 제3자 전송요구권 확대 추진</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12229</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12237</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3413,7 +3413,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>58</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3423,39 +3423,39 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-03 15:30:33.546332+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-03 15:30:33.546332+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>561</t>
+          <t>1043</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>1271</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>신뢰로 여는 인공지능(AI) 혁신, 달라지는 개인정보 체계로 이끈다</t>
+          <t>개인정보위, 대전에서 ‘찾아가는 개인정보 현장 컨설팅 및 교육’ 개최</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12228</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12227</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>개인정보보호정책과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3480,44 +3480,44 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-03 10:00:33.422568+09:00</t>
+          <t>2026-07-03 16:00:28.543767+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-03 10:00:33.422568+09:00</t>
+          <t>2026-07-03 16:00:28.543767+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>1001</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>1269</t>
+          <t>1272</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>개인정보위, 인공지능(AI) 시대 데이터 혁신적 활용을 지역 주도로 확산한다.</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.3.자)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12225</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12229</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3527,7 +3527,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3537,44 +3537,44 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-07-02 16:45:30.717611+09:00</t>
+          <t>2026-07-03 15:30:33.546332+09:00</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-02 16:45:30.717611+09:00</t>
+          <t>2026-07-03 15:30:33.546332+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>561</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>1269</t>
+          <t>1271</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>개인정보위, 개인정보보호 현장 간담회 개최</t>
+          <t>신뢰로 여는 인공지능(AI) 혁신, 달라지는 개인정보 체계로 이끈다</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12224</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12228</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>조사1과</t>
+          <t>개인정보보호정책과</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3584,7 +3584,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3594,44 +3594,44 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-03 10:00:33.422568+09:00</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-03 10:00:33.422568+09:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>281</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>1266</t>
+          <t>1269</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>글로벌 개인정보 감독기구에 인공지능(AI) 대응 ‘실전해법’ 제시</t>
+          <t>개인정보위, 인공지능(AI) 시대 데이터 혁신적 활용을 지역 주도로 확산한다.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12218</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12225</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>국제협력담당관</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3641,7 +3641,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>924</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3651,44 +3651,44 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 16:45:30.717611+09:00</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 16:45:30.717611+09:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>1267</t>
+          <t>1269</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>투숙객 개인정보보호에 앞장선 호텔, 호텔업 등급평가시 우대</t>
+          <t>개인정보위, 개인정보보호 현장 간담회 개최</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12219</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12224</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>조사1과</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3698,7 +3698,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1074</t>
+          <t>98</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3720,27 +3720,27 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>1268</t>
+          <t>1266</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.1.자)</t>
+          <t>글로벌 개인정보 감독기구에 인공지능(AI) 대응 ‘실전해법’ 제시</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12220</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12218</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>국제협력담당관</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3755,7 +3755,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>743</t>
+          <t>924</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3777,32 +3777,32 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>361</t>
+          <t>1267</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령(안) 입법예고</t>
+          <t>투숙객 개인정보보호에 앞장선 호텔, 호텔업 등급평가시 우대</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12216</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12219</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>범정부 마이데이터추진단</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3812,44 +3812,44 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1074</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>1265</t>
+          <t>1268</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.6.30.자)</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.1.자)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12217</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12220</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3859,7 +3859,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1029</t>
+          <t>743</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3891,32 +3891,32 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>361</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고</t>
+          <t>「개인정보 보호법 시행령」 일부개정령(안) 입법예고</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12202</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12216</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>범정부 마이데이터추진단</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3926,7 +3926,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>2800</t>
+          <t>1842</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3948,32 +3948,32 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>1262</t>
+          <t>1265</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>개인정보위원장, G7 개인정보 감독기구 라운드테이블 참석</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.6.30.자)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12201</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12217</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>국제협력담당관</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>2144</t>
+          <t>1029</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4005,22 +4005,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>1263</t>
+          <t>360</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>「2026 개인정보 보호·활용 기술 대상」 참여기업 모집</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12203</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12202</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -4040,49 +4040,49 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>2092</t>
+          <t>2800</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>1264</t>
+          <t>1262</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>AI 범죄 대응 범부처 협의체 출범</t>
+          <t>개인정보위원장, G7 개인정보 감독기구 라운드테이블 참석</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12204</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12201</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>인공지능프라이버시팀</t>
+          <t>국제협력담당관</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -4097,7 +4097,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>2638</t>
+          <t>2144</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4119,32 +4119,32 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>359</t>
+          <t>1263</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>본인전송요구 대리인의 사전협의 요청 시범기간(6.25.~7.10.) 운영 안내</t>
+          <t>「2026 개인정보 보호·활용 기술 대상」 참여기업 모집</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12200</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12203</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>신기술개인정보과</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4154,54 +4154,54 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>3745</t>
+          <t>2092</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>1260</t>
+          <t>1264</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>개인정보위, 상조서비스 개인정보 보호 취약요인 선제 점검</t>
+          <t>AI 범죄 대응 범부처 협의체 출범</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12197</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12204</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>사전실태점검과</t>
+          <t>인공지능프라이버시팀</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -4211,7 +4211,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>2754</t>
+          <t>2638</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4233,22 +4233,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>1261</t>
+          <t>359</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>개인정보위, 국민이 필요로 하는 정보 중심 ‘본인전송요구권’ 안착 지원한다</t>
+          <t>본인전송요구 대리인의 사전협의 요청 시범기간(6.25.~7.10.) 운영 안내</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12198</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12200</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -4268,54 +4268,54 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>3085</t>
+          <t>3745</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>358</t>
+          <t>1260</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>정보보호 및 개인정보보호 관리체계 심사기관 지정 공고(제2026-73호)</t>
+          <t>개인정보위, 상조서비스 개인정보 보호 취약요인 선제 점검</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12185</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12197</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>사전실태점검과</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -4325,54 +4325,54 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>7681</t>
+          <t>2754</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>357</t>
+          <t>1261</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>「자율기구 공공실태점검단 설치 및 운영에 관한 규정」 발령(2026-70)</t>
+          <t>개인정보위, 국민이 필요로 하는 정보 중심 ‘본인전송요구권’ 안착 지원한다</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12174</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12198</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>혁신기획담당관</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -4382,44 +4382,44 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>6533</t>
+          <t>3085</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>358</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>공공기관 개인정보 보호수준 평가단원 지원 공고</t>
+          <t>정보보호 및 개인정보보호 관리체계 심사기관 지정 공고(제2026-73호)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12160</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12185</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -4429,7 +4429,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -4439,7 +4439,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>9023</t>
+          <t>7681</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -4461,32 +4461,32 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>352</t>
+          <t>357</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
+          <t>「자율기구 공공실태점검단 설치 및 운영에 관한 규정」 발령(2026-70)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12126</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12174</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>개인정보보호정책과</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>11169</t>
+          <t>6533</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -4518,32 +4518,32 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>354</t>
+          <t>356</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
+          <t>공공기관 개인정보 보호수준 평가단원 지원 공고</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12131</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12160</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -4553,7 +4553,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>13472</t>
+          <t>9023</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -4575,32 +4575,32 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>355</t>
+          <t>352</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12136</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12126</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>개인정보보호정책과</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -4610,7 +4610,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>9724</t>
+          <t>11169</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -4632,55 +4632,169 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>354</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12131</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>조사총괄과</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>13472</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>355</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12136</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>신기술개인정보과</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>9724</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>19</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>353</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>「개인정보 처리 방법에 관한 고시」 일부개정고시안 행정예고</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12127</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>전략기획팀</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F56" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
         <is>
           <t>11519</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
+      <c r="I56" t="inlineStr">
         <is>
           <t>공지사항</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
+      <c r="J56" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
+      <c r="K56" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-29 18:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -6001,7 +6001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K53"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6064,7 +6064,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>20771</t>
+          <t>22464</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6074,50 +6074,50 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
+          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>20191</t>
+          <t>20771</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6127,12 +6127,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
+          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -6142,7 +6142,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -6158,34 +6158,34 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>20061</t>
+          <t>20191</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
+          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -6195,7 +6195,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>287</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -6203,64 +6203,64 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>16785</t>
+          <t>20061</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1496</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
+          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>246</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6268,34 +6268,34 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>16784</t>
+          <t>16785</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1497</t>
+          <t>1496</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -6305,7 +6305,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -6333,22 +6333,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>16781</t>
+          <t>16784</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1497</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>260</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -6366,11 +6366,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6390,22 +6386,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>16691</t>
+          <t>16781</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -6415,35 +6411,39 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>242</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>16464</t>
+          <t>16691</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6453,12 +6453,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
+          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -6468,35 +6468,35 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>278</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>16051</t>
+          <t>16464</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6506,12 +6506,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
+          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -6521,35 +6521,35 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -6559,22 +6559,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -6590,19 +6590,19 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -6612,12 +6612,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -6627,7 +6627,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -6643,34 +6643,34 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -6680,7 +6680,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -6688,56 +6688,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -6745,7 +6741,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6753,34 +6753,34 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -6801,96 +6801,92 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -6900,7 +6896,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -6908,7 +6904,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6916,19 +6916,19 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -6938,12 +6938,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -6953,12 +6953,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -6969,19 +6969,19 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -6991,22 +6991,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -7022,19 +7022,19 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -7044,12 +7044,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -7059,7 +7059,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -7070,96 +7070,92 @@
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -7169,35 +7165,39 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -7207,22 +7207,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -7233,24 +7233,24 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -7260,12 +7260,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -7275,7 +7275,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -7286,24 +7286,24 @@
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -7313,22 +7313,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -7344,44 +7344,44 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -7397,44 +7397,44 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -7442,31 +7442,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -7476,12 +7472,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -7491,7 +7487,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -7523,22 +7519,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -7548,7 +7544,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -7556,27 +7552,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7586,12 +7586,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -7601,113 +7601,113 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -7715,31 +7715,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -7749,12 +7745,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -7764,7 +7760,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -7796,32 +7792,32 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -7829,7 +7825,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7849,22 +7849,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -7874,7 +7874,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -7902,22 +7902,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -7927,19 +7927,15 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7959,7 +7955,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7969,12 +7965,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -7984,7 +7980,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -8016,40 +8012,44 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8069,22 +8069,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -8102,11 +8102,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8126,32 +8122,32 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -8159,7 +8155,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8167,34 +8167,34 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -8204,7 +8204,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -8215,49 +8215,49 @@
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -8285,22 +8285,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -8310,7 +8310,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -8338,32 +8338,32 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -8391,22 +8391,22 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -8416,39 +8416,35 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8458,27 +8454,27 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -8505,32 +8501,32 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -8538,52 +8534,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -8611,32 +8611,32 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -8664,32 +8664,32 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -8717,32 +8717,32 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -8750,46 +8750,42 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14403</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -8799,7 +8795,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>6587</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -8807,52 +8803,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -8872,6 +8872,59 @@
         </is>
       </c>
       <c r="K53" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-29 19:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -6001,7 +6001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K54"/>
+  <dimension ref="A1:K55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6064,7 +6064,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>22464</t>
+          <t>22504</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6074,12 +6074,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -6089,7 +6089,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -6105,19 +6105,19 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>20771</t>
+          <t>22464</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6127,50 +6127,50 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
+          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>20191</t>
+          <t>20771</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6180,12 +6180,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
+          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -6195,7 +6195,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -6211,34 +6211,34 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>20061</t>
+          <t>20191</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
+          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -6248,7 +6248,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>287</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -6256,64 +6256,64 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>16785</t>
+          <t>20061</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1496</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
+          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>246</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6321,34 +6321,34 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>16784</t>
+          <t>16785</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1497</t>
+          <t>1496</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -6386,22 +6386,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>16781</t>
+          <t>16784</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1497</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -6411,7 +6411,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>260</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -6419,11 +6419,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6443,22 +6439,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>16691</t>
+          <t>16781</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -6468,35 +6464,39 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>242</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>16464</t>
+          <t>16691</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6506,12 +6506,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
+          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -6521,35 +6521,35 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>278</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>16051</t>
+          <t>16464</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -6559,12 +6559,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
+          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -6574,35 +6574,35 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -6612,22 +6612,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -6643,19 +6643,19 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -6665,12 +6665,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -6680,7 +6680,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -6696,34 +6696,34 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -6733,7 +6733,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -6741,56 +6741,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -6798,7 +6794,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6806,34 +6806,34 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -6843,7 +6843,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -6854,96 +6854,92 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -6953,7 +6949,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -6961,7 +6957,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6969,19 +6969,19 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -6991,12 +6991,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -7006,12 +7006,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -7022,19 +7022,19 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -7044,22 +7044,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -7075,19 +7075,19 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -7097,12 +7097,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -7112,7 +7112,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -7123,96 +7123,92 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -7222,35 +7218,39 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -7260,22 +7260,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -7286,24 +7286,24 @@
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -7313,12 +7313,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -7328,7 +7328,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -7339,24 +7339,24 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -7366,22 +7366,22 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -7397,44 +7397,44 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -7450,44 +7450,44 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -7495,31 +7495,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -7529,12 +7525,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -7544,7 +7540,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -7576,22 +7572,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -7601,7 +7597,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -7609,27 +7605,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7639,12 +7639,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -7654,113 +7654,113 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -7768,31 +7768,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -7802,12 +7798,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -7817,7 +7813,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -7849,32 +7845,32 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -7882,7 +7878,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7902,22 +7902,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -7927,7 +7927,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -7955,22 +7955,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -7980,19 +7980,15 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8012,7 +8008,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -8022,12 +8018,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -8037,7 +8033,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -8069,40 +8065,44 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8122,22 +8122,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -8147,7 +8147,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -8155,11 +8155,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8179,32 +8175,32 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -8212,7 +8208,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I41" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8220,34 +8220,34 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -8257,7 +8257,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -8268,49 +8268,49 @@
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -8338,22 +8338,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -8363,7 +8363,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -8391,32 +8391,32 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -8444,22 +8444,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -8469,39 +8469,35 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -8511,27 +8507,27 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -8558,32 +8554,32 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -8591,52 +8587,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -8664,32 +8664,32 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -8717,32 +8717,32 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -8770,32 +8770,32 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -8803,46 +8803,42 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14403</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -8852,7 +8848,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>6587</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -8860,52 +8856,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -8925,6 +8925,59 @@
         </is>
       </c>
       <c r="K54" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-30 10:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,27 +465,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -495,39 +495,39 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -537,39 +537,39 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -579,39 +579,39 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -621,29 +621,29 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -675,27 +675,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -717,27 +717,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -759,27 +759,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -801,27 +801,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -843,27 +843,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -885,27 +885,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -927,27 +927,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -969,40 +969,82 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-30 11:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -1647,7 +1647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K56"/>
+  <dimension ref="A1:K57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1710,32 +1710,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>22391</t>
+          <t>22661</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>374</t>
+          <t>1289</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>개인정보 영향평가기관 지정갱신 공고</t>
+          <t>개인정보위, ‘㈜KT의개인정보 유출사고’ 제재처분 의결</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12346</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12349</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>조사2과</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1745,29 +1745,29 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>50</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-29 17:16:05.593491+09:00</t>
+          <t>2026-07-30 10:30:27.268351+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-29 17:16:05.593491+09:00</t>
+          <t>2026-07-30 10:30:27.268351+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>22351</t>
+          <t>22391</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12345</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12346</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1812,44 +1812,44 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-29 16:46:07.286593+09:00</t>
+          <t>2026-07-29 17:16:05.593491+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-29 16:46:07.286593+09:00</t>
+          <t>2026-07-29 17:16:05.593491+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>17701</t>
+          <t>22351</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1288</t>
+          <t>374</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>유럽연합, 한국 개인정보 보호 수준 재확인… 적정성 결정 유지</t>
+          <t>개인정보 영향평가기관 지정갱신 공고</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12333</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12345</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>국제협력담당관</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1859,54 +1859,54 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-24 10:00:27.219427+09:00</t>
+          <t>2026-07-29 16:46:07.286593+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-24 10:00:27.219427+09:00</t>
+          <t>2026-07-29 16:46:07.286593+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>17362</t>
+          <t>17701</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1286</t>
+          <t>1288</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>「2026 개인정보 미래포럼」 제3차 전체회의 개최</t>
+          <t>유럽연합, 한국 개인정보 보호 수준 재확인… 적정성 결정 유지</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12329</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12333</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>혁신기획담당관</t>
+          <t>국제협력담당관</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1916,7 +1916,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1926,39 +1926,39 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-23 16:00:30.422263+09:00</t>
+          <t>2026-07-24 10:00:27.219427+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-23 16:00:30.422263+09:00</t>
+          <t>2026-07-24 10:00:27.219427+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>16883</t>
+          <t>17362</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1285</t>
+          <t>1286</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>국민이 신뢰할 수 있는 공공 인공지능 전환(AX),프라이버시 보호로 적극 뒷받침</t>
+          <t>「2026 개인정보 미래포럼」 제3차 전체회의 개최</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12307</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12329</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>인공지능프라이버시팀</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1983,34 +1983,34 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-23 10:00:38.625145+09:00</t>
+          <t>2026-07-23 16:00:30.422263+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-23 10:00:38.625145+09:00</t>
+          <t>2026-07-23 16:00:30.422263+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>16882</t>
+          <t>16883</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1286</t>
+          <t>1285</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>대도약의 골든타임, 초격차 성장동력 확보와 AI 생태계 발전기반 강화</t>
+          <t>국민이 신뢰할 수 있는 공공 인공지능 전환(AX),프라이버시 보호로 적극 뒷받침</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12308</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12307</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -2052,27 +2052,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>16881</t>
+          <t>16882</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1287</t>
+          <t>1286</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>개인정보위, 적법 근거 없이 개인정보수집·이용한 틱톡·애플 제재</t>
+          <t>대도약의 골든타임, 초격차 성장동력 확보와 AI 생태계 발전기반 강화</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12330</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12308</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>조사1과</t>
+          <t>인공지능프라이버시팀</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -2109,32 +2109,32 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>16314</t>
+          <t>16881</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>370</t>
+          <t>1287</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>「개인정보 보호위원회의 조사 및 처분에 관한 규정」 일부개정안 행정예고</t>
+          <t>개인정보위, 적법 근거 없이 개인정보수집·이용한 틱톡·애플 제재</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12309</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12330</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>조사1과</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2144,44 +2144,44 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-22 13:01:11.478354+09:00</t>
+          <t>2026-07-23 10:00:38.625145+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-22 13:01:11.478354+09:00</t>
+          <t>2026-07-23 10:00:38.625145+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>16313</t>
+          <t>16314</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>371</t>
+          <t>370</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>「개인정보 보호 법규 위반에 대한 고발 기준」 제정안 행정예고</t>
+          <t>「개인정보 보호위원회의 조사 및 처분에 관한 규정」 일부개정안 행정예고</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12310</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12309</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -2223,22 +2223,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>16312</t>
+          <t>16313</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>372</t>
+          <t>371</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>「개인정보 보호 법규 위반에 대한 징계권고 기준」 제정안 행정예고</t>
+          <t>「개인정보 보호 법규 위반에 대한 고발 기준」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12311</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12310</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -2280,22 +2280,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>16311</t>
+          <t>16312</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>373</t>
+          <t>372</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 위반에 대한 공표 및 공표명령 지침」 제정안 행정예고</t>
+          <t>「개인정보 보호 법규 위반에 대한 징계권고 기준」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12312</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12311</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -2315,7 +2315,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -2337,32 +2337,32 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>14451</t>
+          <t>16311</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>369</t>
+          <t>373</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>본인전송요구 대리인의 사전협의 요청 시범기간 추가운영(7.20.~31.) 안내</t>
+          <t>「개인정보 보호법 위반에 대한 공표 및 공표명령 지침」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12289</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12312</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -2382,39 +2382,39 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-20 10:16:06.541093+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-20 10:16:06.541093+09:00</t>
+          <t>2026-07-22 13:01:11.478354+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>14433</t>
+          <t>14451</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>366</t>
+          <t>369</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>본인전송요구 대리인의 사전협의 요청 시범기간 추가운영(7.20.~31.) 안내</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12278</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12289</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -2439,34 +2439,34 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:08.116520+09:00</t>
+          <t>2026-07-20 10:16:06.541093+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:08.116520+09:00</t>
+          <t>2026-07-20 10:16:06.541093+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>14422</t>
+          <t>14433</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1282</t>
+          <t>366</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>「개인정보 이노베이션 존」 신규 운영기관 공모</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12287</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12278</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -2486,49 +2486,49 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-20 10:00:27.102836+09:00</t>
+          <t>2026-07-20 10:01:08.116520+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-20 10:00:27.102836+09:00</t>
+          <t>2026-07-20 10:01:08.116520+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14422</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1283</t>
+          <t>1282</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>개인정보위, ‘본인전송요구권’ 사전협의 지원 시범운영 7월 31일까지 추가신청 받는다</t>
+          <t>「개인정보 이노베이션 존」 신규 운영기관 공모</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12288</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12287</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2565,32 +2565,32 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>11392</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>367</t>
+          <t>1283</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 위반에 대한 과징금 부과기준」 일부개정안 행정예고</t>
+          <t>개인정보위, ‘본인전송요구권’ 사전협의 지원 시범운영 7월 31일까지 추가신청 받는다</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12282</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12288</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2600,44 +2600,44 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-16 13:01:06.075969+09:00</t>
+          <t>2026-07-20 10:00:27.102836+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-16 13:01:06.075969+09:00</t>
+          <t>2026-07-20 10:00:27.102836+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>11391</t>
+          <t>11392</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>368</t>
+          <t>367</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 위반에 대한 과태료 부과기준」 제정안 행정예고</t>
+          <t>「개인정보 보호법 위반에 대한 과징금 부과기준」 일부개정안 행정예고</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12284</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12282</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2679,27 +2679,27 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>11221</t>
+          <t>11391</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1281</t>
+          <t>368</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AI 혁신을 뒷받침하고 국민 권익을 증진하는 예방중심 개인정보 보호 실현</t>
+          <t>「개인정보 보호법 위반에 대한 과태료 부과기준」 제정안 행정예고</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12281</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12284</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>혁신기획담당관</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2714,54 +2714,54 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-16 11:00:27.819143+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-16 11:00:27.819143+09:00</t>
+          <t>2026-07-16 13:01:06.075969+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>10301</t>
+          <t>11221</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1280</t>
+          <t>1281</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.15.자)</t>
+          <t>AI 혁신을 뒷받침하고 국민 권익을 증진하는 예방중심 개인정보 보호 실현</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12276</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12281</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2781,44 +2781,44 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-15 09:45:30.272302+09:00</t>
+          <t>2026-07-16 11:00:27.819143+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-15 09:45:30.272302+09:00</t>
+          <t>2026-07-16 11:00:27.819143+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>9501</t>
+          <t>10301</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1279</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>개인정보 전송요구권 전송체계 기술적 기틀, 고용⋅교육 부문까지 확대 마련</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.15.자)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12266</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12276</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>인프라표준화팀</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2828,7 +2828,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2838,44 +2838,44 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-14 10:00:29.933870+09:00</t>
+          <t>2026-07-15 09:45:30.272302+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-14 10:00:29.933870+09:00</t>
+          <t>2026-07-15 09:45:30.272302+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>9381</t>
+          <t>9501</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1280</t>
+          <t>1279</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>정보주체의 본인전송요구권, 더 안전하게 이용할 수 있습니다</t>
+          <t>개인정보 전송요구권 전송체계 기술적 기틀, 고용⋅교육 부문까지 확대 마련</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12273</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12266</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>범정부마이데이터추진단 전략기획팀</t>
+          <t>인프라표준화팀</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2885,7 +2885,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2895,39 +2895,39 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-14 08:30:26.475160+09:00</t>
+          <t>2026-07-14 10:00:29.933870+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-14 08:30:26.475160+09:00</t>
+          <t>2026-07-14 10:00:29.933870+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>9271</t>
+          <t>9381</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>365</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>공공기관 종합청렴도 평가 관련 개인정보 제3자 제공사항 알림</t>
+          <t>정보주체의 본인전송요구권, 더 안전하게 이용할 수 있습니다</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12267</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12273</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>법무감사담당관</t>
+          <t>범정부마이데이터추진단 전략기획팀</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2937,116 +2937,116 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>303</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-13 17:16:17.898453+09:00</t>
+          <t>2026-07-14 08:30:26.475160+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-13 17:16:17.898453+09:00</t>
+          <t>2026-07-14 08:30:26.475160+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>6541</t>
+          <t>9271</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>1278</t>
+          <t>365</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>개인정보 온라인 불법유통 청년들이 직접 차단한다.</t>
+          <t>공공기관 종합청렴도 평가 관련 개인정보 제3자 제공사항 알림</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12262</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12267</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>조사2과</t>
+          <t>법무감사담당관</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-10 14:00:31.832545+09:00</t>
+          <t>2026-07-13 17:16:17.898453+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-10 14:00:31.832545+09:00</t>
+          <t>2026-07-13 17:16:17.898453+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>5491</t>
+          <t>6541</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>364</t>
+          <t>1278</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>제4회 개인정보보호 모의재판 경연대회 참가자 모집</t>
+          <t>개인정보 온라인 불법유통 청년들이 직접 차단한다.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12245</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12262</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>침해평가과</t>
+          <t>조사2과</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -3056,49 +3056,49 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-09 11:01:05.002078+09:00</t>
+          <t>2026-07-10 14:00:31.832545+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-09 11:01:05.002078+09:00</t>
+          <t>2026-07-10 14:00:31.832545+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>5402</t>
+          <t>5491</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>1276</t>
+          <t>364</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>개인정보위, 안전조치 의무 위반 3개 사업자 제재</t>
+          <t>제4회 개인정보보호 모의재판 경연대회 참가자 모집</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12242</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12245</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>장석인</t>
+          <t>침해평가과</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3113,49 +3113,49 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-09 11:01:05.002078+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-09 10:00:57.524524+09:00</t>
+          <t>2026-07-09 11:01:05.002078+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>5401</t>
+          <t>5402</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1277</t>
+          <t>1276</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>미래의 개인정보 법률 전문가 모여 인공지능 시대 법적 쟁점 논의한다</t>
+          <t>개인정보위, 안전조치 의무 위반 3개 사업자 제재</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12243</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12242</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>침해평가과</t>
+          <t>장석인</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -3192,27 +3192,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>5391</t>
+          <t>5401</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>363</t>
+          <t>1277</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>「개인정보 보호책임자 경력 인정에 관한 고시」 일부개정고시안 행정예고</t>
+          <t>미래의 개인정보 법률 전문가 모여 인공지능 시대 법적 쟁점 논의한다</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12244</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12243</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>침해평가과</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3227,54 +3227,54 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-09 09:46:03.809898+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-09 09:46:03.809898+09:00</t>
+          <t>2026-07-09 10:00:57.524524+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>4581</t>
+          <t>5391</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>1275</t>
+          <t>363</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>개인정보위, 응용프로그램 인터페이스(API) 활용 확대에 따른 개인정보 유출 예방 당부</t>
+          <t>「개인정보 보호책임자 경력 인정에 관한 고시」 일부개정고시안 행정예고</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12241</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12244</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>사전실태점검과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3284,54 +3284,54 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-08 10:00:27.128578+09:00</t>
+          <t>2026-07-09 09:46:03.809898+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-08 10:00:27.128578+09:00</t>
+          <t>2026-07-09 09:46:03.809898+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>3251</t>
+          <t>4581</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>1275</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026년 가명정보 활용 지원체계 설명회 개최 안내</t>
+          <t>개인정보위, 응용프로그램 인터페이스(API) 활용 확대에 따른 개인정보 유출 예방 당부</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12238</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12241</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>사전실태점검과</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3341,49 +3341,49 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-06 13:46:04.662402+09:00</t>
+          <t>2026-07-08 10:00:27.128578+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-06 13:46:04.662402+09:00</t>
+          <t>2026-07-08 10:00:27.128578+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>3182</t>
+          <t>3251</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>1273</t>
+          <t>362</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>개인정보 처리방침 평가, 국민 눈높이에서 더 꼼꼼히 본다</t>
+          <t>2026년 가명정보 활용 지원체계 설명회 개최 안내</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12236</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12238</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3398,49 +3398,49 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-06 13:46:04.662402+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-06 12:45:29.985993+09:00</t>
+          <t>2026-07-06 13:46:04.662402+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>3181</t>
+          <t>3182</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>1274</t>
+          <t>1273</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>개인정보위, 교육‧고용 분야까지 개인정보 제3자 전송요구권 확대 추진</t>
+          <t>개인정보 처리방침 평가, 국민 눈높이에서 더 꼼꼼히 본다</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12237</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12236</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3455,7 +3455,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>60</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3477,32 +3477,32 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1043</t>
+          <t>3181</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>1274</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>개인정보위, 대전에서 ‘찾아가는 개인정보 현장 컨설팅 및 교육’ 개최</t>
+          <t>개인정보위, 교육‧고용 분야까지 개인정보 제3자 전송요구권 확대 추진</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12227</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12237</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>58</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3522,39 +3522,39 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-03 16:00:28.543767+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-03 16:00:28.543767+09:00</t>
+          <t>2026-07-06 12:45:29.985993+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>1043</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>1272</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.3.자)</t>
+          <t>개인정보위, 대전에서 ‘찾아가는 개인정보 현장 컨설팅 및 교육’ 개최</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12229</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12227</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -3569,7 +3569,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3579,39 +3579,39 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-07-03 15:30:33.546332+09:00</t>
+          <t>2026-07-03 16:00:28.543767+09:00</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-03 15:30:33.546332+09:00</t>
+          <t>2026-07-03 16:00:28.543767+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>561</t>
+          <t>1001</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>1271</t>
+          <t>1272</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>신뢰로 여는 인공지능(AI) 혁신, 달라지는 개인정보 체계로 이끈다</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.3.자)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12228</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12229</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>개인정보보호정책과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3636,44 +3636,44 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-07-03 10:00:33.422568+09:00</t>
+          <t>2026-07-03 15:30:33.546332+09:00</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-07-03 10:00:33.422568+09:00</t>
+          <t>2026-07-03 15:30:33.546332+09:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>561</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>1269</t>
+          <t>1271</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>개인정보위, 인공지능(AI) 시대 데이터 혁신적 활용을 지역 주도로 확산한다.</t>
+          <t>신뢰로 여는 인공지능(AI) 혁신, 달라지는 개인정보 체계로 이끈다</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12225</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12228</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>데이터안전정책과</t>
+          <t>개인정보보호정책과</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3693,19 +3693,19 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-07-02 16:45:30.717611+09:00</t>
+          <t>2026-07-03 10:00:33.422568+09:00</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-02 16:45:30.717611+09:00</t>
+          <t>2026-07-03 10:00:33.422568+09:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>281</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3715,17 +3715,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>개인정보위, 개인정보보호 현장 간담회 개최</t>
+          <t>개인정보위, 인공지능(AI) 시대 데이터 혁신적 활용을 지역 주도로 확산한다.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12224</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12225</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>조사1과</t>
+          <t>데이터안전정책과</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -3740,7 +3740,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3750,44 +3750,44 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 16:45:30.717611+09:00</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 16:45:30.717611+09:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>1266</t>
+          <t>1269</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>글로벌 개인정보 감독기구에 인공지능(AI) 대응 ‘실전해법’ 제시</t>
+          <t>개인정보위, 개인정보보호 현장 간담회 개최</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12218</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12224</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>국제협력담당관</t>
+          <t>조사1과</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>924</t>
+          <t>98</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3819,27 +3819,27 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>1267</t>
+          <t>1266</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>투숙객 개인정보보호에 앞장선 호텔, 호텔업 등급평가시 우대</t>
+          <t>글로벌 개인정보 감독기구에 인공지능(AI) 대응 ‘실전해법’ 제시</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12219</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12218</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>국제협력담당관</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3854,7 +3854,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1074</t>
+          <t>924</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3876,27 +3876,27 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>1268</t>
+          <t>1267</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.1.자)</t>
+          <t>투숙객 개인정보보호에 앞장선 호텔, 호텔업 등급평가시 우대</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12220</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12219</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3911,7 +3911,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>743</t>
+          <t>1074</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3933,32 +3933,32 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>361</t>
+          <t>1268</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령(안) 입법예고</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.7.1.자)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12216</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12220</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>범정부 마이데이터추진단</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3968,49 +3968,49 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>743</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>1265</t>
+          <t>361</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>(인사발령) 개인정보보호위원회 인사발령('26.6.30.자)</t>
+          <t>「개인정보 보호법 시행령」 일부개정령(안) 입법예고</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12217</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12216</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>범정부 마이데이터추진단</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -4025,54 +4025,54 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1029</t>
+          <t>1842</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>1265</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고</t>
+          <t>(인사발령) 개인정보보호위원회 인사발령('26.6.30.자)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12202</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12217</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4082,49 +4082,49 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>2800</t>
+          <t>1029</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>1262</t>
+          <t>360</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>개인정보위원장, G7 개인정보 감독기구 라운드테이블 참석</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12201</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12202</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>국제협력담당관</t>
+          <t>신기술개인정보과</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -4139,49 +4139,49 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>2144</t>
+          <t>2800</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>1263</t>
+          <t>1262</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>「2026 개인정보 보호·활용 기술 대상」 참여기업 모집</t>
+          <t>개인정보위원장, G7 개인정보 감독기구 라운드테이블 참석</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12203</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12201</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>국제협력담당관</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -4196,7 +4196,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>2092</t>
+          <t>2144</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4218,27 +4218,27 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>1264</t>
+          <t>1263</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>AI 범죄 대응 범부처 협의체 출범</t>
+          <t>「2026 개인정보 보호·활용 기술 대상」 참여기업 모집</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12204</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12203</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>인공지능프라이버시팀</t>
+          <t>신기술개인정보과</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -4253,7 +4253,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>2638</t>
+          <t>2092</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4275,32 +4275,32 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>359</t>
+          <t>1264</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>본인전송요구 대리인의 사전협의 요청 시범기간(6.25.~7.10.) 운영 안내</t>
+          <t>AI 범죄 대응 범부처 협의체 출범</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12200</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12204</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>인공지능프라이버시팀</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -4310,49 +4310,49 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>3745</t>
+          <t>2638</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>1260</t>
+          <t>359</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>개인정보위, 상조서비스 개인정보 보호 취약요인 선제 점검</t>
+          <t>본인전송요구 대리인의 사전협의 요청 시범기간(6.25.~7.10.) 운영 안내</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12197</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12200</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>사전실태점검과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -4367,49 +4367,49 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>2754</t>
+          <t>3745</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:32.838364+09:00</t>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>1261</t>
+          <t>1260</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>개인정보위, 국민이 필요로 하는 정보 중심 ‘본인전송요구권’ 안착 지원한다</t>
+          <t>개인정보위, 상조서비스 개인정보 보호 취약요인 선제 점검</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12198</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12197</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>전략기획팀</t>
+          <t>사전실태점검과</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -4424,7 +4424,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>3085</t>
+          <t>2754</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -4446,32 +4446,32 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>358</t>
+          <t>1261</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>정보보호 및 개인정보보호 관리체계 심사기관 지정 공고(제2026-73호)</t>
+          <t>개인정보위, 국민이 필요로 하는 정보 중심 ‘본인전송요구권’ 안착 지원한다</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12185</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS074&amp;mCode=C020010000&amp;nttId=12198</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>전략기획팀</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -4481,54 +4481,54 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>7681</t>
+          <t>3085</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:09.583121+09:00</t>
+          <t>2026-07-02 13:14:32.838364+09:00</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>357</t>
+          <t>358</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>「자율기구 공공실태점검단 설치 및 운영에 관한 규정」 발령(2026-70)</t>
+          <t>정보보호 및 개인정보보호 관리체계 심사기관 지정 공고(제2026-73호)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12174</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12185</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>혁신기획담당관</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -4538,7 +4538,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>6533</t>
+          <t>7681</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -4560,32 +4560,32 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>357</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>공공기관 개인정보 보호수준 평가단원 지원 공고</t>
+          <t>「자율기구 공공실태점검단 설치 및 운영에 관한 규정」 발령(2026-70)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12160</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12174</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>자율보호정책과</t>
+          <t>혁신기획담당관</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -4595,7 +4595,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>9023</t>
+          <t>6533</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -4617,32 +4617,32 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>352</t>
+          <t>356</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
+          <t>공공기관 개인정보 보호수준 평가단원 지원 공고</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12126</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12160</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>개인정보보호정책과</t>
+          <t>자율보호정책과</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -4652,7 +4652,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>11169</t>
+          <t>9023</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -4674,12 +4674,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>354</t>
+          <t>352</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -4689,17 +4689,17 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12131</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12126</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>조사총괄과</t>
+          <t>개인정보보호정책과</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -4709,7 +4709,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>13472</t>
+          <t>11169</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -4731,27 +4731,27 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>355</t>
+          <t>354</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+          <t>「개인정보 보호법 시행령」 일부개정령안 입법예고</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12136</t>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12131</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>신기술개인정보과</t>
+          <t>조사총괄과</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>9724</t>
+          <t>13472</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -4788,55 +4788,112 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>355</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12136</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>신기술개인정보과</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>9724</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:09.583121+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>19</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>353</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>「개인정보 처리 방법에 관한 고시」 일부개정고시안 행정예고</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D57" t="inlineStr">
         <is>
           <t>https://www.pipc.go.kr/np/cop/bbs/selectBoardArticle.do?bbsId=BS061&amp;mCode=C010010000&amp;nttId=12127</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>전략기획팀</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="F57" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
         <is>
           <t>11519</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
+      <c r="I57" t="inlineStr">
         <is>
           <t>공지사항</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
+      <c r="J57" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr">
+      <c r="K57" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:09.583121+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-30 17:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -6100,7 +6100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6163,40 +6163,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>22504</t>
+          <t>23221</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
+          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6204,19 +6208,19 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>22464</t>
+          <t>22504</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6226,12 +6230,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -6241,7 +6245,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -6257,19 +6261,19 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>20771</t>
+          <t>22464</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6279,50 +6283,50 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
+          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>20191</t>
+          <t>20771</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6332,12 +6336,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
+          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -6347,7 +6351,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -6363,34 +6367,34 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>20061</t>
+          <t>20191</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
+          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -6400,7 +6404,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>287</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -6408,64 +6412,64 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>16785</t>
+          <t>20061</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1496</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
+          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>246</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6473,34 +6477,34 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>16784</t>
+          <t>16785</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1497</t>
+          <t>1496</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -6510,7 +6514,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -6538,22 +6542,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>16781</t>
+          <t>16784</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1497</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -6563,7 +6567,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>260</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -6571,11 +6575,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6595,22 +6595,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>16691</t>
+          <t>16781</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -6620,35 +6620,39 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>242</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>16464</t>
+          <t>16691</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -6658,12 +6662,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
+          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -6673,35 +6677,35 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>278</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>16051</t>
+          <t>16464</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -6711,12 +6715,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
+          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -6726,35 +6730,35 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -6764,22 +6768,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -6795,19 +6799,19 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -6817,12 +6821,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -6832,7 +6836,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -6848,34 +6852,34 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -6885,7 +6889,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -6893,56 +6897,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -6950,7 +6950,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6958,34 +6962,34 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -6995,7 +6999,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -7006,96 +7010,92 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -7105,7 +7105,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -7113,7 +7113,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7121,19 +7125,19 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -7143,12 +7147,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -7158,12 +7162,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -7174,19 +7178,19 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -7196,22 +7200,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -7227,19 +7231,19 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -7249,12 +7253,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -7264,7 +7268,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -7275,96 +7279,92 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -7374,35 +7374,39 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -7412,22 +7416,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -7438,24 +7442,24 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -7465,12 +7469,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -7480,7 +7484,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -7491,24 +7495,24 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -7518,22 +7522,22 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -7549,44 +7553,44 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -7602,44 +7606,44 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -7647,31 +7651,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7681,12 +7681,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -7728,22 +7728,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -7753,7 +7753,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -7761,27 +7761,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -7791,12 +7795,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -7806,113 +7810,113 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -7920,31 +7924,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -7954,12 +7954,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -7969,7 +7969,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -8001,32 +8001,32 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -8034,7 +8034,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8054,22 +8058,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -8079,7 +8083,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -8107,22 +8111,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -8132,19 +8136,15 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8164,7 +8164,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -8174,12 +8174,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -8189,7 +8189,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -8221,40 +8221,44 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8274,22 +8278,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -8299,7 +8303,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -8307,11 +8311,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8331,32 +8331,32 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -8364,7 +8364,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8372,34 +8376,34 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -8409,7 +8413,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -8420,49 +8424,49 @@
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -8490,22 +8494,22 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -8515,7 +8519,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -8543,32 +8547,32 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -8596,22 +8600,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -8621,39 +8625,35 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -8663,27 +8663,27 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -8710,32 +8710,32 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -8743,52 +8743,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -8816,32 +8820,32 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -8869,32 +8873,32 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -8922,32 +8926,32 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -8955,46 +8959,42 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14403</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -9004,7 +9004,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>6587</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -9012,52 +9012,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -9077,6 +9081,59 @@
         </is>
       </c>
       <c r="K55" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-31 10:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,27 +465,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -495,39 +495,39 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -537,39 +537,39 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -579,39 +579,39 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -621,39 +621,39 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -663,29 +663,29 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -717,27 +717,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -759,27 +759,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -801,27 +801,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -843,27 +843,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -885,27 +885,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -927,27 +927,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -969,27 +969,27 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1011,40 +1011,82 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-07-31 11:20:02 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,22 +465,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>11711</t>
+          <t>11761</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
+          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법제교육과</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -495,39 +495,39 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -537,39 +537,39 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -579,39 +579,39 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -621,39 +621,39 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -663,39 +663,39 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -705,29 +705,29 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -759,27 +759,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -801,27 +801,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -843,27 +843,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -885,27 +885,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -927,27 +927,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -969,27 +969,27 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1011,27 +1011,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1053,40 +1053,82 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-08-03 09:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -6184,7 +6184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K56"/>
+  <dimension ref="A1:K60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6247,7 +6247,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>23221</t>
+          <t>25864</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6257,22 +6257,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
+          <t>2026년 전남광주통합특별시 소상공인·사회적경제기업 판로 확대 지원기업 선발 안내(~8.14)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3730&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -6292,52 +6292,56 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>22504</t>
+          <t>25863</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
+          <t>2026년 전남광주통합특별시 지역문제 해결 프로젝트 공모전 개최 안내(~8.21)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3731&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6345,52 +6349,56 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>22464</t>
+          <t>25862</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
+          <t>2026년 한국인터넷진흥원 지역공부방 참여 대학생 장학금 지원자 모집 안내(~8.28)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3732&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6398,44 +6406,44 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>20771</t>
+          <t>25861</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
+          <t>2026년 암호모듈 시험자 양성교육 및 필기시험 안내(8.3~8.21)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3733&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -6443,52 +6451,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>20191</t>
+          <t>23221</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
+          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -6496,64 +6508,64 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>20061</t>
+          <t>22504</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6561,44 +6573,44 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>16785</t>
+          <t>22464</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1496</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
+          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -6614,154 +6626,150 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>16784</t>
+          <t>20771</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1497</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
+          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>16781</t>
+          <t>20191</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
+          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>287</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>16691</t>
+          <t>20061</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
+          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>246</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -6769,42 +6777,46 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>16464</t>
+          <t>16785</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1496</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -6814,7 +6826,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -6830,34 +6842,34 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>16051</t>
+          <t>16784</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1497</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -6867,88 +6879,92 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>260</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16781</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>242</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>16691</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -6958,22 +6974,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>278</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -6989,56 +7005,52 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>16464</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7046,44 +7058,44 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -7094,24 +7106,24 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -7121,22 +7133,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -7152,109 +7164,109 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7262,44 +7274,44 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -7315,19 +7327,19 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -7337,22 +7349,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -7363,102 +7375,106 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -7466,11 +7482,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7478,19 +7490,19 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -7500,22 +7512,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -7526,24 +7538,24 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -7553,22 +7565,22 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -7584,19 +7596,19 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -7606,22 +7618,22 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -7637,97 +7649,101 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -7743,39 +7759,39 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -7788,11 +7804,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7800,44 +7812,44 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -7845,31 +7857,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -7879,22 +7887,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -7910,97 +7918,97 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -8008,27 +8016,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -8038,22 +8050,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -8073,44 +8085,44 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -8118,61 +8130,57 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
@@ -8183,44 +8191,44 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -8231,24 +8239,24 @@
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -8258,27 +8266,27 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -8305,7 +8313,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -8315,27 +8323,27 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -8362,32 +8370,32 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -8415,32 +8423,32 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -8448,11 +8456,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8472,40 +8476,44 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I43" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8513,97 +8521,101 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -8614,49 +8626,49 @@
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -8664,52 +8676,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -8720,106 +8736,102 @@
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -8827,56 +8839,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -8904,32 +8912,32 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -8957,85 +8965,89 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -9043,52 +9055,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -9096,56 +9112,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -9173,32 +9185,32 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -9218,6 +9230,222 @@
         </is>
       </c>
       <c r="K56" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>951</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>184573</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>14403</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>공지</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>6587</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>950</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>51749</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-08-03 10:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,27 +465,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>11761</t>
+          <t>12952</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
+          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>법제교육과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -495,39 +495,39 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>11711</t>
+          <t>12951</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
+          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -537,39 +537,39 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11761</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>법제교육과</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -579,39 +579,39 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -621,39 +621,39 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -663,39 +663,39 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -705,39 +705,39 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -747,39 +747,39 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -789,39 +789,39 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -843,27 +843,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -885,27 +885,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -927,27 +927,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -969,27 +969,27 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1011,27 +1011,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1053,27 +1053,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1095,40 +1095,124 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>혁신행정감사담당관실</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
@@ -6184,7 +6268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K60"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6247,22 +6331,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>25864</t>
+          <t>25891</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026년 전남광주통합특별시 소상공인·사회적경제기업 판로 확대 지원기업 선발 안내(~8.14)</t>
+          <t>한국인터넷진흥원, 지역 상생 3대 사업 참여자 모집</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3730&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2621&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -6272,7 +6356,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>80</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -6280,31 +6364,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-08-03 09:16:35.817723+09:00</t>
+          <t>2026-08-03 09:31:46.854132+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-08-03 09:16:35.817723+09:00</t>
+          <t>2026-08-03 09:31:46.854132+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>25863</t>
+          <t>25864</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6314,12 +6394,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026년 전남광주통합특별시 지역문제 해결 프로젝트 공모전 개최 안내(~8.21)</t>
+          <t>2026년 전남광주통합특별시 소상공인·사회적경제기업 판로 확대 지원기업 선발 안내(~8.14)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3731&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3730&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -6329,7 +6409,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -6361,7 +6441,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>25862</t>
+          <t>25863</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6371,12 +6451,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026년 한국인터넷진흥원 지역공부방 참여 대학생 장학금 지원자 모집 안내(~8.28)</t>
+          <t>2026년 전남광주통합특별시 지역문제 해결 프로젝트 공모전 개최 안내(~8.21)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3732&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3731&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -6386,7 +6466,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -6418,7 +6498,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>25861</t>
+          <t>25862</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6428,12 +6508,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026년 암호모듈 시험자 양성교육 및 필기시험 안내(8.3~8.21)</t>
+          <t>2026년 한국인터넷진흥원 지역공부방 참여 대학생 장학금 지원자 모집 안내(~8.28)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3733&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3732&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -6443,7 +6523,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -6475,7 +6555,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>23221</t>
+          <t>25861</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6485,22 +6565,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
+          <t>2026년 암호모듈 시험자 양성교육 및 필기시험 안내(8.3~8.21)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3733&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -6520,52 +6600,56 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>22504</t>
+          <t>23221</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
+          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6573,19 +6657,19 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>22464</t>
+          <t>22504</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6595,12 +6679,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -6610,7 +6694,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -6626,19 +6710,19 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>20771</t>
+          <t>22464</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6648,50 +6732,50 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
+          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>20191</t>
+          <t>20771</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6701,12 +6785,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
+          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -6716,7 +6800,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -6732,34 +6816,34 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>20061</t>
+          <t>20191</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
+          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -6769,7 +6853,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>287</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -6777,64 +6861,64 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>16785</t>
+          <t>20061</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1496</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
+          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>246</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6842,34 +6926,34 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>16784</t>
+          <t>16785</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1497</t>
+          <t>1496</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -6879,7 +6963,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -6907,22 +6991,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>16781</t>
+          <t>16784</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1497</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -6932,7 +7016,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>260</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -6940,11 +7024,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6964,22 +7044,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>16691</t>
+          <t>16781</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -6989,35 +7069,39 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>242</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>16464</t>
+          <t>16691</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -7027,12 +7111,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
+          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -7042,35 +7126,35 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>278</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>16051</t>
+          <t>16464</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -7080,12 +7164,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
+          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -7095,35 +7179,35 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -7133,22 +7217,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -7164,19 +7248,19 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -7186,12 +7270,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -7201,7 +7285,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -7217,34 +7301,34 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -7254,7 +7338,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -7262,56 +7346,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -7319,7 +7399,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7327,34 +7411,34 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -7364,7 +7448,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -7375,96 +7459,92 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -7474,7 +7554,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -7482,7 +7562,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7490,19 +7574,19 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -7512,12 +7596,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -7527,12 +7611,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -7543,19 +7627,19 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -7565,22 +7649,22 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -7596,19 +7680,19 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -7618,12 +7702,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -7633,7 +7717,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -7644,96 +7728,92 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -7743,35 +7823,39 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7781,22 +7865,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -7807,24 +7891,24 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7834,12 +7918,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -7849,7 +7933,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -7860,24 +7944,24 @@
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -7887,22 +7971,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -7918,44 +8002,44 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -7971,44 +8055,44 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -8016,31 +8100,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -8050,12 +8130,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -8065,7 +8145,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -8097,22 +8177,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -8122,7 +8202,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -8130,27 +8210,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -8160,12 +8244,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -8175,113 +8259,113 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -8289,31 +8373,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -8323,12 +8403,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -8338,7 +8418,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -8370,32 +8450,32 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -8403,7 +8483,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I41" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8423,22 +8507,22 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -8448,7 +8532,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -8476,22 +8560,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -8501,19 +8585,15 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8533,7 +8613,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -8543,12 +8623,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -8558,7 +8638,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -8590,40 +8670,44 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I45" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8643,22 +8727,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -8668,7 +8752,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -8676,11 +8760,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8700,32 +8780,32 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -8733,7 +8813,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8741,34 +8825,34 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -8778,7 +8862,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -8789,49 +8873,49 @@
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -8859,22 +8943,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -8884,7 +8968,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -8912,32 +8996,32 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -8965,22 +9049,22 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -8990,39 +9074,35 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -9032,27 +9112,27 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -9079,32 +9159,32 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -9112,52 +9192,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -9185,32 +9269,32 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -9238,32 +9322,32 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -9291,32 +9375,32 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -9324,46 +9408,42 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14403</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -9373,7 +9453,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>6587</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -9381,52 +9461,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -9446,6 +9530,59 @@
         </is>
       </c>
       <c r="K60" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-08-03 13:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -6268,7 +6268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:K62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6331,7 +6331,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>25891</t>
+          <t>26188</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6341,12 +6341,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 지역 상생 3대 사업 참여자 모집</t>
+          <t>2026년 8차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(8월 추천) (~8.21(금) 18시까지)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2621&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3734&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -6356,7 +6356,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -6367,39 +6367,39 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-08-03 09:31:46.854132+09:00</t>
+          <t>2026-08-03 13:16:30.325331+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-08-03 09:31:46.854132+09:00</t>
+          <t>2026-08-03 13:16:30.325331+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>25864</t>
+          <t>25891</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026년 전남광주통합특별시 소상공인·사회적경제기업 판로 확대 지원기업 선발 안내(~8.14)</t>
+          <t>한국인터넷진흥원, 지역 상생 3대 사업 참여자 모집</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3730&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2621&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>80</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -6417,31 +6417,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-08-03 09:16:35.817723+09:00</t>
+          <t>2026-08-03 09:31:46.854132+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-08-03 09:16:35.817723+09:00</t>
+          <t>2026-08-03 09:31:46.854132+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>25863</t>
+          <t>25864</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6451,12 +6447,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026년 전남광주통합특별시 지역문제 해결 프로젝트 공모전 개최 안내(~8.21)</t>
+          <t>2026년 전남광주통합특별시 소상공인·사회적경제기업 판로 확대 지원기업 선발 안내(~8.14)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3731&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3730&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -6466,7 +6462,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -6498,7 +6494,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>25862</t>
+          <t>25863</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6508,12 +6504,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026년 한국인터넷진흥원 지역공부방 참여 대학생 장학금 지원자 모집 안내(~8.28)</t>
+          <t>2026년 전남광주통합특별시 지역문제 해결 프로젝트 공모전 개최 안내(~8.21)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3732&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3731&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -6523,7 +6519,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -6555,7 +6551,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>25861</t>
+          <t>25862</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6565,12 +6561,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026년 암호모듈 시험자 양성교육 및 필기시험 안내(8.3~8.21)</t>
+          <t>2026년 한국인터넷진흥원 지역공부방 참여 대학생 장학금 지원자 모집 안내(~8.28)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3733&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3732&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -6580,7 +6576,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -6612,7 +6608,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>23221</t>
+          <t>25861</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6622,22 +6618,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
+          <t>2026년 암호모듈 시험자 양성교육 및 필기시험 안내(8.3~8.21)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3733&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -6657,52 +6653,56 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>22504</t>
+          <t>23221</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
+          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6710,19 +6710,19 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>22464</t>
+          <t>22504</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6732,12 +6732,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -6747,7 +6747,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -6763,19 +6763,19 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>20771</t>
+          <t>22464</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6785,50 +6785,50 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
+          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>20191</t>
+          <t>20771</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -6838,12 +6838,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
+          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -6853,7 +6853,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -6869,34 +6869,34 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>20061</t>
+          <t>20191</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
+          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -6906,7 +6906,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>287</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -6914,64 +6914,64 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>16785</t>
+          <t>20061</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1496</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
+          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>246</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6979,34 +6979,34 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>16784</t>
+          <t>16785</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1497</t>
+          <t>1496</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -7016,7 +7016,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -7044,22 +7044,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>16781</t>
+          <t>16784</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1497</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -7069,7 +7069,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>260</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -7077,11 +7077,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7101,22 +7097,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>16691</t>
+          <t>16781</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -7126,35 +7122,39 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>242</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>16464</t>
+          <t>16691</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -7164,12 +7164,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
+          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -7179,35 +7179,35 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>278</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>16051</t>
+          <t>16464</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -7217,12 +7217,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
+          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -7232,35 +7232,35 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -7270,22 +7270,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -7301,19 +7301,19 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -7323,12 +7323,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -7338,7 +7338,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -7354,34 +7354,34 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -7391,7 +7391,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -7399,56 +7399,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -7456,7 +7452,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7464,34 +7464,34 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -7501,7 +7501,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -7512,96 +7512,92 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -7611,7 +7607,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -7619,7 +7615,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7627,19 +7627,19 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -7649,12 +7649,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -7664,12 +7664,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
@@ -7680,19 +7680,19 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -7702,22 +7702,22 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -7733,19 +7733,19 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -7755,12 +7755,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -7770,7 +7770,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -7781,96 +7781,92 @@
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -7880,35 +7876,39 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7918,22 +7918,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -7944,24 +7944,24 @@
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -7971,12 +7971,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -7986,7 +7986,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -7997,24 +7997,24 @@
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -8024,22 +8024,22 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -8055,44 +8055,44 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -8108,44 +8108,44 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -8153,31 +8153,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -8187,12 +8183,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -8202,7 +8198,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -8234,22 +8230,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -8259,7 +8255,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -8267,27 +8263,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -8297,12 +8297,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -8312,113 +8312,113 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -8426,31 +8426,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -8460,12 +8456,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -8475,7 +8471,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -8507,32 +8503,32 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -8540,7 +8536,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8560,22 +8560,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -8585,7 +8585,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -8613,22 +8613,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -8638,19 +8638,15 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8670,7 +8666,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -8680,12 +8676,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -8695,7 +8691,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -8727,40 +8723,44 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I46" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8780,22 +8780,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -8805,7 +8805,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -8813,11 +8813,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8837,32 +8833,32 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -8870,7 +8866,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I48" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8878,34 +8878,34 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -8915,7 +8915,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -8926,49 +8926,49 @@
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -8996,22 +8996,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -9021,7 +9021,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -9049,32 +9049,32 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -9102,22 +9102,22 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -9127,39 +9127,35 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -9169,27 +9165,27 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -9216,32 +9212,32 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -9249,52 +9245,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -9322,32 +9322,32 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -9375,32 +9375,32 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -9428,32 +9428,32 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -9461,46 +9461,42 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14403</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -9510,7 +9506,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>6587</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -9518,52 +9514,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -9583,6 +9583,59 @@
         </is>
       </c>
       <c r="K61" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-08-03 14:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -6268,7 +6268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K62"/>
+  <dimension ref="A1:K63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6331,7 +6331,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>26188</t>
+          <t>26211</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6341,12 +6341,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026년 8차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(8월 추천) (~8.21(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 암호모듈검증 위한 시험 전문인력 양성</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3734&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2622&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -6356,7 +6356,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>273</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -6367,24 +6367,24 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-08-03 13:16:30.325331+09:00</t>
+          <t>2026-08-03 13:31:41.722921+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-08-03 13:16:30.325331+09:00</t>
+          <t>2026-08-03 13:31:41.722921+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>25891</t>
+          <t>26188</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6394,12 +6394,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 지역 상생 3대 사업 참여자 모집</t>
+          <t>2026년 8차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(8월 추천) (~8.21(금) 18시까지)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2621&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3734&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -6420,39 +6420,39 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-08-03 09:31:46.854132+09:00</t>
+          <t>2026-08-03 13:16:30.325331+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-08-03 09:31:46.854132+09:00</t>
+          <t>2026-08-03 13:16:30.325331+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>25864</t>
+          <t>25891</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026년 전남광주통합특별시 소상공인·사회적경제기업 판로 확대 지원기업 선발 안내(~8.14)</t>
+          <t>한국인터넷진흥원, 지역 상생 3대 사업 참여자 모집</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3730&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2621&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -6462,7 +6462,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>80</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -6470,31 +6470,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-08-03 09:16:35.817723+09:00</t>
+          <t>2026-08-03 09:31:46.854132+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-08-03 09:16:35.817723+09:00</t>
+          <t>2026-08-03 09:31:46.854132+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>25863</t>
+          <t>25864</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6504,12 +6500,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026년 전남광주통합특별시 지역문제 해결 프로젝트 공모전 개최 안내(~8.21)</t>
+          <t>2026년 전남광주통합특별시 소상공인·사회적경제기업 판로 확대 지원기업 선발 안내(~8.14)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3731&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3730&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -6519,7 +6515,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -6551,7 +6547,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>25862</t>
+          <t>25863</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6561,12 +6557,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026년 한국인터넷진흥원 지역공부방 참여 대학생 장학금 지원자 모집 안내(~8.28)</t>
+          <t>2026년 전남광주통합특별시 지역문제 해결 프로젝트 공모전 개최 안내(~8.21)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3732&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3731&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -6576,7 +6572,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -6608,7 +6604,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>25861</t>
+          <t>25862</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6618,12 +6614,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026년 암호모듈 시험자 양성교육 및 필기시험 안내(8.3~8.21)</t>
+          <t>2026년 한국인터넷진흥원 지역공부방 참여 대학생 장학금 지원자 모집 안내(~8.28)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3733&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3732&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -6633,7 +6629,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -6665,7 +6661,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>23221</t>
+          <t>25861</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6675,22 +6671,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
+          <t>2026년 암호모듈 시험자 양성교육 및 필기시험 안내(8.3~8.21)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3733&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -6710,52 +6706,56 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>22504</t>
+          <t>23221</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
+          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6763,19 +6763,19 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>22464</t>
+          <t>22504</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6785,12 +6785,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -6816,19 +6816,19 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>20771</t>
+          <t>22464</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -6838,50 +6838,50 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
+          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>20191</t>
+          <t>20771</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -6891,12 +6891,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
+          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -6906,7 +6906,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -6922,34 +6922,34 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>20061</t>
+          <t>20191</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
+          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -6959,7 +6959,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>287</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -6967,64 +6967,64 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>16785</t>
+          <t>20061</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1496</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
+          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>246</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7032,34 +7032,34 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>16784</t>
+          <t>16785</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1497</t>
+          <t>1496</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -7069,7 +7069,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -7097,22 +7097,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>16781</t>
+          <t>16784</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1497</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -7122,7 +7122,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>260</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -7130,11 +7130,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7154,22 +7150,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>16691</t>
+          <t>16781</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -7179,35 +7175,39 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>242</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>16464</t>
+          <t>16691</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -7217,12 +7217,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
+          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -7232,35 +7232,35 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>278</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>16051</t>
+          <t>16464</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -7270,12 +7270,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
+          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -7285,35 +7285,35 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -7323,22 +7323,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -7354,19 +7354,19 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -7376,12 +7376,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -7391,7 +7391,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -7407,34 +7407,34 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -7444,7 +7444,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -7452,56 +7452,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -7509,7 +7505,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7517,34 +7517,34 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -7554,7 +7554,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -7565,96 +7565,92 @@
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -7664,7 +7660,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -7672,7 +7668,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7680,19 +7680,19 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -7702,12 +7702,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -7717,12 +7717,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -7733,19 +7733,19 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -7755,22 +7755,22 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -7786,19 +7786,19 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -7808,12 +7808,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -7823,7 +7823,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -7834,96 +7834,92 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -7933,35 +7929,39 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -7971,22 +7971,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -7997,24 +7997,24 @@
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -8024,12 +8024,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -8039,7 +8039,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -8050,24 +8050,24 @@
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -8077,22 +8077,22 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -8108,44 +8108,44 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -8161,44 +8161,44 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -8206,31 +8206,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -8240,12 +8236,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -8255,7 +8251,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -8287,22 +8283,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -8312,7 +8308,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -8320,27 +8316,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -8350,12 +8350,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -8365,113 +8365,113 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -8479,31 +8479,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -8513,12 +8509,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -8528,7 +8524,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -8560,32 +8556,32 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -8593,7 +8589,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I43" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8613,22 +8613,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -8638,7 +8638,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -8666,22 +8666,22 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -8691,19 +8691,15 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8723,7 +8719,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8733,12 +8729,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -8748,7 +8744,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -8780,40 +8776,44 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8833,22 +8833,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -8858,7 +8858,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -8866,11 +8866,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8890,32 +8886,32 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -8923,7 +8919,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I49" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8931,34 +8931,34 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -8968,7 +8968,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -8979,49 +8979,49 @@
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -9049,22 +9049,22 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -9074,7 +9074,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -9102,32 +9102,32 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -9155,22 +9155,22 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -9180,39 +9180,35 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -9222,27 +9218,27 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -9269,32 +9265,32 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -9302,52 +9298,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -9375,32 +9375,32 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -9428,32 +9428,32 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -9481,32 +9481,32 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -9514,46 +9514,42 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14403</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -9563,7 +9559,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>6587</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -9571,52 +9567,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -9636,6 +9636,59 @@
         </is>
       </c>
       <c r="K62" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-08-04 15:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -6268,7 +6268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K63"/>
+  <dimension ref="A1:K64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6331,7 +6331,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>26211</t>
+          <t>27128</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6341,50 +6341,50 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 암호모듈검증 위한 시험 전문인력 양성</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 20회차 교육생 모집(~9.4)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2622&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3735&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>273</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-08-03 13:31:41.722921+09:00</t>
+          <t>2026-08-04 14:46:28.764255+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-08-03 13:31:41.722921+09:00</t>
+          <t>2026-08-04 14:46:28.764255+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>26188</t>
+          <t>26211</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6394,12 +6394,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026년 8차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(8월 추천) (~8.21(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 암호모듈검증 위한 시험 전문인력 양성</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3734&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2622&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>273</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -6420,24 +6420,24 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-08-03 13:16:30.325331+09:00</t>
+          <t>2026-08-03 13:31:41.722921+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-08-03 13:16:30.325331+09:00</t>
+          <t>2026-08-03 13:31:41.722921+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>25891</t>
+          <t>26188</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6447,12 +6447,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 지역 상생 3대 사업 참여자 모집</t>
+          <t>2026년 8차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(8월 추천) (~8.21(금) 18시까지)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2621&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3734&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -6462,7 +6462,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -6473,39 +6473,39 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-08-03 09:31:46.854132+09:00</t>
+          <t>2026-08-03 13:16:30.325331+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-08-03 09:31:46.854132+09:00</t>
+          <t>2026-08-03 13:16:30.325331+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>25864</t>
+          <t>25891</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026년 전남광주통합특별시 소상공인·사회적경제기업 판로 확대 지원기업 선발 안내(~8.14)</t>
+          <t>한국인터넷진흥원, 지역 상생 3대 사업 참여자 모집</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3730&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2621&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -6515,7 +6515,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>80</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -6523,31 +6523,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-08-03 09:16:35.817723+09:00</t>
+          <t>2026-08-03 09:31:46.854132+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-08-03 09:16:35.817723+09:00</t>
+          <t>2026-08-03 09:31:46.854132+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>25863</t>
+          <t>25864</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6557,12 +6553,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026년 전남광주통합특별시 지역문제 해결 프로젝트 공모전 개최 안내(~8.21)</t>
+          <t>2026년 전남광주통합특별시 소상공인·사회적경제기업 판로 확대 지원기업 선발 안내(~8.14)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3731&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3730&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -6572,7 +6568,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -6604,7 +6600,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>25862</t>
+          <t>25863</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6614,12 +6610,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026년 한국인터넷진흥원 지역공부방 참여 대학생 장학금 지원자 모집 안내(~8.28)</t>
+          <t>2026년 전남광주통합특별시 지역문제 해결 프로젝트 공모전 개최 안내(~8.21)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3732&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3731&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -6629,7 +6625,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -6661,7 +6657,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>25861</t>
+          <t>25862</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6671,12 +6667,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026년 암호모듈 시험자 양성교육 및 필기시험 안내(8.3~8.21)</t>
+          <t>2026년 한국인터넷진흥원 지역공부방 참여 대학생 장학금 지원자 모집 안내(~8.28)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3733&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3732&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -6686,7 +6682,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -6718,7 +6714,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>23221</t>
+          <t>25861</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6728,22 +6724,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
+          <t>2026년 암호모듈 시험자 양성교육 및 필기시험 안내(8.3~8.21)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3733&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -6763,52 +6759,56 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>22504</t>
+          <t>23221</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
+          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6816,19 +6816,19 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>22464</t>
+          <t>22504</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -6838,12 +6838,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -6853,7 +6853,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -6869,19 +6869,19 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>20771</t>
+          <t>22464</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -6891,50 +6891,50 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
+          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>20191</t>
+          <t>20771</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -6944,12 +6944,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
+          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -6959,7 +6959,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -6975,34 +6975,34 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>20061</t>
+          <t>20191</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
+          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -7012,7 +7012,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>287</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -7020,64 +7020,64 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>16785</t>
+          <t>20061</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1496</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
+          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>246</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7085,34 +7085,34 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>16784</t>
+          <t>16785</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1497</t>
+          <t>1496</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -7122,7 +7122,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -7150,22 +7150,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>16781</t>
+          <t>16784</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1497</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -7175,7 +7175,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>260</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -7183,11 +7183,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7207,22 +7203,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>16691</t>
+          <t>16781</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -7232,35 +7228,39 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>242</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>16464</t>
+          <t>16691</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -7270,12 +7270,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
+          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -7285,35 +7285,35 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>278</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>16051</t>
+          <t>16464</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -7323,12 +7323,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
+          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -7338,35 +7338,35 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -7376,22 +7376,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -7407,19 +7407,19 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -7429,12 +7429,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -7444,7 +7444,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -7460,34 +7460,34 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -7497,7 +7497,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -7505,56 +7505,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -7562,7 +7558,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7570,34 +7570,34 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -7607,7 +7607,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -7618,96 +7618,92 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -7717,7 +7713,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -7725,7 +7721,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7733,19 +7733,19 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -7755,12 +7755,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -7770,12 +7770,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
@@ -7786,19 +7786,19 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -7808,22 +7808,22 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -7839,19 +7839,19 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7861,12 +7861,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -7876,7 +7876,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -7887,96 +7887,92 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -7986,35 +7982,39 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -8024,22 +8024,22 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -8050,24 +8050,24 @@
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -8077,12 +8077,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -8092,7 +8092,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -8103,24 +8103,24 @@
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -8130,22 +8130,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -8161,44 +8161,44 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -8214,44 +8214,44 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -8259,31 +8259,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -8293,12 +8289,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -8308,7 +8304,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -8340,22 +8336,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -8365,7 +8361,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -8373,27 +8369,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -8403,12 +8403,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -8418,113 +8418,113 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -8532,31 +8532,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -8566,12 +8562,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -8581,7 +8577,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -8613,32 +8609,32 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -8646,7 +8642,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8666,22 +8666,22 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -8719,22 +8719,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -8744,19 +8744,15 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8776,7 +8772,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -8786,12 +8782,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -8801,7 +8797,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -8833,40 +8829,44 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I48" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8886,22 +8886,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -8911,7 +8911,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -8919,11 +8919,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8943,32 +8939,32 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -8976,7 +8972,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I50" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8984,34 +8984,34 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -9021,7 +9021,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -9032,49 +9032,49 @@
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -9102,22 +9102,22 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -9127,7 +9127,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -9155,32 +9155,32 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -9208,22 +9208,22 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -9233,39 +9233,35 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -9275,27 +9271,27 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -9322,32 +9318,32 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -9355,52 +9351,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -9428,32 +9428,32 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -9481,32 +9481,32 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -9534,32 +9534,32 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -9567,46 +9567,42 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14403</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -9616,7 +9612,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>6587</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -9624,52 +9620,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -9689,6 +9689,59 @@
         </is>
       </c>
       <c r="K63" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-08-04 17:20:02 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -6268,7 +6268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K64"/>
+  <dimension ref="A1:K65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6331,7 +6331,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>27128</t>
+          <t>27268</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6341,12 +6341,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 20회차 교육생 모집(~9.4)</t>
+          <t>양자내성암호 국제 표준화 동향 분석</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3735&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3736&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -6356,12 +6356,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -6372,19 +6372,19 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-08-04 14:46:28.764255+09:00</t>
+          <t>2026-08-04 16:31:26.502205+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-08-04 14:46:28.764255+09:00</t>
+          <t>2026-08-04 16:31:26.502205+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>26211</t>
+          <t>27128</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6394,50 +6394,50 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 암호모듈검증 위한 시험 전문인력 양성</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 20회차 교육생 모집(~9.4)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2622&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3735&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>273</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-08-03 13:31:41.722921+09:00</t>
+          <t>2026-08-04 14:46:28.764255+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-08-03 13:31:41.722921+09:00</t>
+          <t>2026-08-04 14:46:28.764255+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>26188</t>
+          <t>26211</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6447,12 +6447,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026년 8차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(8월 추천) (~8.21(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 암호모듈검증 위한 시험 전문인력 양성</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3734&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2622&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -6462,7 +6462,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>273</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -6473,24 +6473,24 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-08-03 13:16:30.325331+09:00</t>
+          <t>2026-08-03 13:31:41.722921+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-08-03 13:16:30.325331+09:00</t>
+          <t>2026-08-03 13:31:41.722921+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>25891</t>
+          <t>26188</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6500,12 +6500,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 지역 상생 3대 사업 참여자 모집</t>
+          <t>2026년 8차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(8월 추천) (~8.21(금) 18시까지)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2621&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3734&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -6515,7 +6515,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -6526,39 +6526,39 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-08-03 09:31:46.854132+09:00</t>
+          <t>2026-08-03 13:16:30.325331+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-08-03 09:31:46.854132+09:00</t>
+          <t>2026-08-03 13:16:30.325331+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>25864</t>
+          <t>25891</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026년 전남광주통합특별시 소상공인·사회적경제기업 판로 확대 지원기업 선발 안내(~8.14)</t>
+          <t>한국인터넷진흥원, 지역 상생 3대 사업 참여자 모집</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3730&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2621&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -6568,7 +6568,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>80</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -6576,31 +6576,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-08-03 09:16:35.817723+09:00</t>
+          <t>2026-08-03 09:31:46.854132+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-08-03 09:16:35.817723+09:00</t>
+          <t>2026-08-03 09:31:46.854132+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>25863</t>
+          <t>25864</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6610,12 +6606,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026년 전남광주통합특별시 지역문제 해결 프로젝트 공모전 개최 안내(~8.21)</t>
+          <t>2026년 전남광주통합특별시 소상공인·사회적경제기업 판로 확대 지원기업 선발 안내(~8.14)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3731&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3730&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -6625,7 +6621,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -6657,7 +6653,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>25862</t>
+          <t>25863</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6667,12 +6663,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026년 한국인터넷진흥원 지역공부방 참여 대학생 장학금 지원자 모집 안내(~8.28)</t>
+          <t>2026년 전남광주통합특별시 지역문제 해결 프로젝트 공모전 개최 안내(~8.21)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3732&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3731&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -6682,7 +6678,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -6714,7 +6710,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>25861</t>
+          <t>25862</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6724,12 +6720,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026년 암호모듈 시험자 양성교육 및 필기시험 안내(8.3~8.21)</t>
+          <t>2026년 한국인터넷진흥원 지역공부방 참여 대학생 장학금 지원자 모집 안내(~8.28)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3733&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3732&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -6739,7 +6735,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -6771,7 +6767,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>23221</t>
+          <t>25861</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6781,22 +6777,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
+          <t>2026년 암호모듈 시험자 양성교육 및 필기시험 안내(8.3~8.21)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3733&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -6816,52 +6812,56 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>22504</t>
+          <t>23221</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
+          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -6869,19 +6869,19 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>22464</t>
+          <t>22504</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -6891,12 +6891,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -6906,7 +6906,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -6922,19 +6922,19 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>20771</t>
+          <t>22464</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -6944,50 +6944,50 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
+          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>20191</t>
+          <t>20771</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -6997,12 +6997,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
+          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -7012,7 +7012,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -7028,34 +7028,34 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>20061</t>
+          <t>20191</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
+          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -7065,7 +7065,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>287</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -7073,64 +7073,64 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>16785</t>
+          <t>20061</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1496</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
+          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>246</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7138,34 +7138,34 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>16784</t>
+          <t>16785</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1497</t>
+          <t>1496</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -7175,7 +7175,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -7203,22 +7203,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>16781</t>
+          <t>16784</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1497</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -7228,7 +7228,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>260</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -7236,11 +7236,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7260,22 +7256,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>16691</t>
+          <t>16781</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -7285,35 +7281,39 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>242</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>16464</t>
+          <t>16691</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -7323,12 +7323,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
+          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -7338,35 +7338,35 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>278</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>16051</t>
+          <t>16464</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -7376,12 +7376,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
+          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -7391,35 +7391,35 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -7429,22 +7429,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -7460,19 +7460,19 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -7482,12 +7482,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -7497,7 +7497,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -7513,34 +7513,34 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -7550,7 +7550,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -7558,56 +7558,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -7615,7 +7611,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7623,34 +7623,34 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -7660,7 +7660,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -7671,96 +7671,92 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -7770,7 +7766,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -7778,7 +7774,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -7786,19 +7786,19 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -7808,12 +7808,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -7823,12 +7823,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -7839,19 +7839,19 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7861,22 +7861,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -7892,19 +7892,19 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7914,12 +7914,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -7929,7 +7929,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -7940,96 +7940,92 @@
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -8039,35 +8035,39 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -8077,22 +8077,22 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -8103,24 +8103,24 @@
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -8130,12 +8130,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -8145,7 +8145,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -8156,24 +8156,24 @@
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -8183,22 +8183,22 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -8214,44 +8214,44 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -8267,44 +8267,44 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -8312,31 +8312,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -8346,12 +8342,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -8361,7 +8357,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -8393,22 +8389,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -8418,7 +8414,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -8426,27 +8422,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -8456,12 +8456,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -8471,113 +8471,113 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -8585,31 +8585,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -8619,12 +8615,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -8634,7 +8630,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -8666,32 +8662,32 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -8699,7 +8695,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I45" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8719,22 +8719,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -8744,7 +8744,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -8772,22 +8772,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -8797,19 +8797,15 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8829,7 +8825,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -8839,12 +8835,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -8854,7 +8850,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -8886,40 +8882,44 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I49" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -8939,22 +8939,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
   